<commit_message>
Corrige extensoes do mapa
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github_corrigido_dashboard_obrasdinamico\github\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DCFF995-9770-4685-8FB4-A2A5EF8D83C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06CC311A-5D85-4D5F-B548-ADAB37F513D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LEIA-ME" sheetId="1" r:id="rId1"/>
@@ -18165,6 +18165,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R388"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -18228,7 +18229,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -18278,7 +18279,7 @@
         <v>-46.416253400000002</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -18328,7 +18329,7 @@
         <v>-46.416704099999997</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -18378,7 +18379,7 @@
         <v>-46.417190099999999</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -18428,7 +18429,7 @@
         <v>-46.417341</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -18478,7 +18479,7 @@
         <v>-46.417501700000003</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -18528,7 +18529,7 @@
         <v>-46.4176821</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -18578,7 +18579,7 @@
         <v>-46.417981300000001</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -18628,7 +18629,7 @@
         <v>-46.418407199999997</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -18678,7 +18679,7 @@
         <v>-46.418206699999999</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -18728,7 +18729,7 @@
         <v>-46.4180463</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -18778,7 +18779,7 @@
         <v>-46.418264100000002</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -18828,7 +18829,7 @@
         <v>-46.4183649</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -18878,7 +18879,7 @@
         <v>-46.418435899999999</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -18928,7 +18929,7 @@
         <v>-46.416806899999997</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -18978,7 +18979,7 @@
         <v>-46.416913999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -19028,7 +19029,7 @@
         <v>-46.416511399999997</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -19078,7 +19079,7 @@
         <v>-46.416153399999999</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -19128,7 +19129,7 @@
         <v>-46.416207999999997</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -19178,7 +19179,7 @@
         <v>-46.416177500000003</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -19228,7 +19229,7 @@
         <v>-46.418407199999997</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -19278,7 +19279,7 @@
         <v>-46.418435299999999</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -19328,7 +19329,7 @@
         <v>-46.416253400000002</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -19378,7 +19379,7 @@
         <v>-46.416341899999999</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -19428,7 +19429,7 @@
         <v>-46.416704099999997</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -19478,7 +19479,7 @@
         <v>-46.415709800000002</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -19528,7 +19529,7 @@
         <v>-46.415711799999997</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -19578,7 +19579,7 @@
         <v>-46.416806899999997</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -19628,7 +19629,7 @@
         <v>-46.416340599999998</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -19678,7 +19679,7 @@
         <v>-46.416158799999998</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -19728,7 +19729,7 @@
         <v>-46.416158799999998</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -19778,7 +19779,7 @@
         <v>-46.416511399999997</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>79</v>
       </c>
@@ -19828,7 +19829,7 @@
         <v>-46.38594079802948</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>79</v>
       </c>
@@ -19878,7 +19879,7 @@
         <v>-46.386535748682967</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>79</v>
       </c>
@@ -19928,7 +19929,7 @@
         <v>-46.385331250405009</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>79</v>
       </c>
@@ -19978,7 +19979,7 @@
         <v>-46.385209892569947</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>79</v>
       </c>
@@ -20446,7 +20447,7 @@
         <v>530</v>
       </c>
       <c r="I45">
-        <v>120.49</v>
+        <v>0</v>
       </c>
       <c r="J45">
         <v>8.2200000000000006</v>
@@ -20502,7 +20503,7 @@
         <v>530</v>
       </c>
       <c r="I46">
-        <v>78.569999999999993</v>
+        <v>0</v>
       </c>
       <c r="J46">
         <v>8.16</v>
@@ -20588,7 +20589,7 @@
         <v>-46.401313100000003</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>117</v>
       </c>
@@ -20644,7 +20645,7 @@
         <v>-46.4176511</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>117</v>
       </c>
@@ -20700,7 +20701,7 @@
         <v>-46.417446300000002</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>117</v>
       </c>
@@ -20756,7 +20757,7 @@
         <v>-46.417286599999997</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>117</v>
       </c>
@@ -20812,7 +20813,7 @@
         <v>-46.418029900000001</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>117</v>
       </c>
@@ -20868,7 +20869,7 @@
         <v>-46.417090700000003</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>117</v>
       </c>
@@ -20924,7 +20925,7 @@
         <v>-46.416909699999998</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>117</v>
       </c>
@@ -20980,7 +20981,7 @@
         <v>-46.416524600000002</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>117</v>
       </c>
@@ -21036,7 +21037,7 @@
         <v>-46.416342700000001</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>117</v>
       </c>
@@ -21092,7 +21093,7 @@
         <v>-46.416342700000001</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>117</v>
       </c>
@@ -21148,7 +21149,7 @@
         <v>-46.4159948</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>117</v>
       </c>
@@ -21204,7 +21205,7 @@
         <v>-46.415814900000001</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>117</v>
       </c>
@@ -21260,7 +21261,7 @@
         <v>-46.415814900000001</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>117</v>
       </c>
@@ -21316,7 +21317,7 @@
         <v>-46.415630399999998</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>117</v>
       </c>
@@ -21372,7 +21373,7 @@
         <v>-46.4153284</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>117</v>
       </c>
@@ -21428,7 +21429,7 @@
         <v>-46.414648700000001</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>117</v>
       </c>
@@ -21484,7 +21485,7 @@
         <v>-46.415173099999997</v>
       </c>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>117</v>
       </c>
@@ -21540,7 +21541,7 @@
         <v>-46.4153941</v>
       </c>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>117</v>
       </c>
@@ -21596,7 +21597,7 @@
         <v>-46.4171725</v>
       </c>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>117</v>
       </c>
@@ -21652,7 +21653,7 @@
         <v>-46.4164241</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>117</v>
       </c>
@@ -21708,7 +21709,7 @@
         <v>-46.4165888</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>117</v>
       </c>
@@ -21764,7 +21765,7 @@
         <v>-46.415878399999997</v>
       </c>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>117</v>
       </c>
@@ -21820,7 +21821,7 @@
         <v>-46.417214999999999</v>
       </c>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>165</v>
       </c>
@@ -21876,7 +21877,7 @@
         <v>-46.394514126473538</v>
       </c>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>165</v>
       </c>
@@ -21932,7 +21933,7 @@
         <v>-46.39440497485721</v>
       </c>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>165</v>
       </c>
@@ -21988,7 +21989,7 @@
         <v>-46.394190685187283</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>165</v>
       </c>
@@ -22044,7 +22045,7 @@
         <v>-46.393867676588513</v>
       </c>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>165</v>
       </c>
@@ -22100,7 +22101,7 @@
         <v>-46.393750908484463</v>
       </c>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>165</v>
       </c>
@@ -22156,7 +22157,7 @@
         <v>-46.393754824461297</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>165</v>
       </c>
@@ -22212,7 +22213,7 @@
         <v>-46.393677744048787</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>165</v>
       </c>
@@ -22268,7 +22269,7 @@
         <v>-46.393669850604603</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>165</v>
       </c>
@@ -22324,7 +22325,7 @@
         <v>-46.393617999096797</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>165</v>
       </c>
@@ -22380,7 +22381,7 @@
         <v>-46.39342680270682</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>165</v>
       </c>
@@ -22436,7 +22437,7 @@
         <v>-46.393118667987821</v>
       </c>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>165</v>
       </c>
@@ -22492,7 +22493,7 @@
         <v>-46.392683603256813</v>
       </c>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>165</v>
       </c>
@@ -22548,7 +22549,7 @@
         <v>-46.392567097741733</v>
       </c>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>165</v>
       </c>
@@ -22604,7 +22605,7 @@
         <v>-46.392172750576698</v>
       </c>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>165</v>
       </c>
@@ -22660,7 +22661,7 @@
         <v>-46.391704600778667</v>
       </c>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>165</v>
       </c>
@@ -22716,7 +22717,7 @@
         <v>-46.393984483001361</v>
       </c>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>165</v>
       </c>
@@ -22772,7 +22773,7 @@
         <v>-46.39421417616888</v>
       </c>
     </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>165</v>
       </c>
@@ -22828,7 +22829,7 @@
         <v>-46.393884994376727</v>
       </c>
     </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>165</v>
       </c>
@@ -22884,7 +22885,7 @@
         <v>-46.393931783273203</v>
       </c>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>165</v>
       </c>
@@ -22940,7 +22941,7 @@
         <v>-46.393826949732833</v>
       </c>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>165</v>
       </c>
@@ -22996,7 +22997,7 @@
         <v>-46.393834080493427</v>
       </c>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>165</v>
       </c>
@@ -23052,7 +23053,7 @@
         <v>-46.393874814521602</v>
       </c>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>165</v>
       </c>
@@ -23108,7 +23109,7 @@
         <v>-46.393600080891758</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>165</v>
       </c>
@@ -23164,7 +23165,7 @@
         <v>-46.392812880408918</v>
       </c>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>165</v>
       </c>
@@ -23220,7 +23221,7 @@
         <v>-46.392828108924483</v>
       </c>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>165</v>
       </c>
@@ -23276,7 +23277,7 @@
         <v>-46.392669018473534</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>165</v>
       </c>
@@ -23332,7 +23333,7 @@
         <v>-46.3922548189284</v>
       </c>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>165</v>
       </c>
@@ -23388,7 +23389,7 @@
         <v>-46.391867207322441</v>
       </c>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>221</v>
       </c>
@@ -23441,7 +23442,7 @@
         <v>-46.385538400000002</v>
       </c>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>221</v>
       </c>
@@ -23494,7 +23495,7 @@
         <v>-46.385575299999999</v>
       </c>
     </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>221</v>
       </c>
@@ -23547,7 +23548,7 @@
         <v>-46.385641</v>
       </c>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>221</v>
       </c>
@@ -23600,7 +23601,7 @@
         <v>-46.386125</v>
       </c>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>221</v>
       </c>
@@ -23653,7 +23654,7 @@
         <v>-46.386338700000003</v>
       </c>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>221</v>
       </c>
@@ -23706,7 +23707,7 @@
         <v>-46.387470700000002</v>
       </c>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>221</v>
       </c>
@@ -23759,7 +23760,7 @@
         <v>-46.3881558</v>
       </c>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>221</v>
       </c>
@@ -23812,7 +23813,7 @@
         <v>-46.3889292</v>
       </c>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>221</v>
       </c>
@@ -23865,7 +23866,7 @@
         <v>-46.386140400000002</v>
       </c>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>221</v>
       </c>
@@ -23918,7 +23919,7 @@
         <v>-46.386125</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>221</v>
       </c>
@@ -23971,7 +23972,7 @@
         <v>-46.386821400000002</v>
       </c>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>221</v>
       </c>
@@ -24021,7 +24022,7 @@
         <v>-46.388970100000002</v>
       </c>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>240</v>
       </c>
@@ -24077,7 +24078,7 @@
         <v>-46.400490900000001</v>
       </c>
     </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>240</v>
       </c>
@@ -24133,7 +24134,7 @@
         <v>-46.400497299999998</v>
       </c>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>240</v>
       </c>
@@ -24189,7 +24190,7 @@
         <v>-46.399660099999998</v>
       </c>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>240</v>
       </c>
@@ -24245,7 +24246,7 @@
         <v>-46.399546600000001</v>
       </c>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>240</v>
       </c>
@@ -24301,7 +24302,7 @@
         <v>-46.399546899999997</v>
       </c>
     </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>240</v>
       </c>
@@ -24357,7 +24358,7 @@
         <v>-46.399427899999999</v>
       </c>
     </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>240</v>
       </c>
@@ -24413,7 +24414,7 @@
         <v>-46.399406300000003</v>
       </c>
     </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>240</v>
       </c>
@@ -24469,7 +24470,7 @@
         <v>-46.3993976</v>
       </c>
     </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>240</v>
       </c>
@@ -24525,7 +24526,7 @@
         <v>-46.399673499999999</v>
       </c>
     </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>240</v>
       </c>
@@ -24581,7 +24582,7 @@
         <v>-46.3991951</v>
       </c>
     </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>240</v>
       </c>
@@ -24637,7 +24638,7 @@
         <v>-46.3992</v>
       </c>
     </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>240</v>
       </c>
@@ -24693,7 +24694,7 @@
         <v>-46.399129500000001</v>
       </c>
     </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>240</v>
       </c>
@@ -24749,7 +24750,7 @@
         <v>-46.399120400000001</v>
       </c>
     </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>240</v>
       </c>
@@ -24805,7 +24806,7 @@
         <v>-46.399127700000001</v>
       </c>
     </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>240</v>
       </c>
@@ -24861,7 +24862,7 @@
         <v>-46.399663099999998</v>
       </c>
     </row>
-    <row r="125" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>240</v>
       </c>
@@ -24917,7 +24918,7 @@
         <v>-46.399161700000001</v>
       </c>
     </row>
-    <row r="126" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>240</v>
       </c>
@@ -24973,7 +24974,7 @@
         <v>-46.399083099999999</v>
       </c>
     </row>
-    <row r="127" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>240</v>
       </c>
@@ -25029,7 +25030,7 @@
         <v>-46.399065800000002</v>
       </c>
     </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>240</v>
       </c>
@@ -25085,7 +25086,7 @@
         <v>-46.399676200000002</v>
       </c>
     </row>
-    <row r="129" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>240</v>
       </c>
@@ -25141,7 +25142,7 @@
         <v>-46.399061099999997</v>
       </c>
     </row>
-    <row r="130" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>240</v>
       </c>
@@ -25197,7 +25198,7 @@
         <v>-46.398950800000001</v>
       </c>
     </row>
-    <row r="131" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>240</v>
       </c>
@@ -25253,7 +25254,7 @@
         <v>-46.3990565</v>
       </c>
     </row>
-    <row r="132" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>240</v>
       </c>
@@ -25309,7 +25310,7 @@
         <v>-46.3990103</v>
       </c>
     </row>
-    <row r="133" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>240</v>
       </c>
@@ -25365,7 +25366,7 @@
         <v>-46.398947300000003</v>
       </c>
     </row>
-    <row r="134" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>280</v>
       </c>
@@ -25418,7 +25419,7 @@
         <v>-46.388409799999998</v>
       </c>
     </row>
-    <row r="135" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>280</v>
       </c>
@@ -25471,7 +25472,7 @@
         <v>-46.386588699999997</v>
       </c>
     </row>
-    <row r="136" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>280</v>
       </c>
@@ -25524,7 +25525,7 @@
         <v>-46.3864564</v>
       </c>
     </row>
-    <row r="137" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>280</v>
       </c>
@@ -25577,7 +25578,7 @@
         <v>-46.387386399999997</v>
       </c>
     </row>
-    <row r="138" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>280</v>
       </c>
@@ -25630,7 +25631,7 @@
         <v>-46.387402899999998</v>
       </c>
     </row>
-    <row r="139" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>280</v>
       </c>
@@ -25683,7 +25684,7 @@
         <v>-46.3874511</v>
       </c>
     </row>
-    <row r="140" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>280</v>
       </c>
@@ -25736,7 +25737,7 @@
         <v>-46.386536300000003</v>
       </c>
     </row>
-    <row r="141" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>280</v>
       </c>
@@ -25789,7 +25790,7 @@
         <v>-46.3952478</v>
       </c>
     </row>
-    <row r="142" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>280</v>
       </c>
@@ -25842,7 +25843,7 @@
         <v>-46.395421599999999</v>
       </c>
     </row>
-    <row r="143" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>280</v>
       </c>
@@ -25895,7 +25896,7 @@
         <v>-46.395309099999999</v>
       </c>
     </row>
-    <row r="144" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>280</v>
       </c>
@@ -25948,7 +25949,7 @@
         <v>-46.3922934</v>
       </c>
     </row>
-    <row r="145" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>280</v>
       </c>
@@ -26001,7 +26002,7 @@
         <v>-46.3922934</v>
       </c>
     </row>
-    <row r="146" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>280</v>
       </c>
@@ -26054,7 +26055,7 @@
         <v>-46.391816499999997</v>
       </c>
     </row>
-    <row r="147" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>280</v>
       </c>
@@ -26107,7 +26108,7 @@
         <v>-46.391055199999997</v>
       </c>
     </row>
-    <row r="148" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>280</v>
       </c>
@@ -26160,7 +26161,7 @@
         <v>-46.390884300000003</v>
       </c>
     </row>
-    <row r="149" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>280</v>
       </c>
@@ -26213,7 +26214,7 @@
         <v>-46.3907059</v>
       </c>
     </row>
-    <row r="150" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>280</v>
       </c>
@@ -26266,7 +26267,7 @@
         <v>-46.389563600000002</v>
       </c>
     </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>280</v>
       </c>
@@ -26319,7 +26320,7 @@
         <v>-46.389226299999997</v>
       </c>
     </row>
-    <row r="152" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>280</v>
       </c>
@@ -26372,7 +26373,7 @@
         <v>-46.388674999999999</v>
       </c>
     </row>
-    <row r="153" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>280</v>
       </c>
@@ -26425,7 +26426,7 @@
         <v>-46.388370600000002</v>
       </c>
     </row>
-    <row r="154" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>280</v>
       </c>
@@ -26478,7 +26479,7 @@
         <v>-46.388409799999998</v>
       </c>
     </row>
-    <row r="155" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>280</v>
       </c>
@@ -26531,7 +26532,7 @@
         <v>-46.387695999999998</v>
       </c>
     </row>
-    <row r="156" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>280</v>
       </c>
@@ -26584,7 +26585,7 @@
         <v>-46.387413700000003</v>
       </c>
     </row>
-    <row r="157" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>280</v>
       </c>
@@ -26637,7 +26638,7 @@
         <v>-46.387386399999997</v>
       </c>
     </row>
-    <row r="158" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>280</v>
       </c>
@@ -26690,7 +26691,7 @@
         <v>-46.387402899999998</v>
       </c>
     </row>
-    <row r="159" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>280</v>
       </c>
@@ -26743,7 +26744,7 @@
         <v>-46.386888200000001</v>
       </c>
     </row>
-    <row r="160" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>280</v>
       </c>
@@ -26796,7 +26797,7 @@
         <v>-46.386210499999997</v>
       </c>
     </row>
-    <row r="161" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>280</v>
       </c>
@@ -26849,7 +26850,7 @@
         <v>-46.386560500000002</v>
       </c>
     </row>
-    <row r="162" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>280</v>
       </c>
@@ -26902,7 +26903,7 @@
         <v>-46.392178299999998</v>
       </c>
     </row>
-    <row r="163" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>280</v>
       </c>
@@ -26955,7 +26956,7 @@
         <v>-46.394682400000001</v>
       </c>
     </row>
-    <row r="164" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>280</v>
       </c>
@@ -27008,7 +27009,7 @@
         <v>-46.393901100000001</v>
       </c>
     </row>
-    <row r="165" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>280</v>
       </c>
@@ -27061,7 +27062,7 @@
         <v>-46.393103199999999</v>
       </c>
     </row>
-    <row r="166" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>280</v>
       </c>
@@ -27114,7 +27115,7 @@
         <v>-46.395246</v>
       </c>
     </row>
-    <row r="167" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>280</v>
       </c>
@@ -27167,7 +27168,7 @@
         <v>-46.390622299999997</v>
       </c>
     </row>
-    <row r="168" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>280</v>
       </c>
@@ -27220,7 +27221,7 @@
         <v>-46.388130599999997</v>
       </c>
     </row>
-    <row r="169" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>305</v>
       </c>
@@ -27273,7 +27274,7 @@
         <v>-46.406078299999997</v>
       </c>
     </row>
-    <row r="170" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>305</v>
       </c>
@@ -27326,7 +27327,7 @@
         <v>-46.406567000000003</v>
       </c>
     </row>
-    <row r="171" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>305</v>
       </c>
@@ -27379,7 +27380,7 @@
         <v>-46.407268500000001</v>
       </c>
     </row>
-    <row r="172" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>305</v>
       </c>
@@ -27432,7 +27433,7 @@
         <v>-46.407628899999999</v>
       </c>
     </row>
-    <row r="173" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>305</v>
       </c>
@@ -27485,7 +27486,7 @@
         <v>-46.4079087</v>
       </c>
     </row>
-    <row r="174" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>305</v>
       </c>
@@ -27538,7 +27539,7 @@
         <v>-46.406060400000001</v>
       </c>
     </row>
-    <row r="175" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>305</v>
       </c>
@@ -27591,7 +27592,7 @@
         <v>-46.408232599999998</v>
       </c>
     </row>
-    <row r="176" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>305</v>
       </c>
@@ -27644,7 +27645,7 @@
         <v>-46.408232599999998</v>
       </c>
     </row>
-    <row r="177" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>305</v>
       </c>
@@ -27697,7 +27698,7 @@
         <v>-46.406567000000003</v>
       </c>
     </row>
-    <row r="178" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>305</v>
       </c>
@@ -27750,7 +27751,7 @@
         <v>-46.407268500000001</v>
       </c>
     </row>
-    <row r="179" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>305</v>
       </c>
@@ -27803,7 +27804,7 @@
         <v>-46.406331600000001</v>
       </c>
     </row>
-    <row r="180" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>305</v>
       </c>
@@ -27856,7 +27857,7 @@
         <v>-46.406856099999999</v>
       </c>
     </row>
-    <row r="181" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>312</v>
       </c>
@@ -27903,7 +27904,7 @@
         <v>-46.399636800000003</v>
       </c>
     </row>
-    <row r="182" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>312</v>
       </c>
@@ -27950,7 +27951,7 @@
         <v>-46.399317199999999</v>
       </c>
     </row>
-    <row r="183" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>312</v>
       </c>
@@ -27997,7 +27998,7 @@
         <v>-46.398956400000003</v>
       </c>
     </row>
-    <row r="184" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>312</v>
       </c>
@@ -28044,7 +28045,7 @@
         <v>-46.398719900000003</v>
       </c>
     </row>
-    <row r="185" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>312</v>
       </c>
@@ -28091,7 +28092,7 @@
         <v>-46.398701299999999</v>
       </c>
     </row>
-    <row r="186" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>312</v>
       </c>
@@ -28138,7 +28139,7 @@
         <v>-46.398651000000001</v>
       </c>
     </row>
-    <row r="187" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>312</v>
       </c>
@@ -28185,7 +28186,7 @@
         <v>-46.398395800000003</v>
       </c>
     </row>
-    <row r="188" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>312</v>
       </c>
@@ -28232,7 +28233,7 @@
         <v>-46.397748900000003</v>
       </c>
     </row>
-    <row r="189" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>312</v>
       </c>
@@ -28279,7 +28280,7 @@
         <v>-46.397582200000002</v>
       </c>
     </row>
-    <row r="190" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>312</v>
       </c>
@@ -28326,7 +28327,7 @@
         <v>-46.397804000000001</v>
       </c>
     </row>
-    <row r="191" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>312</v>
       </c>
@@ -28373,7 +28374,7 @@
         <v>-46.398719900000003</v>
       </c>
     </row>
-    <row r="192" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>312</v>
       </c>
@@ -28420,7 +28421,7 @@
         <v>-46.3982283</v>
       </c>
     </row>
-    <row r="193" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>312</v>
       </c>
@@ -28467,7 +28468,7 @@
         <v>-46.3982283</v>
       </c>
     </row>
-    <row r="194" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>312</v>
       </c>
@@ -28514,7 +28515,7 @@
         <v>-46.398651000000001</v>
       </c>
     </row>
-    <row r="195" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>312</v>
       </c>
@@ -28561,7 +28562,7 @@
         <v>-46.397804000000001</v>
       </c>
     </row>
-    <row r="196" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>317</v>
       </c>
@@ -28614,7 +28615,7 @@
         <v>-46.395039500000003</v>
       </c>
     </row>
-    <row r="197" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>317</v>
       </c>
@@ -28667,7 +28668,7 @@
         <v>-46.399920799999997</v>
       </c>
     </row>
-    <row r="198" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>317</v>
       </c>
@@ -28720,7 +28721,7 @@
         <v>-46.399732299999997</v>
       </c>
     </row>
-    <row r="199" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>317</v>
       </c>
@@ -28773,7 +28774,7 @@
         <v>-46.402293800000002</v>
       </c>
     </row>
-    <row r="200" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>317</v>
       </c>
@@ -28826,7 +28827,7 @@
         <v>-46.401741199999996</v>
       </c>
     </row>
-    <row r="201" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>317</v>
       </c>
@@ -28879,7 +28880,7 @@
         <v>-46.4013214</v>
       </c>
     </row>
-    <row r="202" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>317</v>
       </c>
@@ -28932,7 +28933,7 @@
         <v>-46.400779200000002</v>
       </c>
     </row>
-    <row r="203" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>317</v>
       </c>
@@ -28985,7 +28986,7 @@
         <v>-46.400237500000003</v>
       </c>
     </row>
-    <row r="204" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>317</v>
       </c>
@@ -29038,7 +29039,7 @@
         <v>-46.400053399999997</v>
       </c>
     </row>
-    <row r="205" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>317</v>
       </c>
@@ -29091,7 +29092,7 @@
         <v>-46.397993399999997</v>
       </c>
     </row>
-    <row r="206" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>317</v>
       </c>
@@ -29144,7 +29145,7 @@
         <v>-46.3980842</v>
       </c>
     </row>
-    <row r="207" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>317</v>
       </c>
@@ -29197,7 +29198,7 @@
         <v>-46.398204</v>
       </c>
     </row>
-    <row r="208" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>317</v>
       </c>
@@ -29250,7 +29251,7 @@
         <v>-46.398731099999999</v>
       </c>
     </row>
-    <row r="209" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>317</v>
       </c>
@@ -29303,7 +29304,7 @@
         <v>-46.398578299999997</v>
       </c>
     </row>
-    <row r="210" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>317</v>
       </c>
@@ -29356,7 +29357,7 @@
         <v>-46.399111300000001</v>
       </c>
     </row>
-    <row r="211" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>317</v>
       </c>
@@ -29409,7 +29410,7 @@
         <v>-46.399396500000002</v>
       </c>
     </row>
-    <row r="212" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>317</v>
       </c>
@@ -29462,7 +29463,7 @@
         <v>-46.3996371</v>
       </c>
     </row>
-    <row r="213" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>317</v>
       </c>
@@ -29515,7 +29516,7 @@
         <v>-46.399732299999997</v>
       </c>
     </row>
-    <row r="214" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>317</v>
       </c>
@@ -29568,7 +29569,7 @@
         <v>-46.397703300000003</v>
       </c>
     </row>
-    <row r="215" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>317</v>
       </c>
@@ -29621,7 +29622,7 @@
         <v>-46.397365899999997</v>
       </c>
     </row>
-    <row r="216" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>317</v>
       </c>
@@ -29674,7 +29675,7 @@
         <v>-46.396937700000002</v>
       </c>
     </row>
-    <row r="217" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>317</v>
       </c>
@@ -29727,7 +29728,7 @@
         <v>-46.396631800000002</v>
       </c>
     </row>
-    <row r="218" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>317</v>
       </c>
@@ -29780,7 +29781,7 @@
         <v>-46.396280500000003</v>
       </c>
     </row>
-    <row r="219" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>317</v>
       </c>
@@ -29833,7 +29834,7 @@
         <v>-46.395845000000001</v>
       </c>
     </row>
-    <row r="220" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>317</v>
       </c>
@@ -29886,7 +29887,7 @@
         <v>-46.395425600000003</v>
       </c>
     </row>
-    <row r="221" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>317</v>
       </c>
@@ -29939,7 +29940,7 @@
         <v>-46.395425600000003</v>
       </c>
     </row>
-    <row r="222" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>317</v>
       </c>
@@ -29992,7 +29993,7 @@
         <v>-46.393717500000001</v>
       </c>
     </row>
-    <row r="223" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>317</v>
       </c>
@@ -30045,7 +30046,7 @@
         <v>-46.393569399999997</v>
       </c>
     </row>
-    <row r="224" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>317</v>
       </c>
@@ -30098,7 +30099,7 @@
         <v>-46.393071999999997</v>
       </c>
     </row>
-    <row r="225" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>317</v>
       </c>
@@ -30151,7 +30152,7 @@
         <v>-46.392376200000001</v>
       </c>
     </row>
-    <row r="226" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>317</v>
       </c>
@@ -30204,7 +30205,7 @@
         <v>-46.3960948</v>
       </c>
     </row>
-    <row r="227" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>317</v>
       </c>
@@ -30257,7 +30258,7 @@
         <v>-46.398731099999999</v>
       </c>
     </row>
-    <row r="228" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>317</v>
       </c>
@@ -30310,7 +30311,7 @@
         <v>-46.4022632</v>
       </c>
     </row>
-    <row r="229" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>317</v>
       </c>
@@ -30363,7 +30364,7 @@
         <v>-46.395845000000001</v>
       </c>
     </row>
-    <row r="230" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>317</v>
       </c>
@@ -30416,7 +30417,7 @@
         <v>-46.3960948</v>
       </c>
     </row>
-    <row r="231" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>317</v>
       </c>
@@ -30469,7 +30470,7 @@
         <v>-46.396000600000001</v>
       </c>
     </row>
-    <row r="232" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>317</v>
       </c>
@@ -30522,7 +30523,7 @@
         <v>-46.395630199999999</v>
       </c>
     </row>
-    <row r="233" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>317</v>
       </c>
@@ -30575,7 +30576,7 @@
         <v>-46.397993399999997</v>
       </c>
     </row>
-    <row r="234" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>317</v>
       </c>
@@ -30628,7 +30629,7 @@
         <v>-46.397993399999997</v>
       </c>
     </row>
-    <row r="235" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>317</v>
       </c>
@@ -30681,7 +30682,7 @@
         <v>-46.397979200000002</v>
       </c>
     </row>
-    <row r="236" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>317</v>
       </c>
@@ -30734,7 +30735,7 @@
         <v>-46.3980842</v>
       </c>
     </row>
-    <row r="237" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>317</v>
       </c>
@@ -30784,7 +30785,7 @@
         <v>-46.398089400000003</v>
       </c>
     </row>
-    <row r="238" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>317</v>
       </c>
@@ -30837,7 +30838,7 @@
         <v>-46.392376200000001</v>
       </c>
     </row>
-    <row r="239" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>317</v>
       </c>
@@ -30890,7 +30891,7 @@
         <v>-46.390559500000002</v>
       </c>
     </row>
-    <row r="240" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>317</v>
       </c>
@@ -30943,7 +30944,7 @@
         <v>-46.391169300000001</v>
       </c>
     </row>
-    <row r="241" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>317</v>
       </c>
@@ -30996,7 +30997,7 @@
         <v>-46.391454299999999</v>
       </c>
     </row>
-    <row r="242" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>317</v>
       </c>
@@ -31049,7 +31050,7 @@
         <v>-46.391380099999999</v>
       </c>
     </row>
-    <row r="243" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>317</v>
       </c>
@@ -31102,7 +31103,7 @@
         <v>-46.392123900000001</v>
       </c>
     </row>
-    <row r="244" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>317</v>
       </c>
@@ -31155,7 +31156,7 @@
         <v>-46.391454400000001</v>
       </c>
     </row>
-    <row r="245" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>317</v>
       </c>
@@ -31208,7 +31209,7 @@
         <v>-46.391457500000001</v>
       </c>
     </row>
-    <row r="246" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>317</v>
       </c>
@@ -31261,7 +31262,7 @@
         <v>-46.390500799999998</v>
       </c>
     </row>
-    <row r="247" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>317</v>
       </c>
@@ -31314,7 +31315,7 @@
         <v>-46.390509799999997</v>
       </c>
     </row>
-    <row r="248" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>317</v>
       </c>
@@ -31367,7 +31368,7 @@
         <v>-46.391380099999999</v>
       </c>
     </row>
-    <row r="249" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>317</v>
       </c>
@@ -31420,7 +31421,7 @@
         <v>-46.390866699999997</v>
       </c>
     </row>
-    <row r="250" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>317</v>
       </c>
@@ -31473,7 +31474,7 @@
         <v>-46.390534500000001</v>
       </c>
     </row>
-    <row r="251" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>317</v>
       </c>
@@ -31526,7 +31527,7 @@
         <v>-46.391384500000001</v>
       </c>
     </row>
-    <row r="252" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>352</v>
       </c>
@@ -31579,7 +31580,7 @@
         <v>-46.392097399999997</v>
       </c>
     </row>
-    <row r="253" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>352</v>
       </c>
@@ -31632,7 +31633,7 @@
         <v>-46.391953299999997</v>
       </c>
     </row>
-    <row r="254" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>352</v>
       </c>
@@ -31685,7 +31686,7 @@
         <v>-46.391780500000003</v>
       </c>
     </row>
-    <row r="255" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>352</v>
       </c>
@@ -31738,7 +31739,7 @@
         <v>-46.392170900000004</v>
       </c>
     </row>
-    <row r="256" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>352</v>
       </c>
@@ -31791,7 +31792,7 @@
         <v>-46.392086900000002</v>
       </c>
     </row>
-    <row r="257" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>352</v>
       </c>
@@ -31844,7 +31845,7 @@
         <v>-46.392177699999998</v>
       </c>
     </row>
-    <row r="258" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>352</v>
       </c>
@@ -31897,7 +31898,7 @@
         <v>-46.392434799999997</v>
       </c>
     </row>
-    <row r="259" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>352</v>
       </c>
@@ -31950,7 +31951,7 @@
         <v>-46.3926789</v>
       </c>
     </row>
-    <row r="260" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>352</v>
       </c>
@@ -32003,7 +32004,7 @@
         <v>-46.392434799999997</v>
       </c>
     </row>
-    <row r="261" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>352</v>
       </c>
@@ -32056,7 +32057,7 @@
         <v>-46.392170900000004</v>
       </c>
     </row>
-    <row r="262" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>352</v>
       </c>
@@ -32109,7 +32110,7 @@
         <v>-46.391780500000003</v>
       </c>
     </row>
-    <row r="263" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>352</v>
       </c>
@@ -32162,7 +32163,7 @@
         <v>-46.392123900000001</v>
       </c>
     </row>
-    <row r="264" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>352</v>
       </c>
@@ -32215,7 +32216,7 @@
         <v>-46.392097399999997</v>
       </c>
     </row>
-    <row r="265" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>352</v>
       </c>
@@ -32268,7 +32269,7 @@
         <v>-46.391780699999998</v>
       </c>
     </row>
-    <row r="266" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>355</v>
       </c>
@@ -32321,7 +32322,7 @@
         <v>-46.391734700000001</v>
       </c>
     </row>
-    <row r="267" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>355</v>
       </c>
@@ -32374,7 +32375,7 @@
         <v>-46.391399900000003</v>
       </c>
     </row>
-    <row r="268" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>355</v>
       </c>
@@ -32427,7 +32428,7 @@
         <v>-46.390832000000003</v>
       </c>
     </row>
-    <row r="269" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>355</v>
       </c>
@@ -32480,7 +32481,7 @@
         <v>-46.390766499999998</v>
       </c>
     </row>
-    <row r="270" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>355</v>
       </c>
@@ -32533,7 +32534,7 @@
         <v>-46.390832000000003</v>
       </c>
     </row>
-    <row r="271" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>355</v>
       </c>
@@ -32586,7 +32587,7 @@
         <v>-46.390613000000002</v>
       </c>
     </row>
-    <row r="272" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>355</v>
       </c>
@@ -32639,7 +32640,7 @@
         <v>-46.390234300000003</v>
       </c>
     </row>
-    <row r="273" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>355</v>
       </c>
@@ -32692,7 +32693,7 @@
         <v>-46.389846900000002</v>
       </c>
     </row>
-    <row r="274" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>355</v>
       </c>
@@ -32745,7 +32746,7 @@
         <v>-46.3894801</v>
       </c>
     </row>
-    <row r="275" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>355</v>
       </c>
@@ -32798,7 +32799,7 @@
         <v>-46.389092400000003</v>
       </c>
     </row>
-    <row r="276" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>355</v>
       </c>
@@ -32851,7 +32852,7 @@
         <v>-46.388676799999999</v>
       </c>
     </row>
-    <row r="277" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>355</v>
       </c>
@@ -32904,7 +32905,7 @@
         <v>-46.386397299999999</v>
       </c>
     </row>
-    <row r="278" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>355</v>
       </c>
@@ -32957,7 +32958,7 @@
         <v>-46.387154600000002</v>
       </c>
     </row>
-    <row r="279" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>355</v>
       </c>
@@ -33010,7 +33011,7 @@
         <v>-46.3879375</v>
       </c>
     </row>
-    <row r="280" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>355</v>
       </c>
@@ -33063,7 +33064,7 @@
         <v>-46.3859675</v>
       </c>
     </row>
-    <row r="281" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>355</v>
       </c>
@@ -33116,7 +33117,7 @@
         <v>-46.3862132</v>
       </c>
     </row>
-    <row r="282" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>355</v>
       </c>
@@ -33169,7 +33170,7 @@
         <v>-46.3863129</v>
       </c>
     </row>
-    <row r="283" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>355</v>
       </c>
@@ -33222,7 +33223,7 @@
         <v>-46.386583299999998</v>
       </c>
     </row>
-    <row r="284" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>355</v>
       </c>
@@ -33275,7 +33276,7 @@
         <v>-46.392179599999999</v>
       </c>
     </row>
-    <row r="285" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>355</v>
       </c>
@@ -33328,7 +33329,7 @@
         <v>-46.388432899999998</v>
       </c>
     </row>
-    <row r="286" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>355</v>
       </c>
@@ -33381,7 +33382,7 @@
         <v>-46.388676799999999</v>
       </c>
     </row>
-    <row r="287" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>363</v>
       </c>
@@ -33434,7 +33435,7 @@
         <v>-46.397681599999999</v>
       </c>
     </row>
-    <row r="288" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>363</v>
       </c>
@@ -33487,7 +33488,7 @@
         <v>-46.3974324</v>
       </c>
     </row>
-    <row r="289" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>363</v>
       </c>
@@ -33540,7 +33541,7 @@
         <v>-46.396907200000001</v>
       </c>
     </row>
-    <row r="290" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>363</v>
       </c>
@@ -33593,7 +33594,7 @@
         <v>-46.396283199999999</v>
       </c>
     </row>
-    <row r="291" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>363</v>
       </c>
@@ -33646,7 +33647,7 @@
         <v>-46.396234700000001</v>
       </c>
     </row>
-    <row r="292" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>363</v>
       </c>
@@ -33699,7 +33700,7 @@
         <v>-46.396234700000001</v>
       </c>
     </row>
-    <row r="293" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>363</v>
       </c>
@@ -33752,7 +33753,7 @@
         <v>-46.395672300000001</v>
       </c>
     </row>
-    <row r="294" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>363</v>
       </c>
@@ -33805,7 +33806,7 @@
         <v>-46.394411300000002</v>
       </c>
     </row>
-    <row r="295" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>363</v>
       </c>
@@ -33858,7 +33859,7 @@
         <v>-46.393959799999998</v>
       </c>
     </row>
-    <row r="296" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>363</v>
       </c>
@@ -33911,7 +33912,7 @@
         <v>-46.3936408</v>
       </c>
     </row>
-    <row r="297" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>363</v>
       </c>
@@ -33964,7 +33965,7 @@
         <v>-46.393255099999998</v>
       </c>
     </row>
-    <row r="298" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>363</v>
       </c>
@@ -34017,7 +34018,7 @@
         <v>-46.396111300000001</v>
       </c>
     </row>
-    <row r="299" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>363</v>
       </c>
@@ -34070,7 +34071,7 @@
         <v>-46.395125499999999</v>
       </c>
     </row>
-    <row r="300" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>363</v>
       </c>
@@ -34123,7 +34124,7 @@
         <v>-46.397876199999999</v>
       </c>
     </row>
-    <row r="301" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>363</v>
       </c>
@@ -34176,7 +34177,7 @@
         <v>-46.394917599999999</v>
       </c>
     </row>
-    <row r="302" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>363</v>
       </c>
@@ -34229,7 +34230,7 @@
         <v>-46.394633800000001</v>
       </c>
     </row>
-    <row r="303" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>363</v>
       </c>
@@ -34282,7 +34283,7 @@
         <v>-46.392941700000002</v>
       </c>
     </row>
-    <row r="304" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>363</v>
       </c>
@@ -34335,7 +34336,7 @@
         <v>-46.390125500000003</v>
       </c>
     </row>
-    <row r="305" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>363</v>
       </c>
@@ -34388,7 +34389,7 @@
         <v>-46.390125500000003</v>
       </c>
     </row>
-    <row r="306" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>363</v>
       </c>
@@ -34441,7 +34442,7 @@
         <v>-46.389316899999997</v>
       </c>
     </row>
-    <row r="307" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>363</v>
       </c>
@@ -34494,7 +34495,7 @@
         <v>-46.388850499999997</v>
       </c>
     </row>
-    <row r="308" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>363</v>
       </c>
@@ -34547,7 +34548,7 @@
         <v>-46.388869300000003</v>
       </c>
     </row>
-    <row r="309" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>363</v>
       </c>
@@ -34600,7 +34601,7 @@
         <v>-46.388991099999998</v>
       </c>
     </row>
-    <row r="310" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>363</v>
       </c>
@@ -34653,7 +34654,7 @@
         <v>-46.389474800000002</v>
       </c>
     </row>
-    <row r="311" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>363</v>
       </c>
@@ -34706,7 +34707,7 @@
         <v>-46.389775499999999</v>
       </c>
     </row>
-    <row r="312" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>363</v>
       </c>
@@ -34759,7 +34760,7 @@
         <v>-46.3911503</v>
       </c>
     </row>
-    <row r="313" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>363</v>
       </c>
@@ -34812,7 +34813,7 @@
         <v>-46.390674300000001</v>
       </c>
     </row>
-    <row r="314" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>363</v>
       </c>
@@ -34865,7 +34866,7 @@
         <v>-46.390674300000001</v>
       </c>
     </row>
-    <row r="315" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>363</v>
       </c>
@@ -34918,7 +34919,7 @@
         <v>-46.390674300000001</v>
       </c>
     </row>
-    <row r="316" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>363</v>
       </c>
@@ -34971,7 +34972,7 @@
         <v>-46.390125500000003</v>
       </c>
     </row>
-    <row r="317" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>363</v>
       </c>
@@ -35024,7 +35025,7 @@
         <v>-46.3936408</v>
       </c>
     </row>
-    <row r="318" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>363</v>
       </c>
@@ -35077,7 +35078,7 @@
         <v>-46.392461500000003</v>
       </c>
     </row>
-    <row r="319" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>363</v>
       </c>
@@ -35130,7 +35131,7 @@
         <v>-46.392190599999999</v>
       </c>
     </row>
-    <row r="320" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>363</v>
       </c>
@@ -35183,7 +35184,7 @@
         <v>-46.391619599999999</v>
       </c>
     </row>
-    <row r="321" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>363</v>
       </c>
@@ -35236,7 +35237,7 @@
         <v>-46.392941700000002</v>
       </c>
     </row>
-    <row r="322" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>363</v>
       </c>
@@ -35289,7 +35290,7 @@
         <v>-46.389474800000002</v>
       </c>
     </row>
-    <row r="323" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>363</v>
       </c>
@@ -35342,7 +35343,7 @@
         <v>-46.393255099999998</v>
       </c>
     </row>
-    <row r="324" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>363</v>
       </c>
@@ -35395,7 +35396,7 @@
         <v>-46.393256299999997</v>
       </c>
     </row>
-    <row r="325" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>363</v>
       </c>
@@ -35448,7 +35449,7 @@
         <v>-46.393255099999998</v>
       </c>
     </row>
-    <row r="326" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>363</v>
       </c>
@@ -35501,7 +35502,7 @@
         <v>-46.392941700000002</v>
       </c>
     </row>
-    <row r="327" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>363</v>
       </c>
@@ -35554,7 +35555,7 @@
         <v>-46.392921100000002</v>
       </c>
     </row>
-    <row r="328" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>363</v>
       </c>
@@ -35607,7 +35608,7 @@
         <v>-46.392921100000002</v>
       </c>
     </row>
-    <row r="329" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>377</v>
       </c>
@@ -35660,7 +35661,7 @@
         <v>-46.399263099999999</v>
       </c>
     </row>
-    <row r="330" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>377</v>
       </c>
@@ -35713,7 +35714,7 @@
         <v>-46.400001500000002</v>
       </c>
     </row>
-    <row r="331" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>377</v>
       </c>
@@ -35766,7 +35767,7 @@
         <v>-46.400030800000003</v>
       </c>
     </row>
-    <row r="332" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>377</v>
       </c>
@@ -35819,7 +35820,7 @@
         <v>-46.398584399999997</v>
       </c>
     </row>
-    <row r="333" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>377</v>
       </c>
@@ -35872,7 +35873,7 @@
         <v>-46.399263099999999</v>
       </c>
     </row>
-    <row r="334" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>377</v>
       </c>
@@ -35925,7 +35926,7 @@
         <v>-46.399334099999997</v>
       </c>
     </row>
-    <row r="335" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>377</v>
       </c>
@@ -35978,7 +35979,7 @@
         <v>-46.399334099999997</v>
       </c>
     </row>
-    <row r="336" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>377</v>
       </c>
@@ -36031,7 +36032,7 @@
         <v>-46.398702299999997</v>
       </c>
     </row>
-    <row r="337" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>377</v>
       </c>
@@ -36084,7 +36085,7 @@
         <v>-46.398688399999998</v>
       </c>
     </row>
-    <row r="338" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>377</v>
       </c>
@@ -36137,7 +36138,7 @@
         <v>-46.398706799999999</v>
       </c>
     </row>
-    <row r="339" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>377</v>
       </c>
@@ -36190,7 +36191,7 @@
         <v>-46.398702299999997</v>
       </c>
     </row>
-    <row r="340" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>377</v>
       </c>
@@ -36243,7 +36244,7 @@
         <v>-46.400631799999999</v>
       </c>
     </row>
-    <row r="341" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>377</v>
       </c>
@@ -36296,7 +36297,7 @@
         <v>-46.401348900000002</v>
       </c>
     </row>
-    <row r="342" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>377</v>
       </c>
@@ -36337,7 +36338,7 @@
         <v>-46.401348900000002</v>
       </c>
     </row>
-    <row r="343" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>377</v>
       </c>
@@ -36378,7 +36379,7 @@
         <v>-46.401776300000002</v>
       </c>
     </row>
-    <row r="344" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>377</v>
       </c>
@@ -36419,7 +36420,7 @@
         <v>-46.401348900000002</v>
       </c>
     </row>
-    <row r="345" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>377</v>
       </c>
@@ -36472,7 +36473,7 @@
         <v>-46.401958399999998</v>
       </c>
     </row>
-    <row r="346" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>377</v>
       </c>
@@ -36525,7 +36526,7 @@
         <v>-46.402794299999996</v>
       </c>
     </row>
-    <row r="347" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>377</v>
       </c>
@@ -36578,7 +36579,7 @@
         <v>-46.402279700000001</v>
       </c>
     </row>
-    <row r="348" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>377</v>
       </c>
@@ -36631,7 +36632,7 @@
         <v>-46.402184699999999</v>
       </c>
     </row>
-    <row r="349" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>377</v>
       </c>
@@ -36684,7 +36685,7 @@
         <v>-46.402279700000001</v>
       </c>
     </row>
-    <row r="350" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>377</v>
       </c>
@@ -36737,7 +36738,7 @@
         <v>-46.401958399999998</v>
       </c>
     </row>
-    <row r="351" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>363</v>
       </c>
@@ -36793,7 +36794,7 @@
         <v>-46.3959507</v>
       </c>
     </row>
-    <row r="352" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>363</v>
       </c>
@@ -36849,7 +36850,7 @@
         <v>-46.396032599999998</v>
       </c>
     </row>
-    <row r="353" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>388</v>
       </c>
@@ -36905,7 +36906,7 @@
         <v>-46.385066799999997</v>
       </c>
     </row>
-    <row r="354" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>388</v>
       </c>
@@ -36961,7 +36962,7 @@
         <v>-46.3856647</v>
       </c>
     </row>
-    <row r="355" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>388</v>
       </c>
@@ -37017,7 +37018,7 @@
         <v>-46.386281199999999</v>
       </c>
     </row>
-    <row r="356" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>388</v>
       </c>
@@ -37073,7 +37074,7 @@
         <v>-46.385869399999997</v>
       </c>
     </row>
-    <row r="357" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>388</v>
       </c>
@@ -37129,7 +37130,7 @@
         <v>-46.385849999999998</v>
       </c>
     </row>
-    <row r="358" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>165</v>
       </c>
@@ -37185,7 +37186,7 @@
         <v>-46.393826947651448</v>
       </c>
     </row>
-    <row r="359" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>165</v>
       </c>
@@ -37241,7 +37242,7 @@
         <v>-46.392254815122861</v>
       </c>
     </row>
-    <row r="360" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>117</v>
       </c>
@@ -37297,7 +37298,7 @@
         <v>-46.4176511</v>
       </c>
     </row>
-    <row r="361" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>117</v>
       </c>
@@ -37353,7 +37354,7 @@
         <v>-46.415050600000001</v>
       </c>
     </row>
-    <row r="362" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>117</v>
       </c>
@@ -37409,7 +37410,7 @@
         <v>-46.416166400000002</v>
       </c>
     </row>
-    <row r="363" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>117</v>
       </c>
@@ -37659,7 +37660,7 @@
         <v>530</v>
       </c>
       <c r="I367">
-        <v>88.66</v>
+        <v>0</v>
       </c>
       <c r="J367">
         <v>7.38</v>
@@ -37745,7 +37746,7 @@
         <v>-46.401156800000003</v>
       </c>
     </row>
-    <row r="369" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>363</v>
       </c>
@@ -37801,7 +37802,7 @@
         <v>-46.396509199999997</v>
       </c>
     </row>
-    <row r="370" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>363</v>
       </c>
@@ -37857,7 +37858,7 @@
         <v>-46.396530900000002</v>
       </c>
     </row>
-    <row r="371" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>421</v>
       </c>
@@ -37913,7 +37914,7 @@
         <v>-46.388130599999997</v>
       </c>
     </row>
-    <row r="372" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>421</v>
       </c>
@@ -37969,7 +37970,7 @@
         <v>-46.388117800000003</v>
       </c>
     </row>
-    <row r="373" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>421</v>
       </c>
@@ -38025,7 +38026,7 @@
         <v>-46.388055299999998</v>
       </c>
     </row>
-    <row r="374" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>421</v>
       </c>
@@ -38081,7 +38082,7 @@
         <v>-46.3875758</v>
       </c>
     </row>
-    <row r="375" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>421</v>
       </c>
@@ -38137,7 +38138,7 @@
         <v>-46.387807600000002</v>
       </c>
     </row>
-    <row r="376" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>421</v>
       </c>
@@ -38193,7 +38194,7 @@
         <v>-46.388296699999998</v>
       </c>
     </row>
-    <row r="377" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>421</v>
       </c>
@@ -38249,7 +38250,7 @@
         <v>-46.388917999999997</v>
       </c>
     </row>
-    <row r="378" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>421</v>
       </c>
@@ -38305,7 +38306,7 @@
         <v>-46.389496999999999</v>
       </c>
     </row>
-    <row r="379" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>421</v>
       </c>
@@ -38361,7 +38362,7 @@
         <v>-46.390075299999999</v>
       </c>
     </row>
-    <row r="380" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>421</v>
       </c>
@@ -38417,7 +38418,7 @@
         <v>-46.390118399999999</v>
       </c>
     </row>
-    <row r="381" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>421</v>
       </c>
@@ -38473,7 +38474,7 @@
         <v>-46.388296699999998</v>
       </c>
     </row>
-    <row r="382" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>439</v>
       </c>
@@ -38529,7 +38530,7 @@
         <v>-46.416035000000001</v>
       </c>
     </row>
-    <row r="383" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>439</v>
       </c>
@@ -38585,7 +38586,7 @@
         <v>-46.416319799999997</v>
       </c>
     </row>
-    <row r="384" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>439</v>
       </c>
@@ -38641,7 +38642,7 @@
         <v>-46.4161942</v>
       </c>
     </row>
-    <row r="385" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>439</v>
       </c>
@@ -38697,7 +38698,7 @@
         <v>-46.416128800000003</v>
       </c>
     </row>
-    <row r="386" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>439</v>
       </c>
@@ -38753,7 +38754,7 @@
         <v>-46.416162700000001</v>
       </c>
     </row>
-    <row r="387" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>439</v>
       </c>
@@ -38809,7 +38810,7 @@
         <v>-46.416152199999999</v>
       </c>
     </row>
-    <row r="388" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>439</v>
       </c>
@@ -38866,7 +38867,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R388" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
+  <autoFilter ref="A1:R388" xr:uid="{00000000-0001-0000-0300-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="conceicao"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Corrige validacao CTS Joao Canzi
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1165,7 +1165,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>joao_canzi</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -18085,7 +18085,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>joao_canzi</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
@@ -18133,7 +18133,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>joao_canzi</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
@@ -45392,7 +45392,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>joao_canzi</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza PDS e plano de furo Joao Canzi
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1200,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L381"/>
+  <dimension ref="A1:L383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18385,6 +18385,102 @@
       <c r="L381" t="inlineStr">
         <is>
           <t>Atualizado via shape em 04/05/2026; CADASTRO PV - CT ÁGUA VERMELHA - MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>JC-PV-09</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>PV-09</t>
+        </is>
+      </c>
+      <c r="E382" t="n">
+        <v>7396914.814</v>
+      </c>
+      <c r="F382" t="n">
+        <v>358382.74</v>
+      </c>
+      <c r="G382" t="n">
+        <v>-23.5318788</v>
+      </c>
+      <c r="H382" t="n">
+        <v>-46.3872832</v>
+      </c>
+      <c r="I382" t="n">
+        <v>768.775</v>
+      </c>
+      <c r="J382" t="n">
+        <v>766.275</v>
+      </c>
+      <c r="K382" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-03/FL-04 versao 01, 11.MAI.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>JC-PV-10</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>PV-10</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>7396932.164</v>
+      </c>
+      <c r="F383" t="n">
+        <v>358437.094</v>
+      </c>
+      <c r="G383" t="n">
+        <v>-23.5317269</v>
+      </c>
+      <c r="H383" t="n">
+        <v>-46.3867492</v>
+      </c>
+      <c r="I383" t="n">
+        <v>770.008</v>
+      </c>
+      <c r="J383" t="n">
+        <v>767.008</v>
+      </c>
+      <c r="K383" t="n">
+        <v>3</v>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-04 versao 01, 11.MAI.2026</t>
         </is>
       </c>
     </row>
@@ -18399,7 +18495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R401"/>
+  <dimension ref="A1:R403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -46599,6 +46695,154 @@
       </c>
       <c r="R401" t="n">
         <v>-46.416679</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>JC-003</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>PV-08 - PV-09</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>PV-08</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>PV-09</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G402" t="n">
+        <v>355</v>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I402" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="J402" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K402" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L402" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>em planejamento</t>
+        </is>
+      </c>
+      <c r="N402" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-03 versao 01, 11.MAI.2026; GALPAO INTERNO RUA GENI GOMES; taxa 0,0311.</t>
+        </is>
+      </c>
+      <c r="O402" t="n">
+        <v>-23.5320183</v>
+      </c>
+      <c r="P402" t="n">
+        <v>-46.3877736</v>
+      </c>
+      <c r="Q402" t="n">
+        <v>-23.5318788</v>
+      </c>
+      <c r="R402" t="n">
+        <v>-46.3872832</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>JC-004</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>PV-09 - PV-10</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>PV-09</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>PV-10</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G403" t="n">
+        <v>355</v>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I403" t="n">
+        <v>56.92</v>
+      </c>
+      <c r="J403" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K403" t="n">
+        <v>3</v>
+      </c>
+      <c r="L403" t="n">
+        <v>3</v>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>em planejamento</t>
+        </is>
+      </c>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-04 versao 01, 11.MAI.2026; GALPAO INTERNO RUA GENI GOMES; taxa 0,0129.</t>
+        </is>
+      </c>
+      <c r="O403" t="n">
+        <v>-23.5318788</v>
+      </c>
+      <c r="P403" t="n">
+        <v>-46.3872832</v>
+      </c>
+      <c r="Q403" t="n">
+        <v>-23.5317269</v>
+      </c>
+      <c r="R403" t="n">
+        <v>-46.3867492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza PDS 2026-05-20 e planos de furo
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="31.109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1184,6 +1184,33 @@
         </is>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>cts_lourdes_complementar</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CTS Lourdes Complementar</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CTS</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Base criada a partir do plano de furo CT LOURDES FL-01 PV-01 ao PV-02, 14.MAI.2026.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1200,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L383"/>
+  <dimension ref="A1:L386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18481,6 +18508,150 @@
       <c r="L383" t="inlineStr">
         <is>
           <t>Plano de furo FL-04 versao 01, 11.MAI.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>cts_lourdes_complementar</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>LOUR-PV-01</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>PV-01</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>7397151.558</v>
+      </c>
+      <c r="F384" t="n">
+        <v>357586.89</v>
+      </c>
+      <c r="G384" t="n">
+        <v>-23.5296713</v>
+      </c>
+      <c r="H384" t="n">
+        <v>-46.395055</v>
+      </c>
+      <c r="I384" t="n">
+        <v>754.7190000000001</v>
+      </c>
+      <c r="J384" t="n">
+        <v>751.2190000000001</v>
+      </c>
+      <c r="K384" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-01 versao 01, 14.MAI.2026; ALARGADOR 700mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>cts_lourdes_complementar</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>LOUR-PV-02</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>PV-02</t>
+        </is>
+      </c>
+      <c r="E385" t="n">
+        <v>7397168.003</v>
+      </c>
+      <c r="F385" t="n">
+        <v>357669.586</v>
+      </c>
+      <c r="G385" t="n">
+        <v>-23.52953</v>
+      </c>
+      <c r="H385" t="n">
+        <v>-46.3942436</v>
+      </c>
+      <c r="I385" t="n">
+        <v>756.086</v>
+      </c>
+      <c r="J385" t="n">
+        <v>752.086</v>
+      </c>
+      <c r="K385" t="n">
+        <v>4</v>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-01 versao 01, 14.MAI.2026; ALARGADOR 700mm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>JC-PV-02</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>PV-02</t>
+        </is>
+      </c>
+      <c r="E386" t="n">
+        <v>7396941.756</v>
+      </c>
+      <c r="F386" t="n">
+        <v>358324.032</v>
+      </c>
+      <c r="G386" t="n">
+        <v>-23.5316304</v>
+      </c>
+      <c r="H386" t="n">
+        <v>-46.3878556</v>
+      </c>
+      <c r="I386" t="n">
+        <v>767.318</v>
+      </c>
+      <c r="J386" t="n">
+        <v>763.468</v>
+      </c>
+      <c r="K386" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-06 versao 01, 15.MAI.2026; RUA ELVIRA DE ARAUJO.</t>
         </is>
       </c>
     </row>
@@ -18495,7 +18666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R403"/>
+  <dimension ref="A1:R405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -46843,6 +47014,154 @@
       </c>
       <c r="R403" t="n">
         <v>-46.3867492</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>cts_lourdes_complementar</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>LOUR-001</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>PV-01 - PV-02</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>PV-01</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>PV-02</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G404" t="n">
+        <v>450</v>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I404" t="n">
+        <v>84.31999999999999</v>
+      </c>
+      <c r="J404" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="K404" t="n">
+        <v>4</v>
+      </c>
+      <c r="L404" t="n">
+        <v>4</v>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>em planejamento</t>
+        </is>
+      </c>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-01 versao 01, 14.MAI.2026; RUA GONCALVES CASTELAO; ALARGADOR 700mm; taxa 0,0103.</t>
+        </is>
+      </c>
+      <c r="O404" t="n">
+        <v>-23.5296713</v>
+      </c>
+      <c r="P404" t="n">
+        <v>-46.395055</v>
+      </c>
+      <c r="Q404" t="n">
+        <v>-23.52953</v>
+      </c>
+      <c r="R404" t="n">
+        <v>-46.3942436</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>JC-005</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>PV-08 - PV-02</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>PV-08</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>PV-02</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G405" t="n">
+        <v>355</v>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I405" t="n">
+        <v>43.66</v>
+      </c>
+      <c r="J405" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="K405" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="L405" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>em planejamento</t>
+        </is>
+      </c>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-06 versao 01, 15.MAI.2026; RUA ELVIRA DE ARAUJO; taxa 0,0108.</t>
+        </is>
+      </c>
+      <c r="O405" t="n">
+        <v>-23.5320183</v>
+      </c>
+      <c r="P405" t="n">
+        <v>-46.3877736</v>
+      </c>
+      <c r="Q405" t="n">
+        <v>-23.5316304</v>
+      </c>
+      <c r="R405" t="n">
+        <v>-46.3878556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona PV 11 ao PV 13 no mapa
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1227,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L386"/>
+  <dimension ref="A1:L388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18652,6 +18652,102 @@
       <c r="L386" t="inlineStr">
         <is>
           <t>Plano de furo FL-06 versao 01, 15.MAI.2026; RUA ELVIRA DE ARAUJO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>JC-PV-11</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>PV-11</t>
+        </is>
+      </c>
+      <c r="E387" t="n">
+        <v>7396951.048</v>
+      </c>
+      <c r="F387" t="n">
+        <v>358496.854</v>
+      </c>
+      <c r="G387" t="n">
+        <v>-23.5315615</v>
+      </c>
+      <c r="H387" t="n">
+        <v>-46.3861622</v>
+      </c>
+      <c r="I387" t="n">
+        <v>774.981</v>
+      </c>
+      <c r="J387" t="n">
+        <v>768.881</v>
+      </c>
+      <c r="K387" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; trecho PV-11 ao PV-13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>JC-PV-13</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>PV-13</t>
+        </is>
+      </c>
+      <c r="E388" t="n">
+        <v>7397011.057</v>
+      </c>
+      <c r="F388" t="n">
+        <v>358478.68</v>
+      </c>
+      <c r="G388" t="n">
+        <v>-23.5310181</v>
+      </c>
+      <c r="H388" t="n">
+        <v>-46.3863345</v>
+      </c>
+      <c r="I388" t="n">
+        <v>771.8630000000001</v>
+      </c>
+      <c r="J388" t="n">
+        <v>769.8630000000001</v>
+      </c>
+      <c r="K388" t="n">
+        <v>2</v>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; trecho PV-11 ao PV-13.</t>
         </is>
       </c>
     </row>
@@ -18666,7 +18762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R405"/>
+  <dimension ref="A1:R406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -47162,6 +47258,80 @@
       </c>
       <c r="R405" t="n">
         <v>-46.3878556</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>JC-006</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>PV-11 - PV-13</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>PV-11</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>PV-13</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G406" t="n">
+        <v>355</v>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I406" t="n">
+        <v>62.701</v>
+      </c>
+      <c r="J406" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="K406" t="n">
+        <v>2</v>
+      </c>
+      <c r="L406" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-11 ao PV-13; arquivo: planos_furo/cts_joao_canzi_fl07_pv11_pv13.pdf.</t>
+        </is>
+      </c>
+      <c r="O406" t="n">
+        <v>-23.5315615</v>
+      </c>
+      <c r="P406" t="n">
+        <v>-46.3861622</v>
+      </c>
+      <c r="Q406" t="n">
+        <v>-23.5310181</v>
+      </c>
+      <c r="R406" t="n">
+        <v>-46.3863345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona planos de furo Joao Canzi PV14 PV16
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1227,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L390"/>
+  <dimension ref="A1:L392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18844,6 +18844,102 @@
       <c r="L390" t="inlineStr">
         <is>
           <t>Plano de furo FL-02 versao 01, 14.MAI.2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>JC-PV-15</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>PV-15</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>7397079.185</v>
+      </c>
+      <c r="F391" t="n">
+        <v>358592.41</v>
+      </c>
+      <c r="G391" t="n">
+        <v>-23.5304128</v>
+      </c>
+      <c r="H391" t="n">
+        <v>-46.3852142</v>
+      </c>
+      <c r="I391" t="n">
+        <v>779.073</v>
+      </c>
+      <c r="J391" t="n">
+        <v>773.574</v>
+      </c>
+      <c r="K391" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; trecho PV-14 ao PV-15; arquivo: planos_furo/cts_joao_canzi_fl07_pv14_pv15.pdf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>JC-PV-16</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>PV-16</t>
+        </is>
+      </c>
+      <c r="E392" t="n">
+        <v>7397127.313</v>
+      </c>
+      <c r="F392" t="n">
+        <v>358662.509</v>
+      </c>
+      <c r="G392" t="n">
+        <v>-23.5299843</v>
+      </c>
+      <c r="H392" t="n">
+        <v>-46.3845231</v>
+      </c>
+      <c r="I392" t="n">
+        <v>777.73</v>
+      </c>
+      <c r="J392" t="n">
+        <v>774.633</v>
+      </c>
+      <c r="K392" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-01 versao 01, 26.MAI.2026; trecho PV-15 ao PV-16; arquivo: planos_furo/cts_joao_canzi_fl01_pv15_pv16.pdf.</t>
         </is>
       </c>
     </row>
@@ -18858,7 +18954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R408"/>
+  <dimension ref="A1:R410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -47576,6 +47672,154 @@
       </c>
       <c r="R408" t="n">
         <v>-46.3936017</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>JC-008</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>PV-14 - PV-15</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>PV-14</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>PV-15</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G409" t="n">
+        <v>355</v>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I409" t="n">
+        <v>52.62</v>
+      </c>
+      <c r="J409" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K409" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="L409" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-14 ao PV-15; arquivo: planos_furo/cts_joao_canzi_fl07_pv14_pv15.pdf; taxa 0,0095.</t>
+        </is>
+      </c>
+      <c r="O409" t="n">
+        <v>-23.5306805</v>
+      </c>
+      <c r="P409" t="n">
+        <v>-46.38564</v>
+      </c>
+      <c r="Q409" t="n">
+        <v>-23.5304128</v>
+      </c>
+      <c r="R409" t="n">
+        <v>-46.3852142</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>JC-009</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>PV-15 - PV-16</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>PV-15</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>PV-16</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G410" t="n">
+        <v>355</v>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I410" t="n">
+        <v>85.03</v>
+      </c>
+      <c r="J410" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K410" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="L410" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N410" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-01 versao 01, 26.MAI.2026; PV-15 ao PV-16; arquivo: planos_furo/cts_joao_canzi_fl01_pv15_pv16.pdf; taxa 0,0125.</t>
+        </is>
+      </c>
+      <c r="O410" t="n">
+        <v>-23.5304128</v>
+      </c>
+      <c r="P410" t="n">
+        <v>-46.3852142</v>
+      </c>
+      <c r="Q410" t="n">
+        <v>-23.5299843</v>
+      </c>
+      <c r="R410" t="n">
+        <v>-46.3845231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza mapa Lourdes Complementar
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -18850,7 +18850,7 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>cts_lourdes_complementar</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
@@ -18860,45 +18860,45 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>JC-PV-15</t>
+          <t>LOUR-PV-04</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>PV-15</t>
+          <t>PV-04</t>
         </is>
       </c>
       <c r="E391" t="n">
-        <v>7397079.185</v>
+        <v>7397095.58</v>
       </c>
       <c r="F391" t="n">
-        <v>358592.41</v>
+        <v>357808.575</v>
       </c>
       <c r="G391" t="n">
-        <v>-23.5304128</v>
+        <v>-23.5301962</v>
       </c>
       <c r="H391" t="n">
-        <v>-46.3852142</v>
+        <v>-46.3928893</v>
       </c>
       <c r="I391" t="n">
-        <v>779.073</v>
+        <v>759.482</v>
       </c>
       <c r="J391" t="n">
-        <v>773.574</v>
+        <v>754.482</v>
       </c>
       <c r="K391" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; trecho PV-14 ao PV-15; arquivo: planos_furo/cts_joao_canzi_fl07_pv14_pv15.pdf.</t>
+          <t>Plano de furo FL-02 versao 01, 26.MAI.2026; PV-03 ao PV-04.</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>cts_lourdes_complementar</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -18908,38 +18908,38 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>JC-PV-16</t>
+          <t>LOUR-PV-05</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>PV-16</t>
+          <t>PV-05</t>
         </is>
       </c>
       <c r="E392" t="n">
-        <v>7397127.313</v>
+        <v>7397066.391</v>
       </c>
       <c r="F392" t="n">
-        <v>358662.509</v>
+        <v>357868.405</v>
       </c>
       <c r="G392" t="n">
-        <v>-23.5299843</v>
+        <v>-23.530465</v>
       </c>
       <c r="H392" t="n">
-        <v>-46.3845231</v>
+        <v>-46.3923061</v>
       </c>
       <c r="I392" t="n">
-        <v>777.73</v>
+        <v>757.627</v>
       </c>
       <c r="J392" t="n">
-        <v>774.633</v>
+        <v>755.427</v>
       </c>
       <c r="K392" t="n">
-        <v>3.1</v>
+        <v>2.2</v>
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t>Plano de furo FL-01 versao 01, 26.MAI.2026; trecho PV-15 ao PV-16; arquivo: planos_furo/cts_joao_canzi_fl01_pv15_pv16.pdf.</t>
+          <t>Plano de furo FL-02 versao 01, 26.MAI.2026; PV-04 ao PV-05.</t>
         </is>
       </c>
     </row>
@@ -47677,27 +47677,27 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>cts_lourdes_complementar</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>JC-008</t>
+          <t>LOUR-003</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>PV-14 - PV-15</t>
+          <t>PV-03 - PV-04</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>PV-14</t>
+          <t>PV-03</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>PV-15</t>
+          <t>PV-04</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
@@ -47706,7 +47706,7 @@
         </is>
       </c>
       <c r="G409" t="n">
-        <v>355</v>
+        <v>450</v>
       </c>
       <c r="H409" t="inlineStr">
         <is>
@@ -47714,64 +47714,64 @@
         </is>
       </c>
       <c r="I409" t="n">
-        <v>52.62</v>
+        <v>78.843</v>
       </c>
       <c r="J409" t="n">
-        <v>4.5</v>
+        <v>3.4</v>
       </c>
       <c r="K409" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="L409" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>em andamento</t>
+          <t>concluído</t>
         </is>
       </c>
       <c r="N409" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-14 ao PV-15; arquivo: planos_furo/cts_joao_canzi_fl07_pv14_pv15.pdf; taxa 0,0095.</t>
+          <t>Plano de furo FL-02 versao 01, 26.MAI.2026; PV-03 ao PV-04; arquivo: planos_furo/CT LOURDES - FL.02.PLANO DE FURO_PV-03 AO PV-04.pdf; taxa 0,0195.</t>
         </is>
       </c>
       <c r="O409" t="n">
-        <v>-23.5306805</v>
+        <v>-23.5299216</v>
       </c>
       <c r="P409" t="n">
-        <v>-46.38564</v>
+        <v>-46.3936017</v>
       </c>
       <c r="Q409" t="n">
-        <v>-23.5304128</v>
+        <v>-23.5301962</v>
       </c>
       <c r="R409" t="n">
-        <v>-46.3852142</v>
+        <v>-46.3928893</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>cts_lourdes_complementar</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>JC-009</t>
+          <t>LOUR-004</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>PV-15 - PV-16</t>
+          <t>PV-04 - PV-05</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>PV-15</t>
+          <t>PV-04</t>
         </is>
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>PV-16</t>
+          <t>PV-05</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
@@ -47780,7 +47780,7 @@
         </is>
       </c>
       <c r="G410" t="n">
-        <v>355</v>
+        <v>450</v>
       </c>
       <c r="H410" t="inlineStr">
         <is>
@@ -47788,38 +47788,38 @@
         </is>
       </c>
       <c r="I410" t="n">
-        <v>85.03</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="J410" t="n">
+        <v>5</v>
+      </c>
+      <c r="K410" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L410" t="n">
         <v>5.5</v>
       </c>
-      <c r="K410" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="L410" t="n">
-        <v>5.9</v>
-      </c>
       <c r="M410" t="inlineStr">
         <is>
-          <t>em andamento</t>
+          <t>concluído</t>
         </is>
       </c>
       <c r="N410" t="inlineStr">
         <is>
-          <t>Plano de furo FL-01 versao 01, 26.MAI.2026; PV-15 ao PV-16; arquivo: planos_furo/cts_joao_canzi_fl01_pv15_pv16.pdf; taxa 0,0125.</t>
+          <t>Plano de furo FL-02 versao 01, 26.MAI.2026; PV-04 ao PV-05; arquivo: planos_furo/CT LOURDES - FL.02.PLANO DE FURO_PV-04 AO PV-05.pdf; taxa 0,0142.</t>
         </is>
       </c>
       <c r="O410" t="n">
-        <v>-23.5304128</v>
+        <v>-23.5301962</v>
       </c>
       <c r="P410" t="n">
-        <v>-46.3852142</v>
+        <v>-46.3928893</v>
       </c>
       <c r="Q410" t="n">
-        <v>-23.5299843</v>
+        <v>-23.530465</v>
       </c>
       <c r="R410" t="n">
-        <v>-46.3845231</v>
+        <v>-46.3923061</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige base do mapa Joao Canzi PV16 PV18
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1227,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L394"/>
+  <dimension ref="A1:L396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -19036,6 +19036,102 @@
       <c r="L394" t="inlineStr">
         <is>
           <t>Plano de furo FL-08 versao 01, 26.MAI.2026; trecho PV-15 ao PV-16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>JC-PV-17-FL07</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>PV-17</t>
+        </is>
+      </c>
+      <c r="E395" t="n">
+        <v>7397122.275</v>
+      </c>
+      <c r="F395" t="n">
+        <v>358726.884</v>
+      </c>
+      <c r="G395" t="n">
+        <v>-23.5300354</v>
+      </c>
+      <c r="H395" t="n">
+        <v>-46.3838931</v>
+      </c>
+      <c r="I395" t="n">
+        <v>782.299</v>
+      </c>
+      <c r="J395" t="n">
+        <v>779.199</v>
+      </c>
+      <c r="K395" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; trechos PV-16 ao PV-17 e PV-17 ao PV-18.</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>JC-PV-18</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>PV-18</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>7397124.485</v>
+      </c>
+      <c r="F396" t="n">
+        <v>358806.429</v>
+      </c>
+      <c r="G396" t="n">
+        <v>-23.5300223</v>
+      </c>
+      <c r="H396" t="n">
+        <v>-46.3831139</v>
+      </c>
+      <c r="I396" t="n">
+        <v>783.619</v>
+      </c>
+      <c r="J396" t="n">
+        <v>780.119</v>
+      </c>
+      <c r="K396" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; trecho PV-17 ao PV-18.</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R412"/>
+  <dimension ref="A1:R414"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -48064,6 +48160,154 @@
       </c>
       <c r="R412" t="n">
         <v>-46.3852142</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>JC-010</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>PV-16 - PV-17</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>PV-16</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>PV-17</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G413" t="n">
+        <v>355</v>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I413" t="n">
+        <v>64.572</v>
+      </c>
+      <c r="J413" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K413" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="L413" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N413" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; PV-16 ao PV-17; arquivo: planos_furo/cts_joao_canzi_fl07_pv16_pv17.pdf; taxa 0,0707.</t>
+        </is>
+      </c>
+      <c r="O413" t="n">
+        <v>-23.5299843</v>
+      </c>
+      <c r="P413" t="n">
+        <v>-46.3845231</v>
+      </c>
+      <c r="Q413" t="n">
+        <v>-23.5300354</v>
+      </c>
+      <c r="R413" t="n">
+        <v>-46.3838931</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>JC-011</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>PV-17 - PV-18</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>PV-17</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>PV-18</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G414" t="n">
+        <v>355</v>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I414" t="n">
+        <v>79.57599999999999</v>
+      </c>
+      <c r="J414" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K414" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L414" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N414" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; PV-17 ao PV-18; arquivo: planos_furo/cts_joao_canzi_fl07_pv17_pv18.pdf; taxa 0,0116.</t>
+        </is>
+      </c>
+      <c r="O414" t="n">
+        <v>-23.5300354</v>
+      </c>
+      <c r="P414" t="n">
+        <v>-46.3838931</v>
+      </c>
+      <c r="Q414" t="n">
+        <v>-23.5300223</v>
+      </c>
+      <c r="R414" t="n">
+        <v>-46.3831139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige trecho Elvira e curva de producao
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -18970,7 +18970,7 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elias_sleiman</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
@@ -18980,237 +18980,237 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>JC-PV-01</t>
+          <t>ELIAS-PV-21</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>PV-01</t>
+          <t>PV-21</t>
         </is>
       </c>
       <c r="E395" t="n">
-        <v>7396903.634</v>
+        <v>7397111.065</v>
       </c>
       <c r="F395" t="n">
-        <v>358332.744</v>
+        <v>358747.317</v>
       </c>
       <c r="G395" t="n">
-        <v>-23.5319754</v>
+        <v>-23.5301384</v>
       </c>
       <c r="H395" t="n">
-        <v>-46.3877739</v>
+        <v>-46.3836941</v>
       </c>
       <c r="I395" t="n">
-        <v>767.2910000000001</v>
+        <v>784.299</v>
       </c>
       <c r="J395" t="n">
-        <v>763.0069999999999</v>
+        <v>782.215</v>
       </c>
       <c r="K395" t="n">
-        <v>4.28</v>
+        <v>2.08</v>
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elvira de Araujo; complemento em VCA.</t>
+          <t>Adicionado via print do projeto RCE Elias Sleiman; lancamento completo em VCA.</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elias_sleiman</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>JC-PI-1.1</t>
+          <t>ELIAS-PV-22</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>PI-1.1</t>
+          <t>PV-22</t>
         </is>
       </c>
       <c r="E396" t="n">
-        <v>7396905.886</v>
+        <v>7397048.086</v>
       </c>
       <c r="F396" t="n">
-        <v>358329.956</v>
+        <v>358777.873</v>
       </c>
       <c r="G396" t="n">
-        <v>-23.5319548</v>
+        <v>-23.5307098</v>
       </c>
       <c r="H396" t="n">
-        <v>-46.387801</v>
+        <v>-46.3834008</v>
       </c>
       <c r="I396" t="n">
-        <v>767.159</v>
+        <v>794.057</v>
       </c>
       <c r="J396" t="n">
-        <v>765.927</v>
+        <v>791.972</v>
       </c>
       <c r="K396" t="n">
-        <v>1.23</v>
+        <v>2.08</v>
       </c>
       <c r="L396" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elvira de Araujo; complemento em VCA.</t>
+          <t>Adicionado via print do projeto RCE Elias Sleiman; lancamento completo em VCA.</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elias_sleiman</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>JC-PI-1.2</t>
+          <t>ELIAS-PV-23</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>PI-1.2</t>
+          <t>PV-23</t>
         </is>
       </c>
       <c r="E397" t="n">
-        <v>7396922.192</v>
+        <v>7397018.372</v>
       </c>
       <c r="F397" t="n">
-        <v>358327.004</v>
+        <v>358792.29</v>
       </c>
       <c r="G397" t="n">
-        <v>-23.5318073</v>
+        <v>-23.5309793</v>
       </c>
       <c r="H397" t="n">
-        <v>-46.3878284</v>
+        <v>-46.3832624</v>
       </c>
       <c r="I397" t="n">
-        <v>767.21</v>
+        <v>796.528</v>
       </c>
       <c r="J397" t="n">
-        <v>766.01</v>
+        <v>792.947</v>
       </c>
       <c r="K397" t="n">
-        <v>1.2</v>
+        <v>3.58</v>
       </c>
       <c r="L397" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elvira de Araujo; complemento em VCA.</t>
+          <t>Adicionado via print do projeto RCE Elias Sleiman; lancamento completo em VCA.</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>rce_elias_sleiman</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>ELIAS-PV-21</t>
+          <t>ELVIRA-PI-1.1</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>PV-21</t>
+          <t>PI-1.1</t>
         </is>
       </c>
       <c r="E398" t="n">
-        <v>7397111.065</v>
+        <v>7396905.886</v>
       </c>
       <c r="F398" t="n">
-        <v>358747.317</v>
+        <v>358329.956</v>
       </c>
       <c r="G398" t="n">
-        <v>-23.5301384</v>
+        <v>-23.5319548</v>
       </c>
       <c r="H398" t="n">
-        <v>-46.3836941</v>
+        <v>-46.387801</v>
       </c>
       <c r="I398" t="n">
-        <v>784.299</v>
+        <v>767.159</v>
       </c>
       <c r="J398" t="n">
-        <v>782.215</v>
+        <v>765.927</v>
       </c>
       <c r="K398" t="n">
-        <v>2.08</v>
+        <v>1.23</v>
       </c>
       <c r="L398" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elias Sleiman; lancamento completo em VCA.</t>
+          <t>Adicionado conforme solicitação: PI da RCE Elvira de Araujo; interligacao com CTS Joao Canzi mantida sem alterar registros existentes.</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>rce_elias_sleiman</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>PV</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>ELIAS-PV-22</t>
+          <t>ELVIRA-PI-1.2</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>PV-22</t>
+          <t>PI-1.2</t>
         </is>
       </c>
       <c r="E399" t="n">
-        <v>7397048.086</v>
+        <v>7396922.192</v>
       </c>
       <c r="F399" t="n">
-        <v>358777.873</v>
+        <v>358327.004</v>
       </c>
       <c r="G399" t="n">
-        <v>-23.5307098</v>
+        <v>-23.5318073</v>
       </c>
       <c r="H399" t="n">
-        <v>-46.3834008</v>
+        <v>-46.3878284</v>
       </c>
       <c r="I399" t="n">
-        <v>794.057</v>
+        <v>767.21</v>
       </c>
       <c r="J399" t="n">
-        <v>791.972</v>
+        <v>766.01</v>
       </c>
       <c r="K399" t="n">
-        <v>2.08</v>
+        <v>1.2</v>
       </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elias Sleiman; lancamento completo em VCA.</t>
+          <t>Adicionado conforme solicitação: PI da RCE Elvira de Araujo; interligacao com CTS Joao Canzi mantida sem alterar registros existentes.</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>rce_elias_sleiman</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -19220,141 +19220,141 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>ELIAS-PV-23</t>
+          <t>JC-PV-18</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>PV-23</t>
+          <t>PV-18</t>
         </is>
       </c>
       <c r="E400" t="n">
-        <v>7397018.372</v>
+        <v>7397124.485</v>
       </c>
       <c r="F400" t="n">
-        <v>358792.29</v>
+        <v>358806.429</v>
       </c>
       <c r="G400" t="n">
-        <v>-23.5309793</v>
+        <v>-23.5300224</v>
       </c>
       <c r="H400" t="n">
-        <v>-46.3832624</v>
+        <v>-46.3831139</v>
       </c>
       <c r="I400" t="n">
-        <v>796.528</v>
+        <v>783.619</v>
       </c>
       <c r="J400" t="n">
-        <v>792.947</v>
+        <v>780.119</v>
       </c>
       <c r="K400" t="n">
-        <v>3.58</v>
+        <v>3.5</v>
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elias Sleiman; lancamento completo em VCA.</t>
+          <t>Plano de furo FL-07 versao 01, 05.JUN.2026; trecho PV-18 ao PV-19.</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>rce_elvira_de_araujo</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>ELVIRA-PI-1.1</t>
+          <t>JC-PV-19</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>PI-1.1</t>
+          <t>PV-19</t>
         </is>
       </c>
       <c r="E401" t="n">
-        <v>7396905.886</v>
+        <v>7397141.155</v>
       </c>
       <c r="F401" t="n">
-        <v>358329.956</v>
+        <v>358871.038</v>
       </c>
       <c r="G401" t="n">
-        <v>-23.5319548</v>
+        <v>-23.5298774</v>
       </c>
       <c r="H401" t="n">
-        <v>-46.387801</v>
+        <v>-46.3824796</v>
       </c>
       <c r="I401" t="n">
-        <v>767.159</v>
+        <v>787.357</v>
       </c>
       <c r="J401" t="n">
-        <v>765.927</v>
+        <v>783.357</v>
       </c>
       <c r="K401" t="n">
-        <v>1.23</v>
+        <v>4</v>
       </c>
       <c r="L401" t="inlineStr">
         <is>
-          <t>Adicionado conforme solicitação: PI da RCE Elvira de Araujo; interligacao com CTS Joao Canzi mantida sem alterar registros existentes.</t>
+          <t>Plano de furo FL-07 versao 01, 05.JUN.2026; trecho PV-18 ao PV-19.</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>rce_elvira_de_araujo</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PV</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>ELVIRA-PI-1.2</t>
+          <t>JC-PV-17-FL07</t>
         </is>
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>PI-1.2</t>
+          <t>PV-17</t>
         </is>
       </c>
       <c r="E402" t="n">
-        <v>7396922.192</v>
+        <v>7397122.275</v>
       </c>
       <c r="F402" t="n">
-        <v>358327.004</v>
+        <v>358726.884</v>
       </c>
       <c r="G402" t="n">
-        <v>-23.5318073</v>
+        <v>-23.5300354</v>
       </c>
       <c r="H402" t="n">
-        <v>-46.3878284</v>
+        <v>-46.3838931</v>
       </c>
       <c r="I402" t="n">
-        <v>767.21</v>
+        <v>782.299</v>
       </c>
       <c r="J402" t="n">
-        <v>766.01</v>
+        <v>779.199</v>
       </c>
       <c r="K402" t="n">
-        <v>1.2</v>
+        <v>3.1</v>
       </c>
       <c r="L402" t="inlineStr">
         <is>
-          <t>Adicionado conforme solicitação: PI da RCE Elvira de Araujo; interligacao com CTS Joao Canzi mantida sem alterar registros existentes.</t>
+          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; trechos PV-16 ao PV-17 e PV-17 ao PV-18.</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
@@ -19364,45 +19364,45 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>JC-PV-18</t>
+          <t>ELVIRA-PV-08</t>
         </is>
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>PV-18</t>
+          <t>PV-08</t>
         </is>
       </c>
       <c r="E403" t="n">
-        <v>7397124.485</v>
+        <v>7396899.021</v>
       </c>
       <c r="F403" t="n">
-        <v>358806.429</v>
+        <v>358332.965</v>
       </c>
       <c r="G403" t="n">
-        <v>-23.5300224</v>
+        <v>-23.532017</v>
       </c>
       <c r="H403" t="n">
-        <v>-46.3831139</v>
+        <v>-46.3877722</v>
       </c>
       <c r="I403" t="n">
-        <v>783.619</v>
+        <v>767.145</v>
       </c>
       <c r="J403" t="n">
-        <v>780.119</v>
+        <v>762.845</v>
       </c>
       <c r="K403" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 05.JUN.2026; trecho PV-18 ao PV-19.</t>
+          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
@@ -19412,45 +19412,45 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>JC-PV-19</t>
+          <t>ELVIRA-PV-02</t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>PV-19</t>
+          <t>PV-02</t>
         </is>
       </c>
       <c r="E404" t="n">
-        <v>7397141.155</v>
+        <v>7396941.756</v>
       </c>
       <c r="F404" t="n">
-        <v>358871.038</v>
+        <v>358324.032</v>
       </c>
       <c r="G404" t="n">
-        <v>-23.5298774</v>
+        <v>-23.5316304</v>
       </c>
       <c r="H404" t="n">
-        <v>-46.3824796</v>
+        <v>-46.3878556</v>
       </c>
       <c r="I404" t="n">
-        <v>787.357</v>
+        <v>767.318</v>
       </c>
       <c r="J404" t="n">
-        <v>783.357</v>
+        <v>763.468</v>
       </c>
       <c r="K404" t="n">
-        <v>4</v>
+        <v>3.85</v>
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 05.JUN.2026; trecho PV-18 ao PV-19.</t>
+          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
@@ -19460,38 +19460,38 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>JC-PV-17-FL07</t>
+          <t>ELVIRA-PV-01</t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>PV-17</t>
+          <t>PV-01</t>
         </is>
       </c>
       <c r="E405" t="n">
-        <v>7397122.275</v>
+        <v>7396903.634</v>
       </c>
       <c r="F405" t="n">
-        <v>358726.884</v>
+        <v>358332.744</v>
       </c>
       <c r="G405" t="n">
-        <v>-23.5300354</v>
+        <v>-23.5319754</v>
       </c>
       <c r="H405" t="n">
-        <v>-46.3838931</v>
+        <v>-46.3877739</v>
       </c>
       <c r="I405" t="n">
-        <v>782.299</v>
+        <v>767.2910000000001</v>
       </c>
       <c r="J405" t="n">
-        <v>779.199</v>
+        <v>763.0069999999999</v>
       </c>
       <c r="K405" t="n">
-        <v>3.1</v>
+        <v>4.28</v>
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; trechos PV-16 ao PV-17 e PV-17 ao PV-18.</t>
+          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
         </is>
       </c>
     </row>
@@ -47933,12 +47933,12 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>JC-005</t>
+          <t>ELVIRA-001</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -47988,7 +47988,7 @@
       </c>
       <c r="N405" t="inlineStr">
         <is>
-          <t>Plano de furo FL-06 versao 01, 15.MAI.2026; RUA ELVIRA DE ARAUJO; taxa 0,0108.</t>
+          <t>Plano de furo FL-06 versao 01, 15.MAI.2026; PV-08 ao PV-02; RUA ELVIRA DE ARAUJO; arquivo: planos_furo/rce_elvira_fl06_pv08_pv02.pdf; taxa 0,0108. Movido do CTS Joao Canzi para RCE Elvira de Araujo em 09.JUN.2026.</t>
         </is>
       </c>
       <c r="O405" t="n">
@@ -48525,12 +48525,12 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>JC-010</t>
+          <t>ELVIRA-002</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -48580,7 +48580,7 @@
       </c>
       <c r="N413" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elvira de Araujo; complemento em VCA.</t>
+          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
         </is>
       </c>
       <c r="O413" t="n">
@@ -48599,12 +48599,12 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>JC-011</t>
+          <t>ELVIRA-003</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -48654,7 +48654,7 @@
       </c>
       <c r="N414" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elvira de Araujo; complemento em VCA.</t>
+          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
         </is>
       </c>
       <c r="O414" t="n">
@@ -48673,12 +48673,12 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>JC-012</t>
+          <t>ELVIRA-004</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -48728,7 +48728,7 @@
       </c>
       <c r="N415" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elvira de Araujo; complemento em VCA.</t>
+          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
         </is>
       </c>
       <c r="O415" t="n">

</xml_diff>

<commit_message>
Adiciona plano Joao Canzi PV10 PV11
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OBRAS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PONTOS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRECHOS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESUMO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACAO" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACAO_SHAPE" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACAO_SHAPE_0505" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACAO_SHAPE_LUIS_0505" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDACAO_SUBST_AGUA_BOA_0505" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="OBRAS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PONTOS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="TRECHOS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="RESUMO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="VALIDACAO" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="VALIDACAO_SHAPE" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="VALIDACAO_SHAPE_0505" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="VALIDACAO_SHAPE_LUIS_0505" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="VALIDACAO_SUBST_AGUA_BOA_0505" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TRECHOS'!$A$1:$R$445</definedName>
@@ -21171,7 +21171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R452"/>
+  <dimension ref="A1:R453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -53094,6 +53094,80 @@
       </c>
       <c r="R452" t="n">
         <v>-46.3831139</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>JC-005</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>PV-10 - PV-11</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>PV-10</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>PV-11</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G453" t="n">
+        <v>355</v>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I453" t="n">
+        <v>62.673</v>
+      </c>
+      <c r="J453" t="n">
+        <v>3</v>
+      </c>
+      <c r="K453" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="L453" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N453" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-05; PV-10 ao PV-11; arquivo: planos_furo/cts_joao_canzi_fl05_pv10_pv11.pdf.</t>
+        </is>
+      </c>
+      <c r="O453" t="n">
+        <v>-23.5317269</v>
+      </c>
+      <c r="P453" t="n">
+        <v>-46.3867492</v>
+      </c>
+      <c r="Q453" t="n">
+        <v>-23.5315615</v>
+      </c>
+      <c r="R453" t="n">
+        <v>-46.3861622</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restaura trecho PV-10 PV-11 Joao Canzi
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -21219,7 +21219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R453"/>
+  <dimension ref="A1:R454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -49725,22 +49725,22 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>JC-006</t>
+          <t>JC-005</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>PV-11 - PV-13</t>
+          <t>PV-10 - PV-11</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
+          <t>PV-10</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
           <t>PV-11</t>
-        </is>
-      </c>
-      <c r="E406" t="inlineStr">
-        <is>
-          <t>PV-13</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
@@ -49757,13 +49757,13 @@
         </is>
       </c>
       <c r="I406" t="n">
-        <v>62.701</v>
+        <v>62.673</v>
       </c>
       <c r="J406" t="n">
+        <v>3</v>
+      </c>
+      <c r="K406" t="n">
         <v>6.1</v>
-      </c>
-      <c r="K406" t="n">
-        <v>2</v>
       </c>
       <c r="L406" t="n">
         <v>6.1</v>
@@ -49775,20 +49775,20 @@
       </c>
       <c r="N406" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-11 ao PV-13; arquivo: planos_furo/cts_joao_canzi_fl07_pv11_pv13.pdf.</t>
+          <t>Plano de furo FL-05; PV-10 ao PV-11; arquivo: planos_furo/cts_joao_canzi_fl05_pv10_pv11.pdf.</t>
         </is>
       </c>
       <c r="O406" t="n">
+        <v>-23.5317269</v>
+      </c>
+      <c r="P406" t="n">
+        <v>-46.3867492</v>
+      </c>
+      <c r="Q406" t="n">
         <v>-23.5315615</v>
       </c>
-      <c r="P406" t="n">
+      <c r="R406" t="n">
         <v>-46.3861622</v>
-      </c>
-      <c r="Q406" t="n">
-        <v>-23.5310181</v>
-      </c>
-      <c r="R406" t="n">
-        <v>-46.3863345</v>
       </c>
     </row>
     <row r="407" hidden="1">
@@ -49799,22 +49799,22 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>JC-007</t>
+          <t>JC-006</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>PV-13 - PV-14</t>
+          <t>PV-11 - PV-13</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
+          <t>PV-11</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
           <t>PV-13</t>
-        </is>
-      </c>
-      <c r="E407" t="inlineStr">
-        <is>
-          <t>PV-14</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
@@ -49831,16 +49831,16 @@
         </is>
       </c>
       <c r="I407" t="n">
-        <v>80.157</v>
+        <v>62.701</v>
       </c>
       <c r="J407" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="K407" t="n">
         <v>2</v>
       </c>
-      <c r="K407" t="n">
-        <v>4.5</v>
-      </c>
       <c r="L407" t="n">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
       <c r="M407" t="inlineStr">
         <is>
@@ -49849,46 +49849,46 @@
       </c>
       <c r="N407" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-13 ao PV-14; arquivo: planos_furo/cts_joao_canzi_fl07_pv13_pv14.pdf; taxa 0,0400.</t>
+          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-11 ao PV-13; arquivo: planos_furo/cts_joao_canzi_fl07_pv11_pv13.pdf.</t>
         </is>
       </c>
       <c r="O407" t="n">
+        <v>-23.5315615</v>
+      </c>
+      <c r="P407" t="n">
+        <v>-46.3861622</v>
+      </c>
+      <c r="Q407" t="n">
         <v>-23.5310181</v>
       </c>
-      <c r="P407" t="n">
+      <c r="R407" t="n">
         <v>-46.3863345</v>
-      </c>
-      <c r="Q407" t="n">
-        <v>-23.5306805</v>
-      </c>
-      <c r="R407" t="n">
-        <v>-46.38564</v>
       </c>
     </row>
     <row r="408" hidden="1">
       <c r="A408" t="inlineStr">
         <is>
-          <t>cts_lourdes_complementar</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>LOUR-002</t>
+          <t>JC-007</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>PV-02 - PV-03</t>
+          <t>PV-13 - PV-14</t>
         </is>
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>PV-02</t>
+          <t>PV-13</t>
         </is>
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>PV-03</t>
+          <t>PV-14</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
@@ -49897,7 +49897,7 @@
         </is>
       </c>
       <c r="G408" t="n">
-        <v>450</v>
+        <v>355</v>
       </c>
       <c r="H408" t="inlineStr">
         <is>
@@ -49905,38 +49905,38 @@
         </is>
       </c>
       <c r="I408" t="n">
-        <v>78.58</v>
+        <v>80.157</v>
       </c>
       <c r="J408" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K408" t="n">
-        <v>3.4</v>
+        <v>4.5</v>
       </c>
       <c r="L408" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="M408" t="inlineStr">
         <is>
-          <t>concluído</t>
+          <t>em andamento</t>
         </is>
       </c>
       <c r="N408" t="inlineStr">
         <is>
-          <t>Plano de furo FL-02 versao 01, 14.MAI.2026; RUA GONCALVES CASTELAO; PV-02 ao PV-03; arquivo: planos_furo/CT LOURDES - FL.02.PLANO DE FURO_PV-02 AO PV-03.pdf; taxa 0,0109.</t>
+          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-13 ao PV-14; arquivo: planos_furo/cts_joao_canzi_fl07_pv13_pv14.pdf; taxa 0,0400.</t>
         </is>
       </c>
       <c r="O408" t="n">
-        <v>-23.52953</v>
+        <v>-23.5310181</v>
       </c>
       <c r="P408" t="n">
-        <v>-46.3942436</v>
+        <v>-46.3863345</v>
       </c>
       <c r="Q408" t="n">
-        <v>-23.5299216</v>
+        <v>-23.5306805</v>
       </c>
       <c r="R408" t="n">
-        <v>-46.3936017</v>
+        <v>-46.38564</v>
       </c>
     </row>
     <row r="409" hidden="1">
@@ -49947,22 +49947,22 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>LOUR-003</t>
+          <t>LOUR-002</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>PV-03 - PV-04</t>
+          <t>PV-02 - PV-03</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
+          <t>PV-02</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
           <t>PV-03</t>
-        </is>
-      </c>
-      <c r="E409" t="inlineStr">
-        <is>
-          <t>PV-04</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
@@ -49979,16 +49979,16 @@
         </is>
       </c>
       <c r="I409" t="n">
-        <v>78.843</v>
+        <v>78.58</v>
       </c>
       <c r="J409" t="n">
+        <v>4</v>
+      </c>
+      <c r="K409" t="n">
         <v>3.4</v>
       </c>
-      <c r="K409" t="n">
-        <v>5</v>
-      </c>
       <c r="L409" t="n">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="M409" t="inlineStr">
         <is>
@@ -49997,20 +49997,20 @@
       </c>
       <c r="N409" t="inlineStr">
         <is>
-          <t>Plano de furo FL-02 versao 01, 26.MAI.2026; PV-03 ao PV-04; arquivo: planos_furo/CT LOURDES - FL.02.PLANO DE FURO_PV-03 AO PV-04.pdf; taxa 0,0195.</t>
+          <t>Plano de furo FL-02 versao 01, 14.MAI.2026; RUA GONCALVES CASTELAO; PV-02 ao PV-03; arquivo: planos_furo/CT LOURDES - FL.02.PLANO DE FURO_PV-02 AO PV-03.pdf; taxa 0,0109.</t>
         </is>
       </c>
       <c r="O409" t="n">
+        <v>-23.52953</v>
+      </c>
+      <c r="P409" t="n">
+        <v>-46.3942436</v>
+      </c>
+      <c r="Q409" t="n">
         <v>-23.5299216</v>
       </c>
-      <c r="P409" t="n">
+      <c r="R409" t="n">
         <v>-46.3936017</v>
-      </c>
-      <c r="Q409" t="n">
-        <v>-23.5301962</v>
-      </c>
-      <c r="R409" t="n">
-        <v>-46.3928893</v>
       </c>
     </row>
     <row r="410" hidden="1">
@@ -50021,22 +50021,22 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>LOUR-004</t>
+          <t>LOUR-003</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>PV-04 - PV-05</t>
+          <t>PV-03 - PV-04</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
         <is>
+          <t>PV-03</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
           <t>PV-04</t>
-        </is>
-      </c>
-      <c r="E410" t="inlineStr">
-        <is>
-          <t>PV-05</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
@@ -50053,16 +50053,16 @@
         </is>
       </c>
       <c r="I410" t="n">
-        <v>66.56999999999999</v>
+        <v>78.843</v>
       </c>
       <c r="J410" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K410" t="n">
         <v>5</v>
       </c>
-      <c r="K410" t="n">
-        <v>2.2</v>
-      </c>
       <c r="L410" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="M410" t="inlineStr">
         <is>
@@ -50071,46 +50071,46 @@
       </c>
       <c r="N410" t="inlineStr">
         <is>
-          <t>Plano de furo FL-02 versao 01, 26.MAI.2026; PV-04 ao PV-05; arquivo: planos_furo/CT LOURDES - FL.02.PLANO DE FURO_PV-04 AO PV-05.pdf; taxa 0,0142.</t>
+          <t>Plano de furo FL-02 versao 01, 26.MAI.2026; PV-03 ao PV-04; arquivo: planos_furo/CT LOURDES - FL.02.PLANO DE FURO_PV-03 AO PV-04.pdf; taxa 0,0195.</t>
         </is>
       </c>
       <c r="O410" t="n">
+        <v>-23.5299216</v>
+      </c>
+      <c r="P410" t="n">
+        <v>-46.3936017</v>
+      </c>
+      <c r="Q410" t="n">
         <v>-23.5301962</v>
       </c>
-      <c r="P410" t="n">
+      <c r="R410" t="n">
         <v>-46.3928893</v>
-      </c>
-      <c r="Q410" t="n">
-        <v>-23.530465</v>
-      </c>
-      <c r="R410" t="n">
-        <v>-46.3923061</v>
       </c>
     </row>
     <row r="411" hidden="1">
       <c r="A411" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>cts_lourdes_complementar</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>JC-008</t>
+          <t>LOUR-004</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>PV-15 - PV-16</t>
+          <t>PV-04 - PV-05</t>
         </is>
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>PV-15</t>
+          <t>PV-04</t>
         </is>
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>PV-16</t>
+          <t>PV-05</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
@@ -50119,7 +50119,7 @@
         </is>
       </c>
       <c r="G411" t="n">
-        <v>355</v>
+        <v>450</v>
       </c>
       <c r="H411" t="inlineStr">
         <is>
@@ -50127,38 +50127,38 @@
         </is>
       </c>
       <c r="I411" t="n">
-        <v>85.03</v>
+        <v>66.56999999999999</v>
       </c>
       <c r="J411" t="n">
+        <v>5</v>
+      </c>
+      <c r="K411" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L411" t="n">
         <v>5.5</v>
       </c>
-      <c r="K411" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="L411" t="n">
-        <v>5.9</v>
-      </c>
       <c r="M411" t="inlineStr">
         <is>
-          <t>em andamento</t>
+          <t>concluído</t>
         </is>
       </c>
       <c r="N411" t="inlineStr">
         <is>
-          <t>Plano de furo FL-08 versao 01, 26.MAI.2026; PV-15 ao PV-16; arquivo: planos_furo/cts_joao_canzi_fl08_pv15_pv16.pdf; taxa 0,0125.</t>
+          <t>Plano de furo FL-02 versao 01, 26.MAI.2026; PV-04 ao PV-05; arquivo: planos_furo/CT LOURDES - FL.02.PLANO DE FURO_PV-04 AO PV-05.pdf; taxa 0,0142.</t>
         </is>
       </c>
       <c r="O411" t="n">
-        <v>-23.5304128</v>
+        <v>-23.5301962</v>
       </c>
       <c r="P411" t="n">
-        <v>-46.3852142</v>
+        <v>-46.3928893</v>
       </c>
       <c r="Q411" t="n">
-        <v>-23.5299843</v>
+        <v>-23.530465</v>
       </c>
       <c r="R411" t="n">
-        <v>-46.3845231</v>
+        <v>-46.3923061</v>
       </c>
     </row>
     <row r="412" hidden="1">
@@ -50169,22 +50169,22 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>JC-009</t>
+          <t>JC-008</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>PV-14 - PV-15</t>
+          <t>PV-15 - PV-16</t>
         </is>
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>PV-14</t>
+          <t>PV-15</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t>PV-15</t>
+          <t>PV-16</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
@@ -50201,16 +50201,16 @@
         </is>
       </c>
       <c r="I412" t="n">
-        <v>52.62</v>
+        <v>85.03</v>
       </c>
       <c r="J412" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="K412" t="n">
-        <v>5.5</v>
+        <v>3.1</v>
       </c>
       <c r="L412" t="n">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="M412" t="inlineStr">
         <is>
@@ -50219,72 +50219,72 @@
       </c>
       <c r="N412" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-14 ao PV-15; arquivo: planos_furo/cts_joao_canzi_fl07_pv14_pv15.pdf; taxa 0,0095.</t>
+          <t>Plano de furo FL-08 versao 01, 26.MAI.2026; PV-15 ao PV-16; arquivo: planos_furo/cts_joao_canzi_fl08_pv15_pv16.pdf; taxa 0,0125.</t>
         </is>
       </c>
       <c r="O412" t="n">
-        <v>-23.5306805</v>
+        <v>-23.5304128</v>
       </c>
       <c r="P412" t="n">
-        <v>-46.38564</v>
+        <v>-46.3852142</v>
       </c>
       <c r="Q412" t="n">
-        <v>-23.5304128</v>
+        <v>-23.5299843</v>
       </c>
       <c r="R412" t="n">
-        <v>-46.3852142</v>
+        <v>-46.3845231</v>
       </c>
     </row>
     <row r="413" hidden="1">
       <c r="A413" t="inlineStr">
         <is>
-          <t>rce_elvira_de_araujo</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>ELVIRA-002</t>
+          <t>JC-009</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>PV-01 - PI-1.1</t>
+          <t>PV-14 - PV-15</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>PV-01</t>
+          <t>PV-14</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>PI-1.1</t>
+          <t>PV-15</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>PVC</t>
+          <t>PEAD LISO</t>
         </is>
       </c>
       <c r="G413" t="n">
-        <v>200</v>
+        <v>355</v>
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>Vala a Céu Aberto - VCA</t>
+          <t>Metodo Nao Destrutivo - MND</t>
         </is>
       </c>
       <c r="I413" t="n">
-        <v>3.58</v>
+        <v>52.62</v>
       </c>
       <c r="J413" t="n">
-        <v>4.28</v>
+        <v>4.5</v>
       </c>
       <c r="K413" t="n">
-        <v>1.23</v>
+        <v>5.5</v>
       </c>
       <c r="L413" t="n">
-        <v>4.28</v>
+        <v>5.5</v>
       </c>
       <c r="M413" t="inlineStr">
         <is>
@@ -50293,20 +50293,20 @@
       </c>
       <c r="N413" t="inlineStr">
         <is>
-          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
+          <t>Plano de furo FL-07 versao 01, 20.MAI.2026; PV-14 ao PV-15; arquivo: planos_furo/cts_joao_canzi_fl07_pv14_pv15.pdf; taxa 0,0095.</t>
         </is>
       </c>
       <c r="O413" t="n">
-        <v>-23.5319754</v>
+        <v>-23.5306805</v>
       </c>
       <c r="P413" t="n">
-        <v>-46.3877739</v>
+        <v>-46.38564</v>
       </c>
       <c r="Q413" t="n">
-        <v>-23.5319548</v>
+        <v>-23.5304128</v>
       </c>
       <c r="R413" t="n">
-        <v>-46.387801</v>
+        <v>-46.3852142</v>
       </c>
     </row>
     <row r="414" hidden="1">
@@ -50317,22 +50317,22 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>ELVIRA-003</t>
+          <t>ELVIRA-002</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>PI-1.1 - PI-1.2</t>
+          <t>PV-01 - PI-1.1</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
         <is>
+          <t>PV-01</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
           <t>PI-1.1</t>
-        </is>
-      </c>
-      <c r="E414" t="inlineStr">
-        <is>
-          <t>PI-1.2</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
@@ -50349,16 +50349,16 @@
         </is>
       </c>
       <c r="I414" t="n">
-        <v>16.62</v>
+        <v>3.58</v>
       </c>
       <c r="J414" t="n">
+        <v>4.28</v>
+      </c>
+      <c r="K414" t="n">
         <v>1.23</v>
       </c>
-      <c r="K414" t="n">
-        <v>1.2</v>
-      </c>
       <c r="L414" t="n">
-        <v>1.23</v>
+        <v>4.28</v>
       </c>
       <c r="M414" t="inlineStr">
         <is>
@@ -50371,16 +50371,16 @@
         </is>
       </c>
       <c r="O414" t="n">
+        <v>-23.5319754</v>
+      </c>
+      <c r="P414" t="n">
+        <v>-46.3877739</v>
+      </c>
+      <c r="Q414" t="n">
         <v>-23.5319548</v>
       </c>
-      <c r="P414" t="n">
+      <c r="R414" t="n">
         <v>-46.387801</v>
-      </c>
-      <c r="Q414" t="n">
-        <v>-23.5318073</v>
-      </c>
-      <c r="R414" t="n">
-        <v>-46.3878284</v>
       </c>
     </row>
     <row r="415" hidden="1">
@@ -50391,22 +50391,22 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>ELVIRA-004</t>
+          <t>ELVIRA-003</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>PI-1.2 - PV-02</t>
+          <t>PI-1.1 - PI-1.2</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
         <is>
+          <t>PI-1.1</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
           <t>PI-1.2</t>
-        </is>
-      </c>
-      <c r="E415" t="inlineStr">
-        <is>
-          <t>PV-02</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
@@ -50423,16 +50423,16 @@
         </is>
       </c>
       <c r="I415" t="n">
-        <v>5</v>
+        <v>16.62</v>
       </c>
       <c r="J415" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="K415" t="n">
         <v>1.2</v>
       </c>
-      <c r="K415" t="n">
-        <v>4.01</v>
-      </c>
       <c r="L415" t="n">
-        <v>4.01</v>
+        <v>1.23</v>
       </c>
       <c r="M415" t="inlineStr">
         <is>
@@ -50445,42 +50445,42 @@
         </is>
       </c>
       <c r="O415" t="n">
+        <v>-23.5319548</v>
+      </c>
+      <c r="P415" t="n">
+        <v>-46.387801</v>
+      </c>
+      <c r="Q415" t="n">
         <v>-23.5318073</v>
       </c>
-      <c r="P415" t="n">
+      <c r="R415" t="n">
         <v>-46.3878284</v>
-      </c>
-      <c r="Q415" t="n">
-        <v>-23.5317625</v>
-      </c>
-      <c r="R415" t="n">
-        <v>-46.3878221</v>
       </c>
     </row>
     <row r="416" hidden="1">
       <c r="A416" t="inlineStr">
         <is>
-          <t>rce_elias_sleiman</t>
+          <t>rce_elvira_de_araujo</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>ELIAS-001</t>
+          <t>ELVIRA-004</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>PV-21 - PV-22</t>
+          <t>PI-1.2 - PV-02</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>PV-21</t>
+          <t>PI-1.2</t>
         </is>
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>PV-22</t>
+          <t>PV-02</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
@@ -50497,16 +50497,16 @@
         </is>
       </c>
       <c r="I416" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="J416" t="n">
-        <v>2.08</v>
+        <v>1.2</v>
       </c>
       <c r="K416" t="n">
-        <v>2.08</v>
+        <v>4.01</v>
       </c>
       <c r="L416" t="n">
-        <v>2.08</v>
+        <v>4.01</v>
       </c>
       <c r="M416" t="inlineStr">
         <is>
@@ -50515,20 +50515,20 @@
       </c>
       <c r="N416" t="inlineStr">
         <is>
-          <t>Adicionado via print do projeto RCE Elias Sleiman; lancamento completo em VCA.</t>
+          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
         </is>
       </c>
       <c r="O416" t="n">
-        <v>-23.5301384</v>
+        <v>-23.5318073</v>
       </c>
       <c r="P416" t="n">
-        <v>-46.3836941</v>
+        <v>-46.3878284</v>
       </c>
       <c r="Q416" t="n">
-        <v>-23.5307098</v>
+        <v>-23.5317625</v>
       </c>
       <c r="R416" t="n">
-        <v>-46.3834008</v>
+        <v>-46.3878221</v>
       </c>
     </row>
     <row r="417" hidden="1">
@@ -50539,22 +50539,22 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>ELIAS-002</t>
+          <t>ELIAS-001</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>PV-22 - PV-23</t>
+          <t>PV-21 - PV-22</t>
         </is>
       </c>
       <c r="D417" t="inlineStr">
         <is>
+          <t>PV-21</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
           <t>PV-22</t>
-        </is>
-      </c>
-      <c r="E417" t="inlineStr">
-        <is>
-          <t>PV-23</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
@@ -50571,16 +50571,16 @@
         </is>
       </c>
       <c r="I417" t="n">
-        <v>33.03</v>
+        <v>70</v>
       </c>
       <c r="J417" t="n">
         <v>2.08</v>
       </c>
       <c r="K417" t="n">
-        <v>3.58</v>
+        <v>2.08</v>
       </c>
       <c r="L417" t="n">
-        <v>3.58</v>
+        <v>2.08</v>
       </c>
       <c r="M417" t="inlineStr">
         <is>
@@ -50593,68 +50593,68 @@
         </is>
       </c>
       <c r="O417" t="n">
+        <v>-23.5301384</v>
+      </c>
+      <c r="P417" t="n">
+        <v>-46.3836941</v>
+      </c>
+      <c r="Q417" t="n">
         <v>-23.5307098</v>
       </c>
-      <c r="P417" t="n">
+      <c r="R417" t="n">
         <v>-46.3834008</v>
-      </c>
-      <c r="Q417" t="n">
-        <v>-23.5309793</v>
-      </c>
-      <c r="R417" t="n">
-        <v>-46.3832624</v>
       </c>
     </row>
     <row r="418" hidden="1">
       <c r="A418" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_elias_sleiman</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>JC-013</t>
+          <t>ELIAS-002</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>PV-18 - PV-19</t>
+          <t>PV-22 - PV-23</t>
         </is>
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>PV-18</t>
+          <t>PV-22</t>
         </is>
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>PV-19</t>
+          <t>PV-23</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>PEAD LISO</t>
+          <t>PVC</t>
         </is>
       </c>
       <c r="G418" t="n">
-        <v>355</v>
+        <v>200</v>
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>Metodo Nao Destrutivo - MND</t>
+          <t>Vala a Céu Aberto - VCA</t>
         </is>
       </c>
       <c r="I418" t="n">
-        <v>66.72499999999999</v>
+        <v>33.03</v>
       </c>
       <c r="J418" t="n">
-        <v>3.5</v>
+        <v>2.08</v>
       </c>
       <c r="K418" t="n">
-        <v>4</v>
+        <v>3.58</v>
       </c>
       <c r="L418" t="n">
-        <v>4</v>
+        <v>3.58</v>
       </c>
       <c r="M418" t="inlineStr">
         <is>
@@ -50663,72 +50663,72 @@
       </c>
       <c r="N418" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 05.JUN.2026; PV-18 ao PV-19; arquivo: planos_furo/cts_joao_canzi_fl07_pv18_pv19.pdf; taxa 0,0485.</t>
+          <t>Adicionado via print do projeto RCE Elias Sleiman; lancamento completo em VCA.</t>
         </is>
       </c>
       <c r="O418" t="n">
-        <v>-23.5300224</v>
+        <v>-23.5307098</v>
       </c>
       <c r="P418" t="n">
-        <v>-46.3831139</v>
+        <v>-46.3834008</v>
       </c>
       <c r="Q418" t="n">
-        <v>-23.5298774</v>
+        <v>-23.5309793</v>
       </c>
       <c r="R418" t="n">
-        <v>-46.3824796</v>
+        <v>-46.3832624</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>rce_comunidade_sao_lucas</t>
+          <t>cts_joao_canzi</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>SL-001</t>
+          <t>JC-013</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>PV-26 - PV-27</t>
+          <t>PV-18 - PV-19</t>
         </is>
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>PV-26</t>
+          <t>PV-18</t>
         </is>
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>PV-27</t>
+          <t>PV-19</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>PVC</t>
+          <t>PEAD LISO</t>
         </is>
       </c>
       <c r="G419" t="n">
-        <v>200</v>
+        <v>355</v>
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>Vala a Céu Aberto - VCA</t>
+          <t>Metodo Nao Destrutivo - MND</t>
         </is>
       </c>
       <c r="I419" t="n">
-        <v>14.74</v>
+        <v>66.72499999999999</v>
       </c>
       <c r="J419" t="n">
-        <v>3.04</v>
+        <v>3.5</v>
       </c>
       <c r="K419" t="n">
-        <v>3.57</v>
+        <v>4</v>
       </c>
       <c r="L419" t="n">
-        <v>3.57</v>
+        <v>4</v>
       </c>
       <c r="M419" t="inlineStr">
         <is>
@@ -50737,20 +50737,20 @@
       </c>
       <c r="N419" t="inlineStr">
         <is>
-          <t>Adicionado via prints do projeto RCE Comunidade Sao Lucas; trecho em VCA; extensao calculada pela distancia entre coordenadas UTM.</t>
+          <t>Plano de furo FL-07 versao 01, 05.JUN.2026; PV-18 ao PV-19; arquivo: planos_furo/cts_joao_canzi_fl07_pv18_pv19.pdf; taxa 0,0485.</t>
         </is>
       </c>
       <c r="O419" t="n">
-        <v>-23.5236471</v>
+        <v>-23.5300224</v>
       </c>
       <c r="P419" t="n">
-        <v>-46.3767998</v>
+        <v>-46.3831139</v>
       </c>
       <c r="Q419" t="n">
-        <v>-23.5237798</v>
+        <v>-23.5298774</v>
       </c>
       <c r="R419" t="n">
-        <v>-46.3767878</v>
+        <v>-46.3824796</v>
       </c>
     </row>
     <row r="420">
@@ -50761,22 +50761,22 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>SL-002</t>
+          <t>SL-001</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>PV-27 - PV-28</t>
+          <t>PV-26 - PV-27</t>
         </is>
       </c>
       <c r="D420" t="inlineStr">
         <is>
+          <t>PV-26</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
           <t>PV-27</t>
-        </is>
-      </c>
-      <c r="E420" t="inlineStr">
-        <is>
-          <t>PV-28</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
@@ -50793,13 +50793,13 @@
         </is>
       </c>
       <c r="I420" t="n">
-        <v>3.63</v>
+        <v>14.74</v>
       </c>
       <c r="J420" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="K420" t="n">
         <v>3.57</v>
-      </c>
-      <c r="K420" t="n">
-        <v>3.34</v>
       </c>
       <c r="L420" t="n">
         <v>3.57</v>
@@ -50815,16 +50815,16 @@
         </is>
       </c>
       <c r="O420" t="n">
+        <v>-23.5236471</v>
+      </c>
+      <c r="P420" t="n">
+        <v>-46.3767998</v>
+      </c>
+      <c r="Q420" t="n">
         <v>-23.5237798</v>
       </c>
-      <c r="P420" t="n">
+      <c r="R420" t="n">
         <v>-46.3767878</v>
-      </c>
-      <c r="Q420" t="n">
-        <v>-23.5238121</v>
-      </c>
-      <c r="R420" t="n">
-        <v>-46.3767936</v>
       </c>
     </row>
     <row r="421">
@@ -50835,22 +50835,22 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>SL-003</t>
+          <t>SL-002</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>PV-28 - PV-29</t>
+          <t>PV-27 - PV-28</t>
         </is>
       </c>
       <c r="D421" t="inlineStr">
         <is>
+          <t>PV-27</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
           <t>PV-28</t>
-        </is>
-      </c>
-      <c r="E421" t="inlineStr">
-        <is>
-          <t>PV-29</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
@@ -50867,16 +50867,16 @@
         </is>
       </c>
       <c r="I421" t="n">
-        <v>7.51</v>
+        <v>3.63</v>
       </c>
       <c r="J421" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="K421" t="n">
         <v>3.34</v>
       </c>
-      <c r="K421" t="n">
-        <v>1.81</v>
-      </c>
       <c r="L421" t="n">
-        <v>3.34</v>
+        <v>3.57</v>
       </c>
       <c r="M421" t="inlineStr">
         <is>
@@ -50889,16 +50889,16 @@
         </is>
       </c>
       <c r="O421" t="n">
+        <v>-23.5237798</v>
+      </c>
+      <c r="P421" t="n">
+        <v>-46.3767878</v>
+      </c>
+      <c r="Q421" t="n">
         <v>-23.5238121</v>
       </c>
-      <c r="P421" t="n">
+      <c r="R421" t="n">
         <v>-46.3767936</v>
-      </c>
-      <c r="Q421" t="n">
-        <v>-23.5238331</v>
-      </c>
-      <c r="R421" t="n">
-        <v>-46.3768636</v>
       </c>
     </row>
     <row r="422">
@@ -50909,22 +50909,22 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>SL-004</t>
+          <t>SL-003</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>PV-29 - PV-30</t>
+          <t>PV-28 - PV-29</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
+          <t>PV-28</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
           <t>PV-29</t>
-        </is>
-      </c>
-      <c r="E422" t="inlineStr">
-        <is>
-          <t>PV-30</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
@@ -50941,16 +50941,16 @@
         </is>
       </c>
       <c r="I422" t="n">
-        <v>13.61</v>
+        <v>7.51</v>
       </c>
       <c r="J422" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="K422" t="n">
         <v>1.81</v>
       </c>
-      <c r="K422" t="n">
-        <v>1.4</v>
-      </c>
       <c r="L422" t="n">
-        <v>1.81</v>
+        <v>3.34</v>
       </c>
       <c r="M422" t="inlineStr">
         <is>
@@ -50963,16 +50963,16 @@
         </is>
       </c>
       <c r="O422" t="n">
+        <v>-23.5238121</v>
+      </c>
+      <c r="P422" t="n">
+        <v>-46.3767936</v>
+      </c>
+      <c r="Q422" t="n">
         <v>-23.5238331</v>
       </c>
-      <c r="P422" t="n">
+      <c r="R422" t="n">
         <v>-46.3768636</v>
-      </c>
-      <c r="Q422" t="n">
-        <v>-23.5237849</v>
-      </c>
-      <c r="R422" t="n">
-        <v>-46.3769862</v>
       </c>
     </row>
     <row r="423">
@@ -50983,22 +50983,22 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>SL-005</t>
+          <t>SL-004</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>PV-30 - PV-31</t>
+          <t>PV-29 - PV-30</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
+          <t>PV-29</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
           <t>PV-30</t>
-        </is>
-      </c>
-      <c r="E423" t="inlineStr">
-        <is>
-          <t>PV-31</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
@@ -51015,16 +51015,16 @@
         </is>
       </c>
       <c r="I423" t="n">
-        <v>6.62</v>
+        <v>13.61</v>
       </c>
       <c r="J423" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="K423" t="n">
         <v>1.4</v>
       </c>
-      <c r="K423" t="n">
-        <v>1.43</v>
-      </c>
       <c r="L423" t="n">
-        <v>1.43</v>
+        <v>1.81</v>
       </c>
       <c r="M423" t="inlineStr">
         <is>
@@ -51037,16 +51037,16 @@
         </is>
       </c>
       <c r="O423" t="n">
+        <v>-23.5238331</v>
+      </c>
+      <c r="P423" t="n">
+        <v>-46.3768636</v>
+      </c>
+      <c r="Q423" t="n">
         <v>-23.5237849</v>
       </c>
-      <c r="P423" t="n">
+      <c r="R423" t="n">
         <v>-46.3769862</v>
-      </c>
-      <c r="Q423" t="n">
-        <v>-23.5237689</v>
-      </c>
-      <c r="R423" t="n">
-        <v>-46.3770487</v>
       </c>
     </row>
     <row r="424">
@@ -51057,22 +51057,22 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>SL-006</t>
+          <t>SL-005</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>PV-31 - PV-32</t>
+          <t>PV-30 - PV-31</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
+          <t>PV-30</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
           <t>PV-31</t>
-        </is>
-      </c>
-      <c r="E424" t="inlineStr">
-        <is>
-          <t>PV-32</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
@@ -51089,16 +51089,16 @@
         </is>
       </c>
       <c r="I424" t="n">
-        <v>70.89</v>
+        <v>6.62</v>
       </c>
       <c r="J424" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K424" t="n">
         <v>1.43</v>
       </c>
-      <c r="K424" t="n">
-        <v>2.18</v>
-      </c>
       <c r="L424" t="n">
-        <v>2.18</v>
+        <v>1.43</v>
       </c>
       <c r="M424" t="inlineStr">
         <is>
@@ -51111,16 +51111,16 @@
         </is>
       </c>
       <c r="O424" t="n">
+        <v>-23.5237849</v>
+      </c>
+      <c r="P424" t="n">
+        <v>-46.3769862</v>
+      </c>
+      <c r="Q424" t="n">
         <v>-23.5237689</v>
       </c>
-      <c r="P424" t="n">
+      <c r="R424" t="n">
         <v>-46.3770487</v>
-      </c>
-      <c r="Q424" t="n">
-        <v>-23.5233519</v>
-      </c>
-      <c r="R424" t="n">
-        <v>-46.3775754</v>
       </c>
     </row>
     <row r="425">
@@ -51131,22 +51131,22 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>SL-007</t>
+          <t>SL-006</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>PV-32 - PV-33</t>
+          <t>PV-31 - PV-32</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
+          <t>PV-31</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
           <t>PV-32</t>
-        </is>
-      </c>
-      <c r="E425" t="inlineStr">
-        <is>
-          <t>PV-33</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
@@ -51163,13 +51163,13 @@
         </is>
       </c>
       <c r="I425" t="n">
-        <v>62.56</v>
+        <v>70.89</v>
       </c>
       <c r="J425" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="K425" t="n">
         <v>2.18</v>
-      </c>
-      <c r="K425" t="n">
-        <v>2.16</v>
       </c>
       <c r="L425" t="n">
         <v>2.18</v>
@@ -51185,16 +51185,16 @@
         </is>
       </c>
       <c r="O425" t="n">
+        <v>-23.5237689</v>
+      </c>
+      <c r="P425" t="n">
+        <v>-46.3770487</v>
+      </c>
+      <c r="Q425" t="n">
         <v>-23.5233519</v>
       </c>
-      <c r="P425" t="n">
+      <c r="R425" t="n">
         <v>-46.3775754</v>
-      </c>
-      <c r="Q425" t="n">
-        <v>-23.5230626</v>
-      </c>
-      <c r="R425" t="n">
-        <v>-46.3781017</v>
       </c>
     </row>
     <row r="426">
@@ -51205,22 +51205,22 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>SL-008</t>
+          <t>SL-007</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>PV-33 - PV-34</t>
+          <t>PV-32 - PV-33</t>
         </is>
       </c>
       <c r="D426" t="inlineStr">
         <is>
+          <t>PV-32</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
           <t>PV-33</t>
-        </is>
-      </c>
-      <c r="E426" t="inlineStr">
-        <is>
-          <t>PV-34</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
@@ -51237,16 +51237,16 @@
         </is>
       </c>
       <c r="I426" t="n">
-        <v>55.46</v>
+        <v>62.56</v>
       </c>
       <c r="J426" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="K426" t="n">
         <v>2.16</v>
       </c>
-      <c r="K426" t="n">
-        <v>2.45</v>
-      </c>
       <c r="L426" t="n">
-        <v>2.45</v>
+        <v>2.18</v>
       </c>
       <c r="M426" t="inlineStr">
         <is>
@@ -51259,16 +51259,16 @@
         </is>
       </c>
       <c r="O426" t="n">
+        <v>-23.5233519</v>
+      </c>
+      <c r="P426" t="n">
+        <v>-46.3775754</v>
+      </c>
+      <c r="Q426" t="n">
         <v>-23.5230626</v>
       </c>
-      <c r="P426" t="n">
+      <c r="R426" t="n">
         <v>-46.3781017</v>
-      </c>
-      <c r="Q426" t="n">
-        <v>-23.5226874</v>
-      </c>
-      <c r="R426" t="n">
-        <v>-46.3784614</v>
       </c>
     </row>
     <row r="427">
@@ -51279,22 +51279,22 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>SL-009</t>
+          <t>SL-008</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>PV-34 - PV-35</t>
+          <t>PV-33 - PV-34</t>
         </is>
       </c>
       <c r="D427" t="inlineStr">
         <is>
+          <t>PV-33</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
           <t>PV-34</t>
-        </is>
-      </c>
-      <c r="E427" t="inlineStr">
-        <is>
-          <t>PV-35</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
@@ -51311,16 +51311,16 @@
         </is>
       </c>
       <c r="I427" t="n">
-        <v>57.62</v>
+        <v>55.46</v>
       </c>
       <c r="J427" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="K427" t="n">
         <v>2.45</v>
       </c>
-      <c r="K427" t="n">
-        <v>3.88</v>
-      </c>
       <c r="L427" t="n">
-        <v>3.88</v>
+        <v>2.45</v>
       </c>
       <c r="M427" t="inlineStr">
         <is>
@@ -51333,16 +51333,16 @@
         </is>
       </c>
       <c r="O427" t="n">
+        <v>-23.5230626</v>
+      </c>
+      <c r="P427" t="n">
+        <v>-46.3781017</v>
+      </c>
+      <c r="Q427" t="n">
         <v>-23.5226874</v>
       </c>
-      <c r="P427" t="n">
+      <c r="R427" t="n">
         <v>-46.3784614</v>
-      </c>
-      <c r="Q427" t="n">
-        <v>-23.5223561</v>
-      </c>
-      <c r="R427" t="n">
-        <v>-46.3788967</v>
       </c>
     </row>
     <row r="428">
@@ -51353,22 +51353,22 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>SL-010</t>
+          <t>SL-009</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>PV-35 - PV-36</t>
+          <t>PV-34 - PV-35</t>
         </is>
       </c>
       <c r="D428" t="inlineStr">
         <is>
+          <t>PV-34</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
           <t>PV-35</t>
-        </is>
-      </c>
-      <c r="E428" t="inlineStr">
-        <is>
-          <t>PV-36</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
@@ -51385,16 +51385,16 @@
         </is>
       </c>
       <c r="I428" t="n">
-        <v>27.35</v>
+        <v>57.62</v>
       </c>
       <c r="J428" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="K428" t="n">
         <v>3.88</v>
       </c>
-      <c r="K428" t="n">
-        <v>3.97</v>
-      </c>
       <c r="L428" t="n">
-        <v>3.97</v>
+        <v>3.88</v>
       </c>
       <c r="M428" t="inlineStr">
         <is>
@@ -51407,16 +51407,16 @@
         </is>
       </c>
       <c r="O428" t="n">
+        <v>-23.5226874</v>
+      </c>
+      <c r="P428" t="n">
+        <v>-46.3784614</v>
+      </c>
+      <c r="Q428" t="n">
         <v>-23.5223561</v>
       </c>
-      <c r="P428" t="n">
+      <c r="R428" t="n">
         <v>-46.3788967</v>
-      </c>
-      <c r="Q428" t="n">
-        <v>-23.5221552</v>
-      </c>
-      <c r="R428" t="n">
-        <v>-46.3790525</v>
       </c>
     </row>
     <row r="429">
@@ -51427,22 +51427,22 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>SL-011</t>
+          <t>SL-010</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>PV-36 - PV-37</t>
+          <t>PV-35 - PV-36</t>
         </is>
       </c>
       <c r="D429" t="inlineStr">
         <is>
+          <t>PV-35</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
           <t>PV-36</t>
-        </is>
-      </c>
-      <c r="E429" t="inlineStr">
-        <is>
-          <t>PV-37</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
@@ -51459,13 +51459,13 @@
         </is>
       </c>
       <c r="I429" t="n">
-        <v>10.49</v>
+        <v>27.35</v>
       </c>
       <c r="J429" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="K429" t="n">
         <v>3.97</v>
-      </c>
-      <c r="K429" t="n">
-        <v>3.75</v>
       </c>
       <c r="L429" t="n">
         <v>3.97</v>
@@ -51481,16 +51481,16 @@
         </is>
       </c>
       <c r="O429" t="n">
+        <v>-23.5223561</v>
+      </c>
+      <c r="P429" t="n">
+        <v>-46.3788967</v>
+      </c>
+      <c r="Q429" t="n">
         <v>-23.5221552</v>
       </c>
-      <c r="P429" t="n">
+      <c r="R429" t="n">
         <v>-46.3790525</v>
-      </c>
-      <c r="Q429" t="n">
-        <v>-23.5220801</v>
-      </c>
-      <c r="R429" t="n">
-        <v>-46.379115</v>
       </c>
     </row>
     <row r="430">
@@ -51501,22 +51501,22 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>SL-012</t>
+          <t>SL-011</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>PV-37 - PV-38</t>
+          <t>PV-36 - PV-37</t>
         </is>
       </c>
       <c r="D430" t="inlineStr">
         <is>
+          <t>PV-36</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
           <t>PV-37</t>
-        </is>
-      </c>
-      <c r="E430" t="inlineStr">
-        <is>
-          <t>PV-38</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
@@ -51529,20 +51529,20 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>Vala a Ceu Aberto - VCA</t>
+          <t>Vala a Céu Aberto - VCA</t>
         </is>
       </c>
       <c r="I430" t="n">
-        <v>16.89</v>
+        <v>10.49</v>
       </c>
       <c r="J430" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="K430" t="n">
         <v>3.75</v>
       </c>
-      <c r="K430" t="n">
-        <v>3.92</v>
-      </c>
       <c r="L430" t="n">
-        <v>3.92</v>
+        <v>3.97</v>
       </c>
       <c r="M430" t="inlineStr">
         <is>
@@ -51551,20 +51551,20 @@
       </c>
       <c r="N430" t="inlineStr">
         <is>
-          <t>Adicionado via prints do projeto RCE Comunidade Sao Lucas; trecho em VCA. PV-38 incluido conforme novo print.</t>
+          <t>Adicionado via prints do projeto RCE Comunidade Sao Lucas; trecho em VCA; extensao calculada pela distancia entre coordenadas UTM.</t>
         </is>
       </c>
       <c r="O430" t="n">
+        <v>-23.5221552</v>
+      </c>
+      <c r="P430" t="n">
+        <v>-46.3790525</v>
+      </c>
+      <c r="Q430" t="n">
         <v>-23.5220801</v>
       </c>
-      <c r="P430" t="n">
+      <c r="R430" t="n">
         <v>-46.379115</v>
-      </c>
-      <c r="Q430" t="n">
-        <v>-23.5220422</v>
-      </c>
-      <c r="R430" t="n">
-        <v>-46.3789548</v>
       </c>
     </row>
     <row r="431">
@@ -51575,22 +51575,22 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>SL-013</t>
+          <t>SL-012</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>PV-38 - PV-39</t>
+          <t>PV-37 - PV-38</t>
         </is>
       </c>
       <c r="D431" t="inlineStr">
         <is>
+          <t>PV-37</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
           <t>PV-38</t>
-        </is>
-      </c>
-      <c r="E431" t="inlineStr">
-        <is>
-          <t>PV-39</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
@@ -51607,13 +51607,13 @@
         </is>
       </c>
       <c r="I431" t="n">
-        <v>46.47</v>
+        <v>16.89</v>
       </c>
       <c r="J431" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="K431" t="n">
         <v>3.92</v>
-      </c>
-      <c r="K431" t="n">
-        <v>3.64</v>
       </c>
       <c r="L431" t="n">
         <v>3.92</v>
@@ -51629,16 +51629,16 @@
         </is>
       </c>
       <c r="O431" t="n">
+        <v>-23.5220801</v>
+      </c>
+      <c r="P431" t="n">
+        <v>-46.379115</v>
+      </c>
+      <c r="Q431" t="n">
         <v>-23.5220422</v>
       </c>
-      <c r="P431" t="n">
+      <c r="R431" t="n">
         <v>-46.3789548</v>
-      </c>
-      <c r="Q431" t="n">
-        <v>-23.5222906</v>
-      </c>
-      <c r="R431" t="n">
-        <v>-46.378588</v>
       </c>
     </row>
     <row r="432">
@@ -51649,22 +51649,22 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>SL-014</t>
+          <t>SL-013</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>PV-40 - PV-41</t>
+          <t>PV-38 - PV-39</t>
         </is>
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>PV-40</t>
+          <t>PV-38</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>PV-41</t>
+          <t>PV-39</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
@@ -51677,20 +51677,20 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>Vala a Céu Aberto - VCA</t>
+          <t>Vala a Ceu Aberto - VCA</t>
         </is>
       </c>
       <c r="I432" t="n">
-        <v>48.64</v>
+        <v>46.47</v>
       </c>
       <c r="J432" t="n">
-        <v>4.31</v>
+        <v>3.92</v>
       </c>
       <c r="K432" t="n">
-        <v>2.58</v>
+        <v>3.64</v>
       </c>
       <c r="L432" t="n">
-        <v>4.31</v>
+        <v>3.92</v>
       </c>
       <c r="M432" t="inlineStr">
         <is>
@@ -51699,20 +51699,20 @@
       </c>
       <c r="N432" t="inlineStr">
         <is>
-          <t>Adicionado via prints do projeto RCE Comunidade Sao Lucas; trecho em VCA; extensao calculada pela distancia entre coordenadas UTM.</t>
+          <t>Adicionado via prints do projeto RCE Comunidade Sao Lucas; trecho em VCA. PV-38 incluido conforme novo print.</t>
         </is>
       </c>
       <c r="O432" t="n">
-        <v>-23.5224137</v>
+        <v>-23.5220422</v>
       </c>
       <c r="P432" t="n">
-        <v>-46.3783767</v>
+        <v>-46.3789548</v>
       </c>
       <c r="Q432" t="n">
-        <v>-23.5227141</v>
+        <v>-23.5222906</v>
       </c>
       <c r="R432" t="n">
-        <v>-46.378029</v>
+        <v>-46.378588</v>
       </c>
     </row>
     <row r="433">
@@ -51723,22 +51723,22 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>SL-015</t>
+          <t>SL-014</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>PV-41 - PV-42</t>
+          <t>PV-40 - PV-41</t>
         </is>
       </c>
       <c r="D433" t="inlineStr">
         <is>
+          <t>PV-40</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
           <t>PV-41</t>
-        </is>
-      </c>
-      <c r="E433" t="inlineStr">
-        <is>
-          <t>PV-42</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
@@ -51755,16 +51755,16 @@
         </is>
       </c>
       <c r="I433" t="n">
-        <v>38.45</v>
+        <v>48.64</v>
       </c>
       <c r="J433" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="K433" t="n">
         <v>2.58</v>
       </c>
-      <c r="K433" t="n">
-        <v>1.41</v>
-      </c>
       <c r="L433" t="n">
-        <v>2.58</v>
+        <v>4.31</v>
       </c>
       <c r="M433" t="inlineStr">
         <is>
@@ -51777,16 +51777,16 @@
         </is>
       </c>
       <c r="O433" t="n">
+        <v>-23.5224137</v>
+      </c>
+      <c r="P433" t="n">
+        <v>-46.3783767</v>
+      </c>
+      <c r="Q433" t="n">
         <v>-23.5227141</v>
       </c>
-      <c r="P433" t="n">
+      <c r="R433" t="n">
         <v>-46.378029</v>
-      </c>
-      <c r="Q433" t="n">
-        <v>-23.52298</v>
-      </c>
-      <c r="R433" t="n">
-        <v>-46.3777869</v>
       </c>
     </row>
     <row r="434">
@@ -51797,22 +51797,22 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>SL-016</t>
+          <t>SL-015</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>PV-39 - PV-40</t>
+          <t>PV-41 - PV-42</t>
         </is>
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>PV-39</t>
+          <t>PV-41</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>PV-40</t>
+          <t>PV-42</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
@@ -51825,20 +51825,20 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>Vala a Ceu Aberto - VCA</t>
+          <t>Vala a Céu Aberto - VCA</t>
         </is>
       </c>
       <c r="I434" t="n">
-        <v>24.53</v>
+        <v>38.45</v>
       </c>
       <c r="J434" t="n">
-        <v>3.64</v>
+        <v>2.58</v>
       </c>
       <c r="K434" t="n">
-        <v>4.31</v>
+        <v>1.41</v>
       </c>
       <c r="L434" t="n">
-        <v>4.31</v>
+        <v>2.58</v>
       </c>
       <c r="M434" t="inlineStr">
         <is>
@@ -51847,20 +51847,20 @@
       </c>
       <c r="N434" t="inlineStr">
         <is>
-          <t>Adicionado via prints do projeto RCE Comunidade Sao Lucas; trecho em VCA. Extensao lida no print.</t>
+          <t>Adicionado via prints do projeto RCE Comunidade Sao Lucas; trecho em VCA; extensao calculada pela distancia entre coordenadas UTM.</t>
         </is>
       </c>
       <c r="O434" t="n">
-        <v>-23.5222906</v>
+        <v>-23.5227141</v>
       </c>
       <c r="P434" t="n">
-        <v>-46.378588</v>
+        <v>-46.378029</v>
       </c>
       <c r="Q434" t="n">
-        <v>-23.5224137</v>
+        <v>-23.52298</v>
       </c>
       <c r="R434" t="n">
-        <v>-46.3783767</v>
+        <v>-46.3777869</v>
       </c>
     </row>
     <row r="435">
@@ -51871,22 +51871,22 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>SL-017</t>
+          <t>SL-016</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>PV-40 - PV-69</t>
+          <t>PV-39 - PV-40</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
         <is>
+          <t>PV-39</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
           <t>PV-40</t>
-        </is>
-      </c>
-      <c r="E435" t="inlineStr">
-        <is>
-          <t>PV-69</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
@@ -51903,13 +51903,13 @@
         </is>
       </c>
       <c r="I435" t="n">
-        <v>13.08</v>
+        <v>24.53</v>
       </c>
       <c r="J435" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="K435" t="n">
         <v>4.31</v>
-      </c>
-      <c r="K435" t="n">
-        <v>1.93</v>
       </c>
       <c r="L435" t="n">
         <v>4.31</v>
@@ -51925,16 +51925,16 @@
         </is>
       </c>
       <c r="O435" t="n">
+        <v>-23.5222906</v>
+      </c>
+      <c r="P435" t="n">
+        <v>-46.378588</v>
+      </c>
+      <c r="Q435" t="n">
         <v>-23.5224137</v>
       </c>
-      <c r="P435" t="n">
+      <c r="R435" t="n">
         <v>-46.3783767</v>
-      </c>
-      <c r="Q435" t="n">
-        <v>-23.5224631</v>
-      </c>
-      <c r="R435" t="n">
-        <v>-46.3782535</v>
       </c>
     </row>
     <row r="436">
@@ -51945,22 +51945,22 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>SL-018</t>
+          <t>SL-017</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>PV-69 - PV-70</t>
+          <t>PV-40 - PV-69</t>
         </is>
       </c>
       <c r="D436" t="inlineStr">
         <is>
+          <t>PV-40</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
           <t>PV-69</t>
-        </is>
-      </c>
-      <c r="E436" t="inlineStr">
-        <is>
-          <t>PV-70</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
@@ -51977,16 +51977,16 @@
         </is>
       </c>
       <c r="I436" t="n">
-        <v>20.55</v>
+        <v>13.08</v>
       </c>
       <c r="J436" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="K436" t="n">
         <v>1.93</v>
       </c>
-      <c r="K436" t="n">
-        <v>1.41</v>
-      </c>
       <c r="L436" t="n">
-        <v>1.93</v>
+        <v>4.31</v>
       </c>
       <c r="M436" t="inlineStr">
         <is>
@@ -51999,16 +51999,16 @@
         </is>
       </c>
       <c r="O436" t="n">
+        <v>-23.5224137</v>
+      </c>
+      <c r="P436" t="n">
+        <v>-46.3783767</v>
+      </c>
+      <c r="Q436" t="n">
         <v>-23.5224631</v>
       </c>
-      <c r="P436" t="n">
+      <c r="R436" t="n">
         <v>-46.3782535</v>
-      </c>
-      <c r="Q436" t="n">
-        <v>-23.5224276</v>
-      </c>
-      <c r="R436" t="n">
-        <v>-46.378053</v>
       </c>
     </row>
     <row r="437">
@@ -52019,22 +52019,22 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>SL-019</t>
+          <t>SL-018</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>PV-64 - PV-65</t>
+          <t>PV-69 - PV-70</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>PV-64</t>
+          <t>PV-69</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>PV-65</t>
+          <t>PV-70</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
@@ -52047,42 +52047,42 @@
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>VCA</t>
+          <t>Vala a Ceu Aberto - VCA</t>
         </is>
       </c>
       <c r="I437" t="n">
-        <v>39.5</v>
+        <v>20.55</v>
       </c>
       <c r="J437" t="n">
-        <v>2.84</v>
+        <v>1.93</v>
       </c>
       <c r="K437" t="n">
-        <v>1.6</v>
+        <v>1.41</v>
       </c>
       <c r="L437" t="n">
-        <v>2.84</v>
+        <v>1.93</v>
       </c>
       <c r="M437" t="inlineStr">
         <is>
-          <t>ATIVO</t>
+          <t>em andamento</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
         <is>
-          <t>Interligação corrigida PV-64 -&gt; PV-65 conforme projeto.</t>
+          <t>Adicionado via prints do projeto RCE Comunidade Sao Lucas; trecho em VCA. Extensao lida no print.</t>
         </is>
       </c>
       <c r="O437" t="n">
-        <v>-23.522</v>
+        <v>-23.5224631</v>
       </c>
       <c r="P437" t="n">
-        <v>-46.378</v>
+        <v>-46.3782535</v>
       </c>
       <c r="Q437" t="n">
-        <v>-23.5224</v>
+        <v>-23.5224276</v>
       </c>
       <c r="R437" t="n">
-        <v>-46.378</v>
+        <v>-46.378053</v>
       </c>
     </row>
     <row r="438">
@@ -52093,22 +52093,22 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>SL-020</t>
+          <t>SL-019</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>PV-65 - PV-70</t>
+          <t>PV-64 - PV-65</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
         <is>
+          <t>PV-64</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
           <t>PV-65</t>
-        </is>
-      </c>
-      <c r="E438" t="inlineStr">
-        <is>
-          <t>PV-70</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
@@ -52125,16 +52125,16 @@
         </is>
       </c>
       <c r="I438" t="n">
-        <v>2.88</v>
+        <v>39.5</v>
       </c>
       <c r="J438" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="K438" t="n">
         <v>1.6</v>
       </c>
-      <c r="K438" t="n">
-        <v>1.41</v>
-      </c>
       <c r="L438" t="n">
-        <v>1.6</v>
+        <v>2.84</v>
       </c>
       <c r="M438" t="inlineStr">
         <is>
@@ -52143,11 +52143,11 @@
       </c>
       <c r="N438" t="inlineStr">
         <is>
-          <t>Interligação corrigida PV-65 -&gt; PV-70 conforme projeto.</t>
+          <t>Interligação corrigida PV-64 -&gt; PV-65 conforme projeto.</t>
         </is>
       </c>
       <c r="O438" t="n">
-        <v>-23.5224</v>
+        <v>-23.522</v>
       </c>
       <c r="P438" t="n">
         <v>-46.378</v>
@@ -52167,22 +52167,22 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>SL-021</t>
+          <t>SL-020</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>PVE-32 - PV-02</t>
+          <t>PV-65 - PV-70</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>PVE-32</t>
+          <t>PV-65</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>PV-02</t>
+          <t>PV-70</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
@@ -52195,42 +52195,42 @@
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t>Vala a Ceu Aberto - VCA</t>
+          <t>VCA</t>
         </is>
       </c>
       <c r="I439" t="n">
-        <v>12.61</v>
+        <v>2.88</v>
       </c>
       <c r="J439" t="n">
-        <v>2.05</v>
+        <v>1.6</v>
       </c>
       <c r="K439" t="n">
-        <v>1.48</v>
+        <v>1.41</v>
       </c>
       <c r="L439" t="n">
-        <v>2.05</v>
+        <v>1.6</v>
       </c>
       <c r="M439" t="inlineStr">
         <is>
-          <t>em andamento</t>
+          <t>ATIVO</t>
         </is>
       </c>
       <c r="N439" t="inlineStr">
         <is>
-          <t>Corrigido conforme sequencia informada: PVE-32 -&gt; PV-02 -&gt; PV-03 -&gt; PV-04 -&gt; PV-05 -&gt; PV-06 -&gt; PV-07 -&gt; PV-08; trecho em VCA.</t>
+          <t>Interligação corrigida PV-65 -&gt; PV-70 conforme projeto.</t>
         </is>
       </c>
       <c r="O439" t="n">
-        <v>-23.5199037</v>
+        <v>-23.5224</v>
       </c>
       <c r="P439" t="n">
-        <v>-46.3771453</v>
+        <v>-46.378</v>
       </c>
       <c r="Q439" t="n">
-        <v>-23.5200098</v>
+        <v>-23.5224</v>
       </c>
       <c r="R439" t="n">
-        <v>-46.3771007</v>
+        <v>-46.378</v>
       </c>
     </row>
     <row r="440">
@@ -52241,22 +52241,22 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>SL-022</t>
+          <t>SL-021</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>PV-02 - PV-03</t>
+          <t>PVE-32 - PV-02</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
         <is>
+          <t>PVE-32</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
           <t>PV-02</t>
-        </is>
-      </c>
-      <c r="E440" t="inlineStr">
-        <is>
-          <t>PV-03</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
@@ -52273,16 +52273,16 @@
         </is>
       </c>
       <c r="I440" t="n">
-        <v>21</v>
+        <v>12.61</v>
       </c>
       <c r="J440" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="K440" t="n">
         <v>1.48</v>
       </c>
-      <c r="K440" t="n">
-        <v>2.04</v>
-      </c>
       <c r="L440" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="M440" t="inlineStr">
         <is>
@@ -52295,16 +52295,16 @@
         </is>
       </c>
       <c r="O440" t="n">
+        <v>-23.5199037</v>
+      </c>
+      <c r="P440" t="n">
+        <v>-46.3771453</v>
+      </c>
+      <c r="Q440" t="n">
         <v>-23.5200098</v>
       </c>
-      <c r="P440" t="n">
+      <c r="R440" t="n">
         <v>-46.3771007</v>
-      </c>
-      <c r="Q440" t="n">
-        <v>-23.5200681</v>
-      </c>
-      <c r="R440" t="n">
-        <v>-46.376905</v>
       </c>
     </row>
     <row r="441">
@@ -52315,22 +52315,22 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>SL-023</t>
+          <t>SL-022</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>PV-03 - PV-04</t>
+          <t>PV-02 - PV-03</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
+          <t>PV-02</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
           <t>PV-03</t>
-        </is>
-      </c>
-      <c r="E441" t="inlineStr">
-        <is>
-          <t>PV-04</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
@@ -52347,13 +52347,13 @@
         </is>
       </c>
       <c r="I441" t="n">
-        <v>46.15</v>
+        <v>21</v>
       </c>
       <c r="J441" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="K441" t="n">
         <v>2.04</v>
-      </c>
-      <c r="K441" t="n">
-        <v>1.68</v>
       </c>
       <c r="L441" t="n">
         <v>2.04</v>
@@ -52369,16 +52369,16 @@
         </is>
       </c>
       <c r="O441" t="n">
+        <v>-23.5200098</v>
+      </c>
+      <c r="P441" t="n">
+        <v>-46.3771007</v>
+      </c>
+      <c r="Q441" t="n">
         <v>-23.5200681</v>
       </c>
-      <c r="P441" t="n">
+      <c r="R441" t="n">
         <v>-46.376905</v>
-      </c>
-      <c r="Q441" t="n">
-        <v>-23.5204836</v>
-      </c>
-      <c r="R441" t="n">
-        <v>-46.3768696</v>
       </c>
     </row>
     <row r="442">
@@ -52389,22 +52389,22 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>SL-024</t>
+          <t>SL-023</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>PV-04 - PV-05</t>
+          <t>PV-03 - PV-04</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
+          <t>PV-03</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
           <t>PV-04</t>
-        </is>
-      </c>
-      <c r="E442" t="inlineStr">
-        <is>
-          <t>PV-05</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
@@ -52421,16 +52421,16 @@
         </is>
       </c>
       <c r="I442" t="n">
-        <v>38.98</v>
+        <v>46.15</v>
       </c>
       <c r="J442" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="K442" t="n">
         <v>1.68</v>
       </c>
-      <c r="K442" t="n">
-        <v>1.76</v>
-      </c>
       <c r="L442" t="n">
-        <v>1.76</v>
+        <v>2.04</v>
       </c>
       <c r="M442" t="inlineStr">
         <is>
@@ -52443,16 +52443,16 @@
         </is>
       </c>
       <c r="O442" t="n">
+        <v>-23.5200681</v>
+      </c>
+      <c r="P442" t="n">
+        <v>-46.376905</v>
+      </c>
+      <c r="Q442" t="n">
         <v>-23.5204836</v>
       </c>
-      <c r="P442" t="n">
+      <c r="R442" t="n">
         <v>-46.3768696</v>
-      </c>
-      <c r="Q442" t="n">
-        <v>-23.5208354</v>
-      </c>
-      <c r="R442" t="n">
-        <v>-46.3768848</v>
       </c>
     </row>
     <row r="443">
@@ -52463,22 +52463,22 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>SL-025</t>
+          <t>SL-024</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>PV-05 - PV-06</t>
+          <t>PV-04 - PV-05</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
+          <t>PV-04</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
           <t>PV-05</t>
-        </is>
-      </c>
-      <c r="E443" t="inlineStr">
-        <is>
-          <t>PV-06</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
@@ -52495,16 +52495,16 @@
         </is>
       </c>
       <c r="I443" t="n">
-        <v>37.7</v>
+        <v>38.98</v>
       </c>
       <c r="J443" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="K443" t="n">
         <v>1.76</v>
       </c>
-      <c r="K443" t="n">
-        <v>1.85</v>
-      </c>
       <c r="L443" t="n">
-        <v>1.85</v>
+        <v>1.76</v>
       </c>
       <c r="M443" t="inlineStr">
         <is>
@@ -52517,16 +52517,16 @@
         </is>
       </c>
       <c r="O443" t="n">
+        <v>-23.5204836</v>
+      </c>
+      <c r="P443" t="n">
+        <v>-46.3768696</v>
+      </c>
+      <c r="Q443" t="n">
         <v>-23.5208354</v>
       </c>
-      <c r="P443" t="n">
+      <c r="R443" t="n">
         <v>-46.3768848</v>
-      </c>
-      <c r="Q443" t="n">
-        <v>-23.5211749</v>
-      </c>
-      <c r="R443" t="n">
-        <v>-46.3768575</v>
       </c>
     </row>
     <row r="444">
@@ -52537,22 +52537,22 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>SL-026</t>
+          <t>SL-025</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>PV-06 - PV-07</t>
+          <t>PV-05 - PV-06</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
         <is>
+          <t>PV-05</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
           <t>PV-06</t>
-        </is>
-      </c>
-      <c r="E444" t="inlineStr">
-        <is>
-          <t>PV-07</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
@@ -52569,13 +52569,13 @@
         </is>
       </c>
       <c r="I444" t="n">
-        <v>34.53</v>
+        <v>37.7</v>
       </c>
       <c r="J444" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="K444" t="n">
         <v>1.85</v>
-      </c>
-      <c r="K444" t="n">
-        <v>1.44</v>
       </c>
       <c r="L444" t="n">
         <v>1.85</v>
@@ -52591,16 +52591,16 @@
         </is>
       </c>
       <c r="O444" t="n">
+        <v>-23.5208354</v>
+      </c>
+      <c r="P444" t="n">
+        <v>-46.3768848</v>
+      </c>
+      <c r="Q444" t="n">
         <v>-23.5211749</v>
       </c>
-      <c r="P444" t="n">
+      <c r="R444" t="n">
         <v>-46.3768575</v>
-      </c>
-      <c r="Q444" t="n">
-        <v>-23.5214649</v>
-      </c>
-      <c r="R444" t="n">
-        <v>-46.3767334</v>
       </c>
     </row>
     <row r="445">
@@ -52611,22 +52611,22 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>SL-027</t>
+          <t>SL-026</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>PV-07 - PV-08</t>
+          <t>PV-06 - PV-07</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
         <is>
+          <t>PV-06</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
           <t>PV-07</t>
-        </is>
-      </c>
-      <c r="E445" t="inlineStr">
-        <is>
-          <t>PV-08</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
@@ -52643,16 +52643,16 @@
         </is>
       </c>
       <c r="I445" t="n">
-        <v>8.17</v>
+        <v>34.53</v>
       </c>
       <c r="J445" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="K445" t="n">
         <v>1.44</v>
       </c>
-      <c r="K445" t="n">
-        <v>1.41</v>
-      </c>
       <c r="L445" t="n">
-        <v>1.44</v>
+        <v>1.85</v>
       </c>
       <c r="M445" t="inlineStr">
         <is>
@@ -52665,16 +52665,16 @@
         </is>
       </c>
       <c r="O445" t="n">
+        <v>-23.5211749</v>
+      </c>
+      <c r="P445" t="n">
+        <v>-46.3768575</v>
+      </c>
+      <c r="Q445" t="n">
         <v>-23.5214649</v>
       </c>
-      <c r="P445" t="n">
+      <c r="R445" t="n">
         <v>-46.3767334</v>
-      </c>
-      <c r="Q445" t="n">
-        <v>-23.5215374</v>
-      </c>
-      <c r="R445" t="n">
-        <v>-46.3767183</v>
       </c>
     </row>
     <row r="446">
@@ -52685,22 +52685,22 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>SL-028</t>
+          <t>SL-027</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>PVE-31 - PV-37</t>
+          <t>PV-07 - PV-08</t>
         </is>
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>PVE-31</t>
+          <t>PV-07</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>PV-37</t>
+          <t>PV-08</t>
         </is>
       </c>
       <c r="F446" t="inlineStr">
@@ -52717,16 +52717,16 @@
         </is>
       </c>
       <c r="I446" t="n">
-        <v>10.11</v>
+        <v>8.17</v>
       </c>
       <c r="J446" t="n">
-        <v>2.4</v>
+        <v>1.44</v>
       </c>
       <c r="K446" t="n">
-        <v>3.75</v>
+        <v>1.41</v>
       </c>
       <c r="L446" t="n">
-        <v>3.75</v>
+        <v>1.44</v>
       </c>
       <c r="M446" t="inlineStr">
         <is>
@@ -52735,8 +52735,20 @@
       </c>
       <c r="N446" t="inlineStr">
         <is>
-          <t>Interligacao adicionada conforme projeto.</t>
-        </is>
+          <t>Corrigido conforme sequencia informada: PVE-32 -&gt; PV-02 -&gt; PV-03 -&gt; PV-04 -&gt; PV-05 -&gt; PV-06 -&gt; PV-07 -&gt; PV-08; trecho em VCA.</t>
+        </is>
+      </c>
+      <c r="O446" t="n">
+        <v>-23.5214649</v>
+      </c>
+      <c r="P446" t="n">
+        <v>-46.3767334</v>
+      </c>
+      <c r="Q446" t="n">
+        <v>-23.5215374</v>
+      </c>
+      <c r="R446" t="n">
+        <v>-46.3767183</v>
       </c>
     </row>
     <row r="447">
@@ -52747,22 +52759,22 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>SL-029</t>
+          <t>SL-028</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>PV-75 - PV-76</t>
+          <t>PVE-31 - PV-37</t>
         </is>
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>PV-75</t>
+          <t>PVE-31</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>PV-76</t>
+          <t>PV-37</t>
         </is>
       </c>
       <c r="F447" t="inlineStr">
@@ -52779,16 +52791,16 @@
         </is>
       </c>
       <c r="I447" t="n">
-        <v>2.09</v>
+        <v>10.11</v>
       </c>
       <c r="J447" t="n">
-        <v>1.35</v>
+        <v>2.4</v>
       </c>
       <c r="K447" t="n">
-        <v>1.25</v>
+        <v>3.75</v>
       </c>
       <c r="L447" t="n">
-        <v>1.35</v>
+        <v>3.75</v>
       </c>
       <c r="M447" t="inlineStr">
         <is>
@@ -52797,7 +52809,7 @@
       </c>
       <c r="N447" t="inlineStr">
         <is>
-          <t>Interligação adicionada conforme projeto.</t>
+          <t>Interligacao adicionada conforme projeto.</t>
         </is>
       </c>
     </row>
@@ -52809,22 +52821,22 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>SL-030</t>
+          <t>SL-029</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>PV-76 - PV-77</t>
+          <t>PV-75 - PV-76</t>
         </is>
       </c>
       <c r="D448" t="inlineStr">
         <is>
+          <t>PV-75</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
           <t>PV-76</t>
-        </is>
-      </c>
-      <c r="E448" t="inlineStr">
-        <is>
-          <t>PV-77</t>
         </is>
       </c>
       <c r="F448" t="inlineStr">
@@ -52841,16 +52853,16 @@
         </is>
       </c>
       <c r="I448" t="n">
-        <v>18.02</v>
+        <v>2.09</v>
       </c>
       <c r="J448" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="K448" t="n">
         <v>1.25</v>
       </c>
-      <c r="K448" t="n">
-        <v>1.58</v>
-      </c>
       <c r="L448" t="n">
-        <v>1.58</v>
+        <v>1.35</v>
       </c>
       <c r="M448" t="inlineStr">
         <is>
@@ -52871,22 +52883,22 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>SL-031</t>
+          <t>SL-030</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>PV-77 - PV-78</t>
+          <t>PV-76 - PV-77</t>
         </is>
       </c>
       <c r="D449" t="inlineStr">
         <is>
+          <t>PV-76</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
           <t>PV-77</t>
-        </is>
-      </c>
-      <c r="E449" t="inlineStr">
-        <is>
-          <t>PV-78</t>
         </is>
       </c>
       <c r="F449" t="inlineStr">
@@ -52903,10 +52915,10 @@
         </is>
       </c>
       <c r="I449" t="n">
-        <v>21.33</v>
+        <v>18.02</v>
       </c>
       <c r="J449" t="n">
-        <v>1.58</v>
+        <v>1.25</v>
       </c>
       <c r="K449" t="n">
         <v>1.58</v>
@@ -52933,22 +52945,22 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>SL-032</t>
+          <t>SL-031</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>PV-75.1 - PV-75</t>
+          <t>PV-77 - PV-78</t>
         </is>
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>PV-75.1</t>
+          <t>PV-77</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>PV-75</t>
+          <t>PV-78</t>
         </is>
       </c>
       <c r="F450" t="inlineStr">
@@ -52965,13 +52977,16 @@
         </is>
       </c>
       <c r="I450" t="n">
-        <v>5</v>
+        <v>21.33</v>
+      </c>
+      <c r="J450" t="n">
+        <v>1.58</v>
       </c>
       <c r="K450" t="n">
-        <v>1.35</v>
+        <v>1.58</v>
       </c>
       <c r="L450" t="n">
-        <v>1.35</v>
+        <v>1.58</v>
       </c>
       <c r="M450" t="inlineStr">
         <is>
@@ -52980,72 +52995,57 @@
       </c>
       <c r="N450" t="inlineStr">
         <is>
-          <t>Interligacao PV-75.1 -&gt; PV-75 adicionada via Google Earth.</t>
-        </is>
-      </c>
-      <c r="O450" t="n">
-        <v>-23.5198222</v>
-      </c>
-      <c r="P450" t="n">
-        <v>-46.3768722</v>
-      </c>
-      <c r="Q450" t="n">
-        <v>-23.5198</v>
-      </c>
-      <c r="R450" t="n">
-        <v>-46.3763</v>
+          <t>Interligação adicionada conforme projeto.</t>
+        </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>cts_joao_canzi</t>
+          <t>rce_comunidade_sao_lucas</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>JC-014</t>
+          <t>SL-032</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>PV-16 - PV-17</t>
+          <t>PV-75.1 - PV-75</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>PV-16</t>
+          <t>PV-75.1</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>PV-17</t>
+          <t>PV-75</t>
         </is>
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>PEAD LISO</t>
+          <t>PVC</t>
         </is>
       </c>
       <c r="G451" t="n">
-        <v>355</v>
+        <v>200</v>
       </c>
       <c r="H451" t="inlineStr">
         <is>
-          <t>Metodo Nao Destrutivo - MND</t>
+          <t>Vala a Ceu Aberto - VCA</t>
         </is>
       </c>
       <c r="I451" t="n">
-        <v>64.572</v>
-      </c>
-      <c r="J451" t="n">
-        <v>3.1</v>
+        <v>5</v>
       </c>
       <c r="K451" t="n">
-        <v>3.1</v>
+        <v>1.35</v>
       </c>
       <c r="L451" t="n">
-        <v>5.48</v>
+        <v>1.35</v>
       </c>
       <c r="M451" t="inlineStr">
         <is>
@@ -53054,20 +53054,20 @@
       </c>
       <c r="N451" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; PV-16 ao PV-17; arquivo: planos_furo/cts_joao_canzi_fl07_pv16_pv17.pdf; taxa 0,0707.</t>
+          <t>Interligacao PV-75.1 -&gt; PV-75 adicionada via Google Earth.</t>
         </is>
       </c>
       <c r="O451" t="n">
-        <v>-23.5299843</v>
+        <v>-23.5198222</v>
       </c>
       <c r="P451" t="n">
-        <v>-46.3845231</v>
+        <v>-46.3768722</v>
       </c>
       <c r="Q451" t="n">
-        <v>-23.5300354</v>
+        <v>-23.5198</v>
       </c>
       <c r="R451" t="n">
-        <v>-46.3838931</v>
+        <v>-46.3763</v>
       </c>
     </row>
     <row r="452">
@@ -53078,22 +53078,22 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>JC-015</t>
+          <t>JC-014</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>PV-17 - PV-18</t>
+          <t>PV-16 - PV-17</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
         <is>
+          <t>PV-16</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
           <t>PV-17</t>
-        </is>
-      </c>
-      <c r="E452" t="inlineStr">
-        <is>
-          <t>PV-18</t>
         </is>
       </c>
       <c r="F452" t="inlineStr">
@@ -53110,16 +53110,16 @@
         </is>
       </c>
       <c r="I452" t="n">
-        <v>79.57599999999999</v>
+        <v>64.572</v>
       </c>
       <c r="J452" t="n">
         <v>3.1</v>
       </c>
       <c r="K452" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="L452" t="n">
-        <v>3.56</v>
+        <v>5.48</v>
       </c>
       <c r="M452" t="inlineStr">
         <is>
@@ -53128,20 +53128,20 @@
       </c>
       <c r="N452" t="inlineStr">
         <is>
-          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; PV-17 ao PV-18; arquivo: planos_furo/cts_joao_canzi_fl07_pv17_pv18.pdf; taxa 0,0116.</t>
+          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; PV-16 ao PV-17; arquivo: planos_furo/cts_joao_canzi_fl07_pv16_pv17.pdf; taxa 0,0707.</t>
         </is>
       </c>
       <c r="O452" t="n">
+        <v>-23.5299843</v>
+      </c>
+      <c r="P452" t="n">
+        <v>-46.3845231</v>
+      </c>
+      <c r="Q452" t="n">
         <v>-23.5300354</v>
       </c>
-      <c r="P452" t="n">
+      <c r="R452" t="n">
         <v>-46.3838931</v>
-      </c>
-      <c r="Q452" t="n">
-        <v>-23.5300223</v>
-      </c>
-      <c r="R452" t="n">
-        <v>-46.3831139</v>
       </c>
     </row>
     <row r="453">
@@ -53152,22 +53152,22 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>JC-016</t>
+          <t>JC-015</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>PV-19 - PV-20</t>
+          <t>PV-17 - PV-18</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>PV-19</t>
+          <t>PV-17</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>PV-20</t>
+          <t>PV-18</t>
         </is>
       </c>
       <c r="F453" t="inlineStr">
@@ -53184,37 +53184,111 @@
         </is>
       </c>
       <c r="I453" t="n">
+        <v>79.57599999999999</v>
+      </c>
+      <c r="J453" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K453" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L453" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N453" t="inlineStr">
+        <is>
+          <t>Plano de furo FL-07 versao 01, 02.JUN.2026; PV-17 ao PV-18; arquivo: planos_furo/cts_joao_canzi_fl07_pv17_pv18.pdf; taxa 0,0116.</t>
+        </is>
+      </c>
+      <c r="O453" t="n">
+        <v>-23.5300354</v>
+      </c>
+      <c r="P453" t="n">
+        <v>-46.3838931</v>
+      </c>
+      <c r="Q453" t="n">
+        <v>-23.5300223</v>
+      </c>
+      <c r="R453" t="n">
+        <v>-46.3831139</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>cts_joao_canzi</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>JC-016</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>PV-19 - PV-20</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>PV-19</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>PV-20</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>PEAD LISO</t>
+        </is>
+      </c>
+      <c r="G454" t="n">
+        <v>355</v>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>Metodo Nao Destrutivo - MND</t>
+        </is>
+      </c>
+      <c r="I454" t="n">
         <v>57.846</v>
       </c>
-      <c r="J453" t="n">
+      <c r="J454" t="n">
         <v>4</v>
       </c>
-      <c r="K453" t="n">
+      <c r="K454" t="n">
         <v>3.96</v>
       </c>
-      <c r="L453" t="n">
+      <c r="L454" t="n">
         <v>4</v>
       </c>
-      <c r="M453" t="inlineStr">
+      <c r="M454" t="inlineStr">
         <is>
           <t>em andamento</t>
         </is>
       </c>
-      <c r="N453" t="inlineStr">
+      <c r="N454" t="inlineStr">
         <is>
           <t>Plano de furo FL-07 versao 01, 05.JUN.2026; PV-19 ao PV-20; arquivo: planos_furo/cts_joao_canzi_fl07_pv19_pv20.pdf; taxa 0,1224.</t>
         </is>
       </c>
-      <c r="O453" t="n">
+      <c r="O454" t="n">
         <v>-23.529877</v>
       </c>
-      <c r="P453" t="n">
+      <c r="P454" t="n">
         <v>-46.3824799</v>
       </c>
-      <c r="Q453" t="n">
+      <c r="Q454" t="n">
         <v>-23.5295804</v>
       </c>
-      <c r="R453" t="n">
+      <c r="R454" t="n">
         <v>-46.3820136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Restaura mapa Elias Sleiman
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1197,7 +1197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L441"/>
+  <dimension ref="A1:L447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -21205,6 +21205,294 @@
       <c r="L441" t="inlineStr">
         <is>
           <t>Plano de furo FL-07 versao 01, 05.JUN.2026; trecho PV-19 ao PV-20.</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>ELIAS-PV-24</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>PV-24</t>
+        </is>
+      </c>
+      <c r="E442" t="n">
+        <v>7397047.32</v>
+      </c>
+      <c r="F442" t="n">
+        <v>358826.273</v>
+      </c>
+      <c r="G442" t="n">
+        <v>-23.5307209</v>
+      </c>
+      <c r="H442" t="n">
+        <v>-46.3829268</v>
+      </c>
+      <c r="I442" t="n">
+        <v>795.659</v>
+      </c>
+      <c r="J442" t="n">
+        <v>793.298</v>
+      </c>
+      <c r="K442" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>ELIAS-PV-25</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>PV-25</t>
+        </is>
+      </c>
+      <c r="E443" t="n">
+        <v>7397044.193</v>
+      </c>
+      <c r="F443" t="n">
+        <v>358909.128</v>
+      </c>
+      <c r="G443" t="n">
+        <v>-23.5307563</v>
+      </c>
+      <c r="H443" t="n">
+        <v>-46.3821157</v>
+      </c>
+      <c r="I443" t="n">
+        <v>798.554</v>
+      </c>
+      <c r="J443" t="n">
+        <v>795.832</v>
+      </c>
+      <c r="K443" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>ELIAS-PV-26</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>PV-26</t>
+        </is>
+      </c>
+      <c r="E444" t="n">
+        <v>7397000.312</v>
+      </c>
+      <c r="F444" t="n">
+        <v>358903.103</v>
+      </c>
+      <c r="G444" t="n">
+        <v>-23.5311521</v>
+      </c>
+      <c r="H444" t="n">
+        <v>-46.3821788</v>
+      </c>
+      <c r="I444" t="n">
+        <v>803.849</v>
+      </c>
+      <c r="J444" t="n">
+        <v>801.227</v>
+      </c>
+      <c r="K444" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>ELIAS-PV-27</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>PV-27</t>
+        </is>
+      </c>
+      <c r="E445" t="n">
+        <v>7396952.046</v>
+      </c>
+      <c r="F445" t="n">
+        <v>358919.472</v>
+      </c>
+      <c r="G445" t="n">
+        <v>-23.5315893</v>
+      </c>
+      <c r="H445" t="n">
+        <v>-46.3820231</v>
+      </c>
+      <c r="I445" t="n">
+        <v>810.896</v>
+      </c>
+      <c r="J445" t="n">
+        <v>808.804</v>
+      </c>
+      <c r="K445" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>ELIAS-PV-28</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>PV-28</t>
+        </is>
+      </c>
+      <c r="E446" t="n">
+        <v>7396913.479</v>
+      </c>
+      <c r="F446" t="n">
+        <v>358940.543</v>
+      </c>
+      <c r="G446" t="n">
+        <v>-23.5319394</v>
+      </c>
+      <c r="H446" t="n">
+        <v>-46.3818203</v>
+      </c>
+      <c r="I446" t="n">
+        <v>813.813</v>
+      </c>
+      <c r="J446" t="n">
+        <v>811.614</v>
+      </c>
+      <c r="K446" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>ELIAS-PV-29</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>PV-29</t>
+        </is>
+      </c>
+      <c r="E447" t="n">
+        <v>7396888.957</v>
+      </c>
+      <c r="F447" t="n">
+        <v>358954.374</v>
+      </c>
+      <c r="G447" t="n">
+        <v>-23.5321621</v>
+      </c>
+      <c r="H447" t="n">
+        <v>-46.3816872</v>
+      </c>
+      <c r="I447" t="n">
+        <v>815.335</v>
+      </c>
+      <c r="J447" t="n">
+        <v>813.135</v>
+      </c>
+      <c r="K447" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
         </is>
       </c>
     </row>
@@ -21219,7 +21507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R454"/>
+  <dimension ref="A1:R460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -53290,6 +53578,450 @@
       </c>
       <c r="R454" t="n">
         <v>-46.3820136</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>ELIAS-003</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>PV-23 - PV-24</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>PV-23</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>PV-24</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G455" t="n">
+        <v>200</v>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I455" t="n">
+        <v>44.64</v>
+      </c>
+      <c r="J455" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="K455" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="L455" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N455" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+      <c r="O455" t="n">
+        <v>-23.5309793</v>
+      </c>
+      <c r="P455" t="n">
+        <v>-46.3832624</v>
+      </c>
+      <c r="Q455" t="n">
+        <v>-23.5307209</v>
+      </c>
+      <c r="R455" t="n">
+        <v>-46.3829268</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>ELIAS-004</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>PV-24 - PV-25</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>PV-24</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>PV-25</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G456" t="n">
+        <v>200</v>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I456" t="n">
+        <v>82.91</v>
+      </c>
+      <c r="J456" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="K456" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="L456" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N456" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+      <c r="O456" t="n">
+        <v>-23.5307209</v>
+      </c>
+      <c r="P456" t="n">
+        <v>-46.3829268</v>
+      </c>
+      <c r="Q456" t="n">
+        <v>-23.5307563</v>
+      </c>
+      <c r="R456" t="n">
+        <v>-46.3821157</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>ELIAS-005</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>PV-25 - PV-26</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>PV-25</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>PV-26</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G457" t="n">
+        <v>200</v>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I457" t="n">
+        <v>44.29</v>
+      </c>
+      <c r="J457" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="K457" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="L457" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N457" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+      <c r="O457" t="n">
+        <v>-23.5307563</v>
+      </c>
+      <c r="P457" t="n">
+        <v>-46.3821157</v>
+      </c>
+      <c r="Q457" t="n">
+        <v>-23.5311521</v>
+      </c>
+      <c r="R457" t="n">
+        <v>-46.3821788</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>ELIAS-006</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>PV-26 - PV-27</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>PV-26</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>PV-27</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G458" t="n">
+        <v>200</v>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I458" t="n">
+        <v>50.97</v>
+      </c>
+      <c r="J458" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="K458" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="L458" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N458" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+      <c r="O458" t="n">
+        <v>-23.5311521</v>
+      </c>
+      <c r="P458" t="n">
+        <v>-46.3821788</v>
+      </c>
+      <c r="Q458" t="n">
+        <v>-23.5315893</v>
+      </c>
+      <c r="R458" t="n">
+        <v>-46.3820231</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>ELIAS-007</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>PV-27 - PV-28</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>PV-27</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>PV-28</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G459" t="n">
+        <v>200</v>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I459" t="n">
+        <v>43.95</v>
+      </c>
+      <c r="J459" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="K459" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L459" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N459" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+      <c r="O459" t="n">
+        <v>-23.5315893</v>
+      </c>
+      <c r="P459" t="n">
+        <v>-46.3820231</v>
+      </c>
+      <c r="Q459" t="n">
+        <v>-23.5319394</v>
+      </c>
+      <c r="R459" t="n">
+        <v>-46.3818203</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>ELIAS-008</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>PV-28 - PV-29</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>PV-28</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>PV-29</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G460" t="n">
+        <v>200</v>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I460" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="J460" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K460" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L460" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N460" t="inlineStr">
+        <is>
+          <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+      <c r="O460" t="n">
+        <v>-23.5319394</v>
+      </c>
+      <c r="P460" t="n">
+        <v>-46.3818203</v>
+      </c>
+      <c r="Q460" t="n">
+        <v>-23.5321621</v>
+      </c>
+      <c r="R460" t="n">
+        <v>-46.3816872</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona RCE Maria dos Santos Machado ao mapa
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="31.109375" customWidth="1" min="1" max="1"/>
@@ -1181,6 +1181,33 @@
         </is>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RCE Maria dos Santos Machado</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>RCE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1197,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L447"/>
+  <dimension ref="A1:L452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -21493,6 +21520,201 @@
       <c r="L447" t="inlineStr">
         <is>
           <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>PVP</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>MSM-PVP-09</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>PVP-09</t>
+        </is>
+      </c>
+      <c r="E448" t="n">
+        <v>7391178.44</v>
+      </c>
+      <c r="F448" t="n">
+        <v>338156.44</v>
+      </c>
+      <c r="G448" t="n">
+        <v>-23.5817824</v>
+      </c>
+      <c r="H448" t="n">
+        <v>-46.5859865</v>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>MSM-PI-1</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>PI-1</t>
+        </is>
+      </c>
+      <c r="E449" t="n">
+        <v>7391179.4</v>
+      </c>
+      <c r="F449" t="n">
+        <v>338179.5</v>
+      </c>
+      <c r="G449" t="n">
+        <v>-23.581776</v>
+      </c>
+      <c r="H449" t="n">
+        <v>-46.5857605</v>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>MSM-PI-2</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>PI-2</t>
+        </is>
+      </c>
+      <c r="E450" t="n">
+        <v>7391227.64</v>
+      </c>
+      <c r="F450" t="n">
+        <v>338227.56</v>
+      </c>
+      <c r="G450" t="n">
+        <v>-23.5813453</v>
+      </c>
+      <c r="H450" t="n">
+        <v>-46.5852845</v>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>MSM-PI-3</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>PI-3</t>
+        </is>
+      </c>
+      <c r="E451" t="n">
+        <v>7391286.79</v>
+      </c>
+      <c r="F451" t="n">
+        <v>338260.79</v>
+      </c>
+      <c r="G451" t="n">
+        <v>-23.5808145</v>
+      </c>
+      <c r="H451" t="n">
+        <v>-46.5849525</v>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>MSM-PI-4</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>PI-4</t>
+        </is>
+      </c>
+      <c r="E452" t="n">
+        <v>7391325.91</v>
+      </c>
+      <c r="F452" t="n">
+        <v>338287.591</v>
+      </c>
+      <c r="G452" t="n">
+        <v>-23.580464</v>
+      </c>
+      <c r="H452" t="n">
+        <v>-46.5846857</v>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
         </is>
       </c>
     </row>
@@ -21507,7 +21729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R460"/>
+  <dimension ref="A1:R464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -54022,6 +54244,266 @@
       </c>
       <c r="R460" t="n">
         <v>-46.3816872</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>MSM-001</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>PVP-09 - PI-1</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>PVP-09</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>PI-1</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G461" t="n">
+        <v>200</v>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I461" t="n">
+        <v>20</v>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N461" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+      <c r="O461" t="n">
+        <v>-23.5817824</v>
+      </c>
+      <c r="P461" t="n">
+        <v>-46.5859865</v>
+      </c>
+      <c r="Q461" t="n">
+        <v>-23.581776</v>
+      </c>
+      <c r="R461" t="n">
+        <v>-46.5857605</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>MSM-002</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>PI-1 - PI-2</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>PI-1</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>PI-2</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G462" t="n">
+        <v>200</v>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I462" t="n">
+        <v>66</v>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N462" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+      <c r="O462" t="n">
+        <v>-23.581776</v>
+      </c>
+      <c r="P462" t="n">
+        <v>-46.5857605</v>
+      </c>
+      <c r="Q462" t="n">
+        <v>-23.5813453</v>
+      </c>
+      <c r="R462" t="n">
+        <v>-46.5852845</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>MSM-003</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>PI-2 - PI-3</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>PI-2</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>PI-3</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G463" t="n">
+        <v>200</v>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I463" t="n">
+        <v>62</v>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N463" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+      <c r="O463" t="n">
+        <v>-23.5813453</v>
+      </c>
+      <c r="P463" t="n">
+        <v>-46.5852845</v>
+      </c>
+      <c r="Q463" t="n">
+        <v>-23.5808145</v>
+      </c>
+      <c r="R463" t="n">
+        <v>-46.5849525</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>MSM-004</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>PI-3 - PI-4</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>PI-3</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>PI-4</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G464" t="n">
+        <v>200</v>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I464" t="n">
+        <v>41</v>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N464" t="inlineStr">
+        <is>
+          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
+        </is>
+      </c>
+      <c r="O464" t="n">
+        <v>-23.5808145</v>
+      </c>
+      <c r="P464" t="n">
+        <v>-46.5849525</v>
+      </c>
+      <c r="Q464" t="n">
+        <v>-23.580464</v>
+      </c>
+      <c r="R464" t="n">
+        <v>-46.5846857</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove RCE Maria dos Santos Machado do mapa
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="31.109375" customWidth="1" min="1" max="1"/>
@@ -1181,33 +1181,6 @@
         </is>
       </c>
       <c r="E26" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>RCE Maria dos Santos Machado</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>RCE</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1224,7 +1197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L452"/>
+  <dimension ref="A1:L447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -21520,201 +21493,6 @@
       <c r="L447" t="inlineStr">
         <is>
           <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="448">
-      <c r="A448" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B448" t="inlineStr">
-        <is>
-          <t>PVP</t>
-        </is>
-      </c>
-      <c r="C448" t="inlineStr">
-        <is>
-          <t>MSM-PVP-09</t>
-        </is>
-      </c>
-      <c r="D448" t="inlineStr">
-        <is>
-          <t>PVP-09</t>
-        </is>
-      </c>
-      <c r="E448" t="n">
-        <v>7391178.44</v>
-      </c>
-      <c r="F448" t="n">
-        <v>338156.44</v>
-      </c>
-      <c r="G448" t="n">
-        <v>-23.5817824</v>
-      </c>
-      <c r="H448" t="n">
-        <v>-46.5859865</v>
-      </c>
-      <c r="L448" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="449">
-      <c r="A449" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B449" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="C449" t="inlineStr">
-        <is>
-          <t>MSM-PI-1</t>
-        </is>
-      </c>
-      <c r="D449" t="inlineStr">
-        <is>
-          <t>PI-1</t>
-        </is>
-      </c>
-      <c r="E449" t="n">
-        <v>7391179.4</v>
-      </c>
-      <c r="F449" t="n">
-        <v>338179.5</v>
-      </c>
-      <c r="G449" t="n">
-        <v>-23.581776</v>
-      </c>
-      <c r="H449" t="n">
-        <v>-46.5857605</v>
-      </c>
-      <c r="L449" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="450">
-      <c r="A450" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B450" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="C450" t="inlineStr">
-        <is>
-          <t>MSM-PI-2</t>
-        </is>
-      </c>
-      <c r="D450" t="inlineStr">
-        <is>
-          <t>PI-2</t>
-        </is>
-      </c>
-      <c r="E450" t="n">
-        <v>7391227.64</v>
-      </c>
-      <c r="F450" t="n">
-        <v>338227.56</v>
-      </c>
-      <c r="G450" t="n">
-        <v>-23.5813453</v>
-      </c>
-      <c r="H450" t="n">
-        <v>-46.5852845</v>
-      </c>
-      <c r="L450" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="451">
-      <c r="A451" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B451" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="C451" t="inlineStr">
-        <is>
-          <t>MSM-PI-3</t>
-        </is>
-      </c>
-      <c r="D451" t="inlineStr">
-        <is>
-          <t>PI-3</t>
-        </is>
-      </c>
-      <c r="E451" t="n">
-        <v>7391286.79</v>
-      </c>
-      <c r="F451" t="n">
-        <v>338260.79</v>
-      </c>
-      <c r="G451" t="n">
-        <v>-23.5808145</v>
-      </c>
-      <c r="H451" t="n">
-        <v>-46.5849525</v>
-      </c>
-      <c r="L451" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="452">
-      <c r="A452" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B452" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="C452" t="inlineStr">
-        <is>
-          <t>MSM-PI-4</t>
-        </is>
-      </c>
-      <c r="D452" t="inlineStr">
-        <is>
-          <t>PI-4</t>
-        </is>
-      </c>
-      <c r="E452" t="n">
-        <v>7391325.91</v>
-      </c>
-      <c r="F452" t="n">
-        <v>338287.591</v>
-      </c>
-      <c r="G452" t="n">
-        <v>-23.580464</v>
-      </c>
-      <c r="H452" t="n">
-        <v>-46.5846857</v>
-      </c>
-      <c r="L452" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
         </is>
       </c>
     </row>
@@ -21729,7 +21507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R464"/>
+  <dimension ref="A1:R460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -54244,266 +54022,6 @@
       </c>
       <c r="R460" t="n">
         <v>-46.3816872</v>
-      </c>
-    </row>
-    <row r="461">
-      <c r="A461" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B461" t="inlineStr">
-        <is>
-          <t>MSM-001</t>
-        </is>
-      </c>
-      <c r="C461" t="inlineStr">
-        <is>
-          <t>PVP-09 - PI-1</t>
-        </is>
-      </c>
-      <c r="D461" t="inlineStr">
-        <is>
-          <t>PVP-09</t>
-        </is>
-      </c>
-      <c r="E461" t="inlineStr">
-        <is>
-          <t>PI-1</t>
-        </is>
-      </c>
-      <c r="F461" t="inlineStr">
-        <is>
-          <t>PVC</t>
-        </is>
-      </c>
-      <c r="G461" t="n">
-        <v>200</v>
-      </c>
-      <c r="H461" t="inlineStr">
-        <is>
-          <t>Vala a Ceu Aberto - VCA</t>
-        </is>
-      </c>
-      <c r="I461" t="n">
-        <v>20</v>
-      </c>
-      <c r="M461" t="inlineStr">
-        <is>
-          <t>em andamento</t>
-        </is>
-      </c>
-      <c r="N461" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-      <c r="O461" t="n">
-        <v>-23.5817824</v>
-      </c>
-      <c r="P461" t="n">
-        <v>-46.5859865</v>
-      </c>
-      <c r="Q461" t="n">
-        <v>-23.581776</v>
-      </c>
-      <c r="R461" t="n">
-        <v>-46.5857605</v>
-      </c>
-    </row>
-    <row r="462">
-      <c r="A462" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B462" t="inlineStr">
-        <is>
-          <t>MSM-002</t>
-        </is>
-      </c>
-      <c r="C462" t="inlineStr">
-        <is>
-          <t>PI-1 - PI-2</t>
-        </is>
-      </c>
-      <c r="D462" t="inlineStr">
-        <is>
-          <t>PI-1</t>
-        </is>
-      </c>
-      <c r="E462" t="inlineStr">
-        <is>
-          <t>PI-2</t>
-        </is>
-      </c>
-      <c r="F462" t="inlineStr">
-        <is>
-          <t>PVC</t>
-        </is>
-      </c>
-      <c r="G462" t="n">
-        <v>200</v>
-      </c>
-      <c r="H462" t="inlineStr">
-        <is>
-          <t>Vala a Ceu Aberto - VCA</t>
-        </is>
-      </c>
-      <c r="I462" t="n">
-        <v>66</v>
-      </c>
-      <c r="M462" t="inlineStr">
-        <is>
-          <t>em andamento</t>
-        </is>
-      </c>
-      <c r="N462" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-      <c r="O462" t="n">
-        <v>-23.581776</v>
-      </c>
-      <c r="P462" t="n">
-        <v>-46.5857605</v>
-      </c>
-      <c r="Q462" t="n">
-        <v>-23.5813453</v>
-      </c>
-      <c r="R462" t="n">
-        <v>-46.5852845</v>
-      </c>
-    </row>
-    <row r="463">
-      <c r="A463" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B463" t="inlineStr">
-        <is>
-          <t>MSM-003</t>
-        </is>
-      </c>
-      <c r="C463" t="inlineStr">
-        <is>
-          <t>PI-2 - PI-3</t>
-        </is>
-      </c>
-      <c r="D463" t="inlineStr">
-        <is>
-          <t>PI-2</t>
-        </is>
-      </c>
-      <c r="E463" t="inlineStr">
-        <is>
-          <t>PI-3</t>
-        </is>
-      </c>
-      <c r="F463" t="inlineStr">
-        <is>
-          <t>PVC</t>
-        </is>
-      </c>
-      <c r="G463" t="n">
-        <v>200</v>
-      </c>
-      <c r="H463" t="inlineStr">
-        <is>
-          <t>Vala a Ceu Aberto - VCA</t>
-        </is>
-      </c>
-      <c r="I463" t="n">
-        <v>62</v>
-      </c>
-      <c r="M463" t="inlineStr">
-        <is>
-          <t>em andamento</t>
-        </is>
-      </c>
-      <c r="N463" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-      <c r="O463" t="n">
-        <v>-23.5813453</v>
-      </c>
-      <c r="P463" t="n">
-        <v>-46.5852845</v>
-      </c>
-      <c r="Q463" t="n">
-        <v>-23.5808145</v>
-      </c>
-      <c r="R463" t="n">
-        <v>-46.5849525</v>
-      </c>
-    </row>
-    <row r="464">
-      <c r="A464" t="inlineStr">
-        <is>
-          <t>rce_maria_dos_santos_machado</t>
-        </is>
-      </c>
-      <c r="B464" t="inlineStr">
-        <is>
-          <t>MSM-004</t>
-        </is>
-      </c>
-      <c r="C464" t="inlineStr">
-        <is>
-          <t>PI-3 - PI-4</t>
-        </is>
-      </c>
-      <c r="D464" t="inlineStr">
-        <is>
-          <t>PI-3</t>
-        </is>
-      </c>
-      <c r="E464" t="inlineStr">
-        <is>
-          <t>PI-4</t>
-        </is>
-      </c>
-      <c r="F464" t="inlineStr">
-        <is>
-          <t>PVC</t>
-        </is>
-      </c>
-      <c r="G464" t="n">
-        <v>200</v>
-      </c>
-      <c r="H464" t="inlineStr">
-        <is>
-          <t>Vala a Ceu Aberto - VCA</t>
-        </is>
-      </c>
-      <c r="I464" t="n">
-        <v>41</v>
-      </c>
-      <c r="M464" t="inlineStr">
-        <is>
-          <t>em andamento</t>
-        </is>
-      </c>
-      <c r="N464" t="inlineStr">
-        <is>
-          <t>Adicionado via prints enviados em 17/07/2026; coordenadas SIRGAS 2000 / UTM zona 23S convertidas para latitude/longitude; trechos em VCA.</t>
-        </is>
-      </c>
-      <c r="O464" t="n">
-        <v>-23.5808145</v>
-      </c>
-      <c r="P464" t="n">
-        <v>-46.5849525</v>
-      </c>
-      <c r="Q464" t="n">
-        <v>-23.580464</v>
-      </c>
-      <c r="R464" t="n">
-        <v>-46.5846857</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona Maria dos Santos Machado ligada ao PV16
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="31.109375" customWidth="1" min="1" max="1"/>
@@ -1181,6 +1181,33 @@
         </is>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RCE Maria dos Santos Machado</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>RCE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1197,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L447"/>
+  <dimension ref="A1:L452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -21493,6 +21520,186 @@
       <c r="L447" t="inlineStr">
         <is>
           <t>Adicionado via prints do projeto RCE Elias Sleiman recebidos em 22/06/2026; lancamento completo em VCA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>MSM-PV-16</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>PV-16</t>
+        </is>
+      </c>
+      <c r="E448" t="n">
+        <v>7397127.313</v>
+      </c>
+      <c r="F448" t="n">
+        <v>358662.509</v>
+      </c>
+      <c r="G448" t="n">
+        <v>-23.5299843</v>
+      </c>
+      <c r="H448" t="n">
+        <v>-46.3845231</v>
+      </c>
+      <c r="I448" t="n">
+        <v>777.73</v>
+      </c>
+      <c r="J448" t="n">
+        <v>774.633</v>
+      </c>
+      <c r="K448" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t>Ponto de ligação no CTS João Canzi. Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>MSM-PI-1</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>PI-1</t>
+        </is>
+      </c>
+      <c r="G449" t="n">
+        <v>-23.5298809</v>
+      </c>
+      <c r="H449" t="n">
+        <v>-46.3845564</v>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>MSM-PI-2</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>PI-2</t>
+        </is>
+      </c>
+      <c r="G450" t="n">
+        <v>-23.529364</v>
+      </c>
+      <c r="H450" t="n">
+        <v>-46.3847229</v>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>MSM-PI-3</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>PI-3</t>
+        </is>
+      </c>
+      <c r="G451" t="n">
+        <v>-23.5287954</v>
+      </c>
+      <c r="H451" t="n">
+        <v>-46.384906</v>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>MSM-PI-4</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>PI-4</t>
+        </is>
+      </c>
+      <c r="G452" t="n">
+        <v>-23.5281583</v>
+      </c>
+      <c r="H452" t="n">
+        <v>-46.3851111</v>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
         </is>
       </c>
     </row>
@@ -21507,7 +21714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R460"/>
+  <dimension ref="A1:R464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -54022,6 +54229,266 @@
       </c>
       <c r="R460" t="n">
         <v>-46.3816872</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>MSM-001</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>PV-16 - PI-1</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>PV-16</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>PI-1</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G461" t="n">
+        <v>200</v>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I461" t="n">
+        <v>12</v>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N461" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+      <c r="O461" t="n">
+        <v>-23.5299843</v>
+      </c>
+      <c r="P461" t="n">
+        <v>-46.3845231</v>
+      </c>
+      <c r="Q461" t="n">
+        <v>-23.5298809</v>
+      </c>
+      <c r="R461" t="n">
+        <v>-46.3845564</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>MSM-002</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>PI-1 - PI-2</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>PI-1</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>PI-2</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G462" t="n">
+        <v>200</v>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I462" t="n">
+        <v>60</v>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N462" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+      <c r="O462" t="n">
+        <v>-23.5298809</v>
+      </c>
+      <c r="P462" t="n">
+        <v>-46.3845564</v>
+      </c>
+      <c r="Q462" t="n">
+        <v>-23.529364</v>
+      </c>
+      <c r="R462" t="n">
+        <v>-46.3847229</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>MSM-003</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>PI-2 - PI-3</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>PI-2</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>PI-3</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G463" t="n">
+        <v>200</v>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I463" t="n">
+        <v>66</v>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N463" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+      <c r="O463" t="n">
+        <v>-23.529364</v>
+      </c>
+      <c r="P463" t="n">
+        <v>-46.3847229</v>
+      </c>
+      <c r="Q463" t="n">
+        <v>-23.5287954</v>
+      </c>
+      <c r="R463" t="n">
+        <v>-46.384906</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>rce_maria_dos_santos_machado</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>MSM-004</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>PI-3 - PI-4</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>PI-3</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>PI-4</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G464" t="n">
+        <v>200</v>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I464" t="n">
+        <v>73.94</v>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N464" t="inlineStr">
+        <is>
+          <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+      <c r="O464" t="n">
+        <v>-23.5287954</v>
+      </c>
+      <c r="P464" t="n">
+        <v>-46.384906</v>
+      </c>
+      <c r="Q464" t="n">
+        <v>-23.5281583</v>
+      </c>
+      <c r="R464" t="n">
+        <v>-46.3851111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Interliga Joao Canzi com Elias Sleiman
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1224,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L452"/>
+  <dimension ref="A1:L453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -21700,6 +21700,54 @@
       <c r="L452" t="inlineStr">
         <is>
           <t>Adicionado via coordenada PI-4 enviada em 17/07/2026; ligação no PV-16 do CTS João Canzi; PIs intermediários distribuídos por distância informada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>ELIAS-PV-17-LIG-JC</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>PV-17</t>
+        </is>
+      </c>
+      <c r="E453" t="n">
+        <v>7397122.275</v>
+      </c>
+      <c r="F453" t="n">
+        <v>358726.884</v>
+      </c>
+      <c r="G453" t="n">
+        <v>-23.5300354</v>
+      </c>
+      <c r="H453" t="n">
+        <v>-46.3838931</v>
+      </c>
+      <c r="I453" t="n">
+        <v>782.299</v>
+      </c>
+      <c r="J453" t="n">
+        <v>779.199</v>
+      </c>
+      <c r="K453" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t>Interligação adicionada em 17/07/2026 entre o PV-17 do CTS João Canzi e o PV-21 da RCE Elias Sleiman.</t>
         </is>
       </c>
     </row>
@@ -21714,7 +21762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R464"/>
+  <dimension ref="A1:R465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -54489,6 +54537,80 @@
       </c>
       <c r="R464" t="n">
         <v>-46.3851111</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>rce_elias_sleiman</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>ELIAS-000</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>PV-17 - PV-21</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>PV-17</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>PV-21</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G465" t="n">
+        <v>200</v>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I465" t="n">
+        <v>23.32</v>
+      </c>
+      <c r="J465" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="K465" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="L465" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N465" t="inlineStr">
+        <is>
+          <t>Interligação adicionada em 17/07/2026 entre o PV-17 do CTS João Canzi e o PV-21 da RCE Elias Sleiman.</t>
+        </is>
+      </c>
+      <c r="O465" t="n">
+        <v>-23.5300354</v>
+      </c>
+      <c r="P465" t="n">
+        <v>-46.3838931</v>
+      </c>
+      <c r="Q465" t="n">
+        <v>-23.5301384</v>
+      </c>
+      <c r="R465" t="n">
+        <v>-46.3836941</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completa RCE Elvira de Araujo ate PV05
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1224,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L453"/>
+  <dimension ref="A1:L456"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -19442,29 +19442,29 @@
         </is>
       </c>
       <c r="E403" t="n">
-        <v>7396941.756</v>
+        <v>7396927.156</v>
       </c>
       <c r="F403" t="n">
-        <v>358324.032</v>
+        <v>358327.601</v>
       </c>
       <c r="G403" t="n">
-        <v>-23.5316304</v>
+        <v>-23.5317625</v>
       </c>
       <c r="H403" t="n">
-        <v>-46.3878556</v>
+        <v>-46.3878221</v>
       </c>
       <c r="I403" t="n">
-        <v>767.318</v>
+        <v>767.145</v>
       </c>
       <c r="J403" t="n">
-        <v>763.468</v>
+        <v>763.135</v>
       </c>
       <c r="K403" t="n">
-        <v>3.85</v>
+        <v>4.01</v>
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t>Movido para RCE Elvira de Araujo conforme correcao de obra em 09.JUN.2026.</t>
+          <t>Atualizado via prints enviados em 17/07/2026: continuidade da RCE Elvira de Araújo do PV-02 ao PV-05.</t>
         </is>
       </c>
     </row>
@@ -21748,6 +21748,150 @@
       <c r="L453" t="inlineStr">
         <is>
           <t>Interligação adicionada em 17/07/2026 entre o PV-17 do CTS João Canzi e o PV-21 da RCE Elias Sleiman.</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>rce_elvira_de_araujo</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>ELVIRA-PV-03</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>PV-03</t>
+        </is>
+      </c>
+      <c r="E454" t="n">
+        <v>7396959.815</v>
+      </c>
+      <c r="F454" t="n">
+        <v>358322.872</v>
+      </c>
+      <c r="G454" t="n">
+        <v>-23.5314672</v>
+      </c>
+      <c r="H454" t="n">
+        <v>-46.3878653</v>
+      </c>
+      <c r="I454" t="n">
+        <v>769.252</v>
+      </c>
+      <c r="J454" t="n">
+        <v>766.7670000000001</v>
+      </c>
+      <c r="K454" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="L454" t="inlineStr">
+        <is>
+          <t>Atualizado via prints enviados em 17/07/2026: continuidade da RCE Elvira de Araújo do PV-02 ao PV-05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>rce_elvira_de_araujo</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>ELVIRA-PV-04</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>PV-04</t>
+        </is>
+      </c>
+      <c r="E455" t="n">
+        <v>7397004.412</v>
+      </c>
+      <c r="F455" t="n">
+        <v>358316.86</v>
+      </c>
+      <c r="G455" t="n">
+        <v>-23.5310639</v>
+      </c>
+      <c r="H455" t="n">
+        <v>-46.3879199</v>
+      </c>
+      <c r="I455" t="n">
+        <v>776.184</v>
+      </c>
+      <c r="J455" t="n">
+        <v>774.138</v>
+      </c>
+      <c r="K455" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t>Atualizado via prints enviados em 17/07/2026: continuidade da RCE Elvira de Araújo do PV-02 ao PV-05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>rce_elvira_de_araujo</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>ELVIRA-PV-05</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>PV-05</t>
+        </is>
+      </c>
+      <c r="E456" t="n">
+        <v>7397057.922</v>
+      </c>
+      <c r="F456" t="n">
+        <v>358309.601</v>
+      </c>
+      <c r="G456" t="n">
+        <v>-23.5305801</v>
+      </c>
+      <c r="H456" t="n">
+        <v>-46.387986</v>
+      </c>
+      <c r="I456" t="n">
+        <v>782.579</v>
+      </c>
+      <c r="J456" t="n">
+        <v>780.861</v>
+      </c>
+      <c r="K456" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t>Atualizado via prints enviados em 17/07/2026: continuidade da RCE Elvira de Araújo do PV-02 ao PV-05.</t>
         </is>
       </c>
     </row>
@@ -21762,7 +21906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R465"/>
+  <dimension ref="A1:R468"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -50232,7 +50376,7 @@
         <v>4.15</v>
       </c>
       <c r="K405" t="n">
-        <v>3.85</v>
+        <v>4.01</v>
       </c>
       <c r="L405" t="n">
         <v>4.15</v>
@@ -50254,10 +50398,10 @@
         <v>-46.3877736</v>
       </c>
       <c r="Q405" t="n">
-        <v>-23.5316304</v>
+        <v>-23.5317625</v>
       </c>
       <c r="R405" t="n">
-        <v>-46.3878556</v>
+        <v>-46.3878221</v>
       </c>
     </row>
     <row r="406" hidden="1">
@@ -54611,6 +54755,228 @@
       </c>
       <c r="R465" t="n">
         <v>-46.3836941</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>rce_elvira_de_araujo</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>ELVIRA-005</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>PV-02 - PV-03</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>PV-02</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>PV-03</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G466" t="n">
+        <v>200</v>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I466" t="n">
+        <v>33</v>
+      </c>
+      <c r="J466" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="K466" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="L466" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N466" t="inlineStr">
+        <is>
+          <t>Atualizado via prints enviados em 17/07/2026: continuidade da RCE Elvira de Araújo do PV-02 ao PV-05.</t>
+        </is>
+      </c>
+      <c r="O466" t="n">
+        <v>-23.5317625</v>
+      </c>
+      <c r="P466" t="n">
+        <v>-46.3878221</v>
+      </c>
+      <c r="Q466" t="n">
+        <v>-23.5314672</v>
+      </c>
+      <c r="R466" t="n">
+        <v>-46.3878653</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>rce_elvira_de_araujo</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>ELVIRA-006</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>PV-03 - PV-04</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>PV-03</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>PV-04</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G467" t="n">
+        <v>200</v>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I467" t="n">
+        <v>45</v>
+      </c>
+      <c r="J467" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="K467" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="L467" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N467" t="inlineStr">
+        <is>
+          <t>Atualizado via prints enviados em 17/07/2026: continuidade da RCE Elvira de Araújo do PV-02 ao PV-05.</t>
+        </is>
+      </c>
+      <c r="O467" t="n">
+        <v>-23.5314672</v>
+      </c>
+      <c r="P467" t="n">
+        <v>-46.3878653</v>
+      </c>
+      <c r="Q467" t="n">
+        <v>-23.5310639</v>
+      </c>
+      <c r="R467" t="n">
+        <v>-46.3879199</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>rce_elvira_de_araujo</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>ELVIRA-007</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>PV-04 - PV-05</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>PV-04</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>PV-05</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G468" t="n">
+        <v>200</v>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I468" t="n">
+        <v>54</v>
+      </c>
+      <c r="J468" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="K468" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="L468" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N468" t="inlineStr">
+        <is>
+          <t>Atualizado via prints enviados em 17/07/2026: continuidade da RCE Elvira de Araújo do PV-02 ao PV-05.</t>
+        </is>
+      </c>
+      <c r="O468" t="n">
+        <v>-23.5310639</v>
+      </c>
+      <c r="P468" t="n">
+        <v>-46.3879199</v>
+      </c>
+      <c r="Q468" t="n">
+        <v>-23.5305801</v>
+      </c>
+      <c r="R468" t="n">
+        <v>-46.387986</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Interliga PV05 ao PT001 em VCA
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -1224,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L456"/>
+  <dimension ref="A1:L457"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -21892,6 +21892,48 @@
       <c r="L456" t="inlineStr">
         <is>
           <t>Atualizado via prints enviados em 17/07/2026: continuidade da RCE Elvira de Araújo do PV-02 ao PV-05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>cts_lourdes_complementar</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>PV</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>LOUR-PT-001</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>PT-001</t>
+        </is>
+      </c>
+      <c r="E457" t="n">
+        <v>7397075.247974937</v>
+      </c>
+      <c r="F457" t="n">
+        <v>357881.2343928794</v>
+      </c>
+      <c r="G457" t="n">
+        <v>-23.5303862</v>
+      </c>
+      <c r="H457" t="n">
+        <v>-46.3921796</v>
+      </c>
+      <c r="K457" t="n">
+        <v>0</v>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t>Interligação VCA adicionada em 17/07/2026 entre PV-05 do CTS Lourdes Complementar e PT-001 do CTS Jardim Lourdes.</t>
         </is>
       </c>
     </row>
@@ -21906,7 +21948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R468"/>
+  <dimension ref="A1:R469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -54977,6 +55019,80 @@
       </c>
       <c r="R468" t="n">
         <v>-46.387986</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>cts_lourdes_complementar</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>LOUR-005</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>PV-05 - PT-001</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>PV-05</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>PT-001</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G469" t="n">
+        <v>300</v>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>Vala a Ceu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I469" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="J469" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K469" t="n">
+        <v>0</v>
+      </c>
+      <c r="L469" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="N469" t="inlineStr">
+        <is>
+          <t>Interligação VCA adicionada em 17/07/2026 entre PV-05 do CTS Lourdes Complementar e PT-001 do CTS Jardim Lourdes.</t>
+        </is>
+      </c>
+      <c r="O469" t="n">
+        <v>-23.530465</v>
+      </c>
+      <c r="P469" t="n">
+        <v>-46.3923061</v>
+      </c>
+      <c r="Q469" t="n">
+        <v>-23.5303862</v>
+      </c>
+      <c r="R469" t="n">
+        <v>-46.3921796</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Conferencia RCE Sao Joao no mapa
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="31.109375" customWidth="1" min="1" max="1"/>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Base real substituída pelo shape completo enviado em 17/07/2026: 19 PVs, 59 PIs e 75 trechos em VCA.</t>
+          <t>Base real substituída pelo shape completo enviado em 17/07/2026, com trecho PV-4.1 ao PV-06 separado para RCE São João em 20/07/2026: 16 PVs, 59 PIs e 73 trechos em VCA.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1235,6 +1235,33 @@
         </is>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>rce_sao_joao</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>RCE Rua São João</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>RCE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Trecho corrigido em 20/07/2026: PV-4.1 ao PV-06, 3 PVs, 2 trechos em VCA, 82,99 m de PVC DN200.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -22180,7 +22207,7 @@
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>rce_comunidade_sao_lucas</t>
+          <t>rce_sao_joao</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
@@ -22190,7 +22217,7 @@
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>SL-PV-05</t>
+          <t>SJ-PV-05</t>
         </is>
       </c>
       <c r="D460" t="inlineStr">
@@ -22221,14 +22248,14 @@
       </c>
       <c r="L460" t="inlineStr">
         <is>
-          <t>Base substituída pelo shape completo enviado em 17/07/2026: Cadastro PV, Cadastro PI e Cadastro Rede da RCE Comunidade São Lucas.</t>
+          <t>Trecho reclassificado para RCE São João em 20/07/2026, conforme conferência em mapa.</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>rce_comunidade_sao_lucas</t>
+          <t>rce_sao_joao</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
@@ -22238,7 +22265,7 @@
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>SL-PV-06</t>
+          <t>SJ-PV-06</t>
         </is>
       </c>
       <c r="D461" t="inlineStr">
@@ -22269,7 +22296,7 @@
       </c>
       <c r="L461" t="inlineStr">
         <is>
-          <t>Base substituída pelo shape completo enviado em 17/07/2026: Cadastro PV, Cadastro PI e Cadastro Rede da RCE Comunidade São Lucas.</t>
+          <t>Trecho reclassificado para RCE São João em 20/07/2026, conforme conferência em mapa.</t>
         </is>
       </c>
     </row>
@@ -22996,7 +23023,7 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>rce_comunidade_sao_lucas</t>
+          <t>rce_sao_joao</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
@@ -23006,7 +23033,7 @@
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>SL-PV-4.1</t>
+          <t>SJ-PV-4.1</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
@@ -23037,7 +23064,7 @@
       </c>
       <c r="L477" t="inlineStr">
         <is>
-          <t>Base substituída pelo shape completo enviado em 17/07/2026: Cadastro PV, Cadastro PI e Cadastro Rede da RCE Comunidade São Lucas.</t>
+          <t>Trecho reclassificado para RCE São João em 20/07/2026, conforme conferência em mapa.</t>
         </is>
       </c>
     </row>
@@ -55587,12 +55614,12 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>rce_comunidade_sao_lucas</t>
+          <t>rce_sao_joao</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>SL-026</t>
+          <t>SJ-002</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -55642,7 +55669,7 @@
       </c>
       <c r="N443" t="inlineStr">
         <is>
-          <t>Base substituída pelo shape completo enviado em 17/07/2026: Cadastro PV, Cadastro PI e Cadastro Rede da RCE Comunidade São Lucas.</t>
+          <t>Trecho reclassificado para RCE São João em 20/07/2026, conforme conferência em mapa.</t>
         </is>
       </c>
       <c r="O443" t="n">
@@ -58769,12 +58796,12 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>rce_comunidade_sao_lucas</t>
+          <t>rce_sao_joao</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>SL-069</t>
+          <t>SJ-001</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
@@ -58824,7 +58851,7 @@
       </c>
       <c r="N486" t="inlineStr">
         <is>
-          <t>Base substituída pelo shape completo enviado em 17/07/2026: Cadastro PV, Cadastro PI e Cadastro Rede da RCE Comunidade São Lucas.</t>
+          <t>Trecho reclassificado para RCE São João em 20/07/2026, conforme conferência em mapa.</t>
         </is>
       </c>
       <c r="O486" t="n">

</xml_diff>

<commit_message>
Adiciona interligacao Ayrton Senna ao mapa
</commit_message>
<xml_diff>
--- a/docs/planilha_base_mapa.xlsx
+++ b/docs/planilha_base_mapa.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="31.109375" customWidth="1" min="1" max="1"/>
@@ -1262,6 +1262,33 @@
         </is>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>interl_rua_ayrton_senna</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>INTERL. RUA AYRTON SENNA</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>INTERL</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>As built INT Ayrton Senna enviado em 20/07/2026: PIE-01 ao PI-02, 3 pontos, 2 trechos em VCA, PVC DN200. Extensao total no perfil: 62,05 m.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1278,7 +1305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L504"/>
+  <dimension ref="A1:L507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -24361,6 +24388,150 @@
       <c r="L504" t="inlineStr">
         <is>
           <t>Base substituída/adicionada pelo shape enviado em 20/07/2026: RCE Elias Sleiman.</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>interl_rua_ayrton_senna</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>AS-PIE-01</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>PIE-01</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>7397669.226</v>
+      </c>
+      <c r="F505" t="n">
+        <v>358321.476</v>
+      </c>
+      <c r="G505" t="n">
+        <v>-23.525061</v>
+      </c>
+      <c r="H505" t="n">
+        <v>-46.3878118</v>
+      </c>
+      <c r="I505" t="n">
+        <v>798.5599999999999</v>
+      </c>
+      <c r="J505" t="n">
+        <v>796.98</v>
+      </c>
+      <c r="K505" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="L505" t="inlineStr">
+        <is>
+          <t>As built INT Ayrton Senna enviado em 20/07/2026: PIE-01 ao PI-02, 3 pontos, 2 trechos em VCA, PVC DN200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>interl_rua_ayrton_senna</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>AS-PI-01</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>PI-01</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>7397708.236</v>
+      </c>
+      <c r="F506" t="n">
+        <v>358282.877</v>
+      </c>
+      <c r="G506" t="n">
+        <v>-23.5247053</v>
+      </c>
+      <c r="H506" t="n">
+        <v>-46.3881861</v>
+      </c>
+      <c r="I506" t="n">
+        <v>800.347</v>
+      </c>
+      <c r="J506" t="n">
+        <v>798.687</v>
+      </c>
+      <c r="K506" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="L506" t="inlineStr">
+        <is>
+          <t>As built INT Ayrton Senna enviado em 20/07/2026: PIE-01 ao PI-02, 3 pontos, 2 trechos em VCA, PVC DN200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>interl_rua_ayrton_senna</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>AS-PI-02</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>PI-02</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>7397706.339</v>
+      </c>
+      <c r="F507" t="n">
+        <v>358275.959</v>
+      </c>
+      <c r="G507" t="n">
+        <v>-23.5247218</v>
+      </c>
+      <c r="H507" t="n">
+        <v>-46.388254</v>
+      </c>
+      <c r="I507" t="n">
+        <v>799.735</v>
+      </c>
+      <c r="J507" t="n">
+        <v>798.765</v>
+      </c>
+      <c r="K507" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L507" t="inlineStr">
+        <is>
+          <t>As built INT Ayrton Senna enviado em 20/07/2026: PIE-01 ao PI-02, 3 pontos, 2 trechos em VCA, PVC DN200.</t>
         </is>
       </c>
     </row>
@@ -24375,7 +24546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R514"/>
+  <dimension ref="A1:R516"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30.21875" customWidth="1" min="1" max="1"/>
@@ -60937,6 +61108,154 @@
       </c>
       <c r="R514" t="n">
         <v>-46.3838928</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>interl_rua_ayrton_senna</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>AS-001</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>PIE-01 - PI-01</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>PIE-01</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>PI-01</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G515" t="n">
+        <v>200</v>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I515" t="n">
+        <v>54.88</v>
+      </c>
+      <c r="J515" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="K515" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="L515" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="M515" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="N515" t="inlineStr">
+        <is>
+          <t>As built INT Ayrton Senna enviado em 20/07/2026: PIE-01 ao PI-02, 3 pontos, 2 trechos em VCA, PVC DN200.</t>
+        </is>
+      </c>
+      <c r="O515" t="n">
+        <v>-23.525061</v>
+      </c>
+      <c r="P515" t="n">
+        <v>-46.3878118</v>
+      </c>
+      <c r="Q515" t="n">
+        <v>-23.5247053</v>
+      </c>
+      <c r="R515" t="n">
+        <v>-46.3881861</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>interl_rua_ayrton_senna</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>AS-002</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>PI-01 - PI-02</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>PI-01</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>PI-02</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="G516" t="n">
+        <v>200</v>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>Vala a Céu Aberto - VCA</t>
+        </is>
+      </c>
+      <c r="I516" t="n">
+        <v>7.17</v>
+      </c>
+      <c r="J516" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="K516" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L516" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="M516" t="inlineStr">
+        <is>
+          <t>concluída</t>
+        </is>
+      </c>
+      <c r="N516" t="inlineStr">
+        <is>
+          <t>As built INT Ayrton Senna enviado em 20/07/2026: PIE-01 ao PI-02, 3 pontos, 2 trechos em VCA, PVC DN200.</t>
+        </is>
+      </c>
+      <c r="O516" t="n">
+        <v>-23.5247053</v>
+      </c>
+      <c r="P516" t="n">
+        <v>-46.3881861</v>
+      </c>
+      <c r="Q516" t="n">
+        <v>-23.5247218</v>
+      </c>
+      <c r="R516" t="n">
+        <v>-46.388254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>